<commit_message>
Daily refresh: price/yield 2026-08-25
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="資料" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="資料" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="說明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'資料'!$A$1:$S$501</definedName>
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.25</v>
+        <v>24.7</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>33.45</v>
+        <v>34.8</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -791,7 +791,7 @@
       <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="n">
-        <v>27.1</v>
+        <v>26.8</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -860,7 +860,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>51.9</v>
+        <v>52.6</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -911,7 +911,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -980,7 +980,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1029,7 +1029,7 @@
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
       <c r="Q8" s="3" t="n">
-        <v>29.3</v>
+        <v>29.05</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1098,7 +1098,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>40.8</v>
+        <v>41.9</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1147,7 +1147,7 @@
       <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
       <c r="Q10" s="3" t="n">
-        <v>88.09999999999999</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="R10" s="3" t="n"/>
       <c r="S10" s="3">
@@ -1194,7 +1194,7 @@
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
       <c r="Q11" s="3" t="n">
-        <v>151.5</v>
+        <v>157</v>
       </c>
       <c r="R11" s="3" t="n"/>
       <c r="S11" s="3">
@@ -1261,7 +1261,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1330,7 +1330,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>207.5</v>
+        <v>180</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1379,7 +1379,7 @@
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>13.2</v>
+        <v>11.85</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1473,7 +1473,7 @@
       <c r="O16" s="3" t="n"/>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.99</v>
+        <v>7.98</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1540,7 +1540,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>83.90000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1609,7 +1609,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>60.5</v>
+        <v>57.1</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>27.1</v>
+        <v>29.45</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1725,7 +1725,7 @@
       <c r="O20" s="3" t="n"/>
       <c r="P20" s="3" t="n"/>
       <c r="Q20" s="3" t="n">
-        <v>31</v>
+        <v>24.3</v>
       </c>
       <c r="R20" s="3" t="n"/>
       <c r="S20" s="3">
@@ -1772,7 +1772,7 @@
       <c r="O21" s="3" t="n"/>
       <c r="P21" s="3" t="n"/>
       <c r="Q21" s="3" t="n">
-        <v>66.7</v>
+        <v>66</v>
       </c>
       <c r="R21" s="3" t="n"/>
       <c r="S21" s="3">
@@ -1819,7 +1819,7 @@
       <c r="O22" s="3" t="n"/>
       <c r="P22" s="3" t="n"/>
       <c r="Q22" s="3" t="n">
-        <v>17.4</v>
+        <v>17.75</v>
       </c>
       <c r="R22" s="3" t="n"/>
       <c r="S22" s="3">
@@ -1886,7 +1886,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>14</v>
+        <v>13.6</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -1955,7 +1955,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2024,7 +2024,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2087,7 +2087,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>198.5</v>
+        <v>199.5</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2223,7 +2223,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2292,7 +2292,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102.5</v>
+        <v>101.5</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2361,7 +2361,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>727</v>
+        <v>712</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2410,7 +2410,7 @@
       <c r="O31" s="3" t="n"/>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.25</v>
+        <v>49.1</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>725</v>
+        <v>680</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2524,7 +2524,7 @@
       <c r="O33" s="3" t="n"/>
       <c r="P33" s="3" t="n"/>
       <c r="Q33" s="3" t="n">
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="R33" s="3" t="n"/>
       <c r="S33" s="3">
@@ -2580,7 +2580,9 @@
       <c r="P34" s="3" t="n">
         <v>31.09</v>
       </c>
-      <c r="Q34" s="3" t="n"/>
+      <c r="Q34" s="3" t="n">
+        <v>1435</v>
+      </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
       </c>
@@ -2648,7 +2650,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>37.3</v>
+        <v>38.1</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2717,7 +2719,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>35.85</v>
+        <v>36.7</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -2786,7 +2788,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.05</v>
+        <v>37.35</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -2835,7 +2837,7 @@
       <c r="O38" s="3" t="n"/>
       <c r="P38" s="3" t="n"/>
       <c r="Q38" s="3" t="n">
-        <v>51.4</v>
+        <v>49.8</v>
       </c>
       <c r="R38" s="3" t="n"/>
       <c r="S38" s="3">
@@ -2902,7 +2904,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>40.1</v>
+        <v>41.4</v>
       </c>
       <c r="R39" s="3" t="n"/>
       <c r="S39" s="3">
@@ -2969,7 +2971,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>39.55</v>
+        <v>39.8</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3038,7 +3040,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>17</v>
+        <v>16.65</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3107,7 +3109,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>70.2</v>
+        <v>71.3</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3156,7 +3158,7 @@
       <c r="O43" s="3" t="n"/>
       <c r="P43" s="3" t="n"/>
       <c r="Q43" s="3" t="n">
-        <v>10.7</v>
+        <v>10.75</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3223,7 +3225,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>46.25</v>
+        <v>46.2</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3272,7 +3274,7 @@
       <c r="O45" s="3" t="n"/>
       <c r="P45" s="3" t="n"/>
       <c r="Q45" s="3" t="n">
-        <v>88.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="R45" s="3" t="n"/>
       <c r="S45" s="3">
@@ -3319,7 +3321,7 @@
       <c r="O46" s="3" t="n"/>
       <c r="P46" s="3" t="n"/>
       <c r="Q46" s="3" t="n">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="R46" s="3" t="n"/>
       <c r="S46" s="3">
@@ -3366,7 +3368,7 @@
       <c r="O47" s="3" t="n"/>
       <c r="P47" s="3" t="n"/>
       <c r="Q47" s="3" t="n">
-        <v>159.5</v>
+        <v>160</v>
       </c>
       <c r="R47" s="3" t="n"/>
       <c r="S47" s="3">
@@ -3433,7 +3435,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>101</v>
+        <v>101.5</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3482,7 +3484,7 @@
       <c r="O49" s="3" t="n"/>
       <c r="P49" s="3" t="n"/>
       <c r="Q49" s="3" t="n">
-        <v>20.55</v>
+        <v>19.2</v>
       </c>
       <c r="R49" s="3" t="n"/>
       <c r="S49" s="3">
@@ -3547,7 +3549,7 @@
       </c>
       <c r="P50" s="3" t="n"/>
       <c r="Q50" s="3" t="n">
-        <v>180.5</v>
+        <v>196</v>
       </c>
       <c r="R50" s="3" t="n"/>
       <c r="S50" s="3">
@@ -3612,7 +3614,7 @@
       </c>
       <c r="P51" s="3" t="n"/>
       <c r="Q51" s="3" t="n">
-        <v>57.9</v>
+        <v>56.9</v>
       </c>
       <c r="R51" s="3" t="n"/>
       <c r="S51" s="3">
@@ -3679,7 +3681,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>37</v>
+        <v>35.7</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -3748,7 +3750,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>107</v>
+        <v>107.5</v>
       </c>
       <c r="R53" s="3" t="n"/>
       <c r="S53" s="3">
@@ -3795,7 +3797,7 @@
       <c r="O54" s="3" t="n"/>
       <c r="P54" s="3" t="n"/>
       <c r="Q54" s="3" t="n">
-        <v>25.7</v>
+        <v>25.75</v>
       </c>
       <c r="R54" s="3" t="n"/>
       <c r="S54" s="3">
@@ -3842,7 +3844,7 @@
       <c r="O55" s="3" t="n"/>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.65</v>
+        <v>13.4</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -3909,7 +3911,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>28.95</v>
+        <v>31</v>
       </c>
       <c r="R56" s="3" t="n"/>
       <c r="S56" s="3">
@@ -3970,7 +3972,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4039,7 +4041,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>80.90000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="R58" s="3" t="n"/>
       <c r="S58" s="3">
@@ -4086,7 +4088,7 @@
       <c r="O59" s="3" t="n"/>
       <c r="P59" s="3" t="n"/>
       <c r="Q59" s="3" t="n">
-        <v>22.95</v>
+        <v>22.8</v>
       </c>
       <c r="R59" s="3" t="n"/>
       <c r="S59" s="3">
@@ -4133,7 +4135,7 @@
       <c r="O60" s="3" t="n"/>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.5</v>
+        <v>17.3</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4180,7 +4182,7 @@
       <c r="O61" s="3" t="n"/>
       <c r="P61" s="3" t="n"/>
       <c r="Q61" s="3" t="n">
-        <v>60.6</v>
+        <v>64.7</v>
       </c>
       <c r="R61" s="3" t="n"/>
       <c r="S61" s="3">
@@ -4294,7 +4296,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>50.5</v>
+        <v>51</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4363,7 +4365,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>349</v>
+        <v>343.5</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4432,7 +4434,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>12500</v>
+        <v>14410</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -4501,7 +4503,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>155</v>
+        <v>150.5</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -4550,7 +4552,7 @@
       <c r="O67" s="3" t="n"/>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="n">
-        <v>33.25</v>
+        <v>33.5</v>
       </c>
       <c r="R67" s="3" t="n"/>
       <c r="S67" s="3">
@@ -4597,7 +4599,7 @@
       <c r="O68" s="3" t="n"/>
       <c r="P68" s="3" t="n"/>
       <c r="Q68" s="3" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R68" s="3" t="n"/>
       <c r="S68" s="3">
@@ -4664,7 +4666,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.4</v>
+        <v>31.45</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -4733,7 +4735,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.65</v>
+        <v>17.45</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -4782,7 +4784,7 @@
       <c r="O71" s="3" t="n"/>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="n">
-        <v>28</v>
+        <v>29.1</v>
       </c>
       <c r="R71" s="3" t="n"/>
       <c r="S71" s="3">
@@ -4829,7 +4831,7 @@
       <c r="O72" s="3" t="n"/>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="n">
-        <v>55.1</v>
+        <v>54.3</v>
       </c>
       <c r="R72" s="3" t="n"/>
       <c r="S72" s="3">
@@ -4896,7 +4898,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>60.9</v>
+        <v>64</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -4955,7 +4957,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5004,7 +5006,7 @@
       <c r="O75" s="3" t="n"/>
       <c r="P75" s="3" t="n"/>
       <c r="Q75" s="3" t="n">
-        <v>15.91</v>
+        <v>19.2</v>
       </c>
       <c r="R75" s="3" t="n"/>
       <c r="S75" s="3">
@@ -5071,7 +5073,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5120,7 +5122,7 @@
       <c r="O77" s="3" t="n"/>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>49.05</v>
+        <v>49</v>
       </c>
       <c r="R77" s="3" t="n"/>
       <c r="S77" s="3">
@@ -5167,7 +5169,7 @@
       <c r="O78" s="3" t="n"/>
       <c r="P78" s="3" t="n"/>
       <c r="Q78" s="3" t="n">
-        <v>226.5</v>
+        <v>226</v>
       </c>
       <c r="R78" s="3" t="n"/>
       <c r="S78" s="3">
@@ -5232,7 +5234,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.5</v>
+        <v>31.45</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -5299,7 +5301,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>267</v>
+        <v>287</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -5368,7 +5370,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>121</v>
+        <v>123.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -5437,7 +5439,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1620</v>
+        <v>1735</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -5486,7 +5488,7 @@
       <c r="O83" s="3" t="n"/>
       <c r="P83" s="3" t="n"/>
       <c r="Q83" s="3" t="n">
-        <v>31.05</v>
+        <v>31.75</v>
       </c>
       <c r="R83" s="3" t="n"/>
       <c r="S83" s="3">
@@ -5553,7 +5555,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>215.5</v>
+        <v>212.5</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -5622,7 +5624,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>158.5</v>
+        <v>155.5</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -5691,7 +5693,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>264.5</v>
+        <v>243.5</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -5760,7 +5762,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>43.2</v>
+        <v>41.6</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -5829,7 +5831,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>622</v>
+        <v>551</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -5925,7 +5927,7 @@
       <c r="O90" s="3" t="n"/>
       <c r="P90" s="3" t="n"/>
       <c r="Q90" s="3" t="n">
-        <v>52.3</v>
+        <v>43.7</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -5994,7 +5996,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2395</v>
+        <v>2375</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6043,7 +6045,7 @@
       <c r="O92" s="3" t="n"/>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>20.2</v>
+        <v>20.35</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6110,7 +6112,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6175,7 +6177,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>38.25</v>
+        <v>38.35</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -6244,7 +6246,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>183.5</v>
+        <v>177</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -6313,7 +6315,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2300</v>
+        <v>2070</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -6382,7 +6384,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>90.90000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -6431,7 +6433,7 @@
       <c r="O98" s="3" t="n"/>
       <c r="P98" s="3" t="n"/>
       <c r="Q98" s="3" t="n">
-        <v>197.5</v>
+        <v>200.5</v>
       </c>
       <c r="R98" s="3" t="n"/>
       <c r="S98" s="3">
@@ -6498,7 +6500,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>29.5</v>
+        <v>28.65</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -6565,7 +6567,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>32.3</v>
+        <v>31.1</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -6634,7 +6636,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>62.5</v>
+        <v>60.5</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -6683,7 +6685,7 @@
       <c r="O102" s="3" t="n"/>
       <c r="P102" s="3" t="n"/>
       <c r="Q102" s="3" t="n">
-        <v>41.7</v>
+        <v>41.65</v>
       </c>
       <c r="R102" s="3" t="n"/>
       <c r="S102" s="3">
@@ -6750,7 +6752,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>69.90000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -6815,7 +6817,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>996</v>
+        <v>923</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -6864,7 +6866,7 @@
       <c r="O105" s="3" t="n"/>
       <c r="P105" s="3" t="n"/>
       <c r="Q105" s="3" t="n">
-        <v>150</v>
+        <v>145.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -6927,7 +6929,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2300</v>
+        <v>2070</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -6976,7 +6978,7 @@
       <c r="O107" s="3" t="n"/>
       <c r="P107" s="3" t="n"/>
       <c r="Q107" s="3" t="n">
-        <v>47.35</v>
+        <v>48.85</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7025,7 +7027,7 @@
       <c r="O108" s="3" t="n"/>
       <c r="P108" s="3" t="n"/>
       <c r="Q108" s="3" t="n">
-        <v>51</v>
+        <v>50.6</v>
       </c>
       <c r="R108" s="3" t="n"/>
       <c r="S108" s="3">
@@ -7080,7 +7082,7 @@
       <c r="O109" s="3" t="n"/>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>51.5</v>
+        <v>42.5</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -7147,7 +7149,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1015</v>
+        <v>948</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -7214,7 +7216,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>26.35</v>
+        <v>27.45</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -7261,7 +7263,7 @@
       <c r="O112" s="3" t="n"/>
       <c r="P112" s="3" t="n"/>
       <c r="Q112" s="3" t="n">
-        <v>68.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R112" s="3" t="n"/>
       <c r="S112" s="3">
@@ -7308,7 +7310,7 @@
       <c r="O113" s="3" t="n"/>
       <c r="P113" s="3" t="n"/>
       <c r="Q113" s="3" t="n">
-        <v>122.5</v>
+        <v>120.5</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -7370,7 +7372,9 @@
       <c r="P114" s="3" t="n">
         <v>12.87</v>
       </c>
-      <c r="Q114" s="3" t="n"/>
+      <c r="Q114" s="3" t="n">
+        <v>341</v>
+      </c>
       <c r="R114" s="3" t="n"/>
       <c r="S114" s="3">
         <f>IF(OR(Q114="",R114="",Q114=0),"",R114/Q114*100)</f>
@@ -7436,7 +7440,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -7503,7 +7507,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>703</v>
+        <v>716</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -7570,7 +7574,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -7639,7 +7643,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>6165</v>
+        <v>5430</v>
       </c>
       <c r="R118" s="3" t="n"/>
       <c r="S118" s="3">
@@ -7700,7 +7704,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>107.5</v>
+        <v>105.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -7749,7 +7753,7 @@
       <c r="O120" s="3" t="n"/>
       <c r="P120" s="3" t="n"/>
       <c r="Q120" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="R120" s="3" t="n"/>
       <c r="S120" s="3">
@@ -7796,7 +7800,7 @@
       <c r="O121" s="3" t="n"/>
       <c r="P121" s="3" t="n"/>
       <c r="Q121" s="3" t="n">
-        <v>41.6</v>
+        <v>44.25</v>
       </c>
       <c r="R121" s="3" t="n"/>
       <c r="S121" s="3">
@@ -7863,7 +7867,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>64.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -7932,7 +7936,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>683</v>
+        <v>658</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -7981,7 +7985,7 @@
       <c r="O124" s="3" t="n"/>
       <c r="P124" s="3" t="n"/>
       <c r="Q124" s="3" t="n">
-        <v>25.5</v>
+        <v>25.2</v>
       </c>
       <c r="R124" s="3" t="n"/>
       <c r="S124" s="3">
@@ -8028,7 +8032,7 @@
       <c r="O125" s="3" t="n"/>
       <c r="P125" s="3" t="n"/>
       <c r="Q125" s="3" t="n">
-        <v>54.8</v>
+        <v>54.4</v>
       </c>
       <c r="R125" s="3" t="n"/>
       <c r="S125" s="3">
@@ -8095,7 +8099,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1125</v>
+        <v>1065</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -8164,7 +8168,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>512</v>
+        <v>501</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -8233,7 +8237,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>25.6</v>
+        <v>25.25</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -8351,7 +8355,7 @@
       <c r="O130" s="3" t="n"/>
       <c r="P130" s="3" t="n"/>
       <c r="Q130" s="3" t="n">
-        <v>125.5</v>
+        <v>143.5</v>
       </c>
       <c r="R130" s="3" t="n"/>
       <c r="S130" s="3">
@@ -8398,7 +8402,7 @@
       <c r="O131" s="3" t="n"/>
       <c r="P131" s="3" t="n"/>
       <c r="Q131" s="3" t="n">
-        <v>82.2</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R131" s="3" t="n"/>
       <c r="S131" s="3">
@@ -8445,7 +8449,7 @@
       <c r="O132" s="3" t="n"/>
       <c r="P132" s="3" t="n"/>
       <c r="Q132" s="3" t="n">
-        <v>276.5</v>
+        <v>250.5</v>
       </c>
       <c r="R132" s="3" t="n"/>
       <c r="S132" s="3">
@@ -8492,7 +8496,7 @@
       <c r="O133" s="3" t="n"/>
       <c r="P133" s="3" t="n"/>
       <c r="Q133" s="3" t="n">
-        <v>82.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="R133" s="3" t="n"/>
       <c r="S133" s="3">
@@ -8539,7 +8543,7 @@
       <c r="O134" s="3" t="n"/>
       <c r="P134" s="3" t="n"/>
       <c r="Q134" s="3" t="n">
-        <v>112.5</v>
+        <v>113.5</v>
       </c>
       <c r="R134" s="3" t="n"/>
       <c r="S134" s="3">
@@ -8606,7 +8610,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -8675,7 +8679,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>284.5</v>
+        <v>316</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -8744,7 +8748,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4210</v>
+        <v>3765</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -8793,7 +8797,7 @@
       <c r="O138" s="3" t="n"/>
       <c r="P138" s="3" t="n"/>
       <c r="Q138" s="3" t="n">
-        <v>364</v>
+        <v>381.5</v>
       </c>
       <c r="R138" s="3" t="n"/>
       <c r="S138" s="3">
@@ -8840,7 +8844,7 @@
       <c r="O139" s="3" t="n"/>
       <c r="P139" s="3" t="n"/>
       <c r="Q139" s="3" t="n">
-        <v>140.5</v>
+        <v>139</v>
       </c>
       <c r="R139" s="3" t="n"/>
       <c r="S139" s="3">
@@ -8889,7 +8893,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>174.5</v>
+        <v>187.5</v>
       </c>
       <c r="R140" s="3" t="n"/>
       <c r="S140" s="3">
@@ -8936,7 +8940,7 @@
       <c r="O141" s="3" t="n"/>
       <c r="P141" s="3" t="n"/>
       <c r="Q141" s="3" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -9003,7 +9007,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -9052,7 +9056,7 @@
       <c r="O143" s="3" t="n"/>
       <c r="P143" s="3" t="n"/>
       <c r="Q143" s="3" t="n">
-        <v>376</v>
+        <v>220</v>
       </c>
       <c r="R143" s="3" t="n"/>
       <c r="S143" s="3">
@@ -9168,7 +9172,7 @@
       <c r="O145" s="3" t="n"/>
       <c r="P145" s="3" t="n"/>
       <c r="Q145" s="3" t="n">
-        <v>121.82</v>
+        <v>115.5</v>
       </c>
       <c r="R145" s="3" t="n"/>
       <c r="S145" s="3">
@@ -9215,7 +9219,7 @@
       <c r="O146" s="3" t="n"/>
       <c r="P146" s="3" t="n"/>
       <c r="Q146" s="3" t="n">
-        <v>225.5</v>
+        <v>120.5</v>
       </c>
       <c r="R146" s="3" t="n"/>
       <c r="S146" s="3">
@@ -9282,7 +9286,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>160</v>
+        <v>160.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -9331,7 +9335,7 @@
       <c r="O148" s="3" t="n"/>
       <c r="P148" s="3" t="n"/>
       <c r="Q148" s="3" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R148" s="3" t="n"/>
       <c r="S148" s="3">
@@ -9378,7 +9382,7 @@
       <c r="O149" s="3" t="n"/>
       <c r="P149" s="3" t="n"/>
       <c r="Q149" s="3" t="n">
-        <v>276.5</v>
+        <v>249</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -9447,7 +9451,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>35.65</v>
+        <v>36.9</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -9516,7 +9520,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>302.5</v>
+        <v>265</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -9565,7 +9569,7 @@
       <c r="O152" s="3" t="n"/>
       <c r="P152" s="3" t="n"/>
       <c r="Q152" s="3" t="n">
-        <v>265</v>
+        <v>174</v>
       </c>
       <c r="R152" s="3" t="n"/>
       <c r="S152" s="3">
@@ -9612,7 +9616,7 @@
       <c r="O153" s="3" t="n"/>
       <c r="P153" s="3" t="n"/>
       <c r="Q153" s="3" t="n">
-        <v>40.95</v>
+        <v>40.5</v>
       </c>
       <c r="R153" s="3" t="n"/>
       <c r="S153" s="3">
@@ -9679,7 +9683,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>23.15</v>
+        <v>23.1</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -9748,7 +9752,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.3</v>
+        <v>31.9</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -9844,7 +9848,7 @@
       <c r="O157" s="3" t="n"/>
       <c r="P157" s="3" t="n"/>
       <c r="Q157" s="3" t="n">
-        <v>36.8</v>
+        <v>36.45</v>
       </c>
       <c r="R157" s="3" t="n"/>
       <c r="S157" s="3">
@@ -9891,7 +9895,7 @@
       <c r="O158" s="3" t="n"/>
       <c r="P158" s="3" t="n"/>
       <c r="Q158" s="3" t="n">
-        <v>19.9</v>
+        <v>19.45</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -9938,7 +9942,7 @@
       <c r="O159" s="3" t="n"/>
       <c r="P159" s="3" t="n"/>
       <c r="Q159" s="3" t="n">
-        <v>91.59999999999999</v>
+        <v>91</v>
       </c>
       <c r="R159" s="3" t="n"/>
       <c r="S159" s="3">
@@ -10005,7 +10009,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>41.3</v>
+        <v>35.05</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -10072,7 +10076,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>45.5</v>
+        <v>46.3</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -10141,7 +10145,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>46.2</v>
+        <v>48.3</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -10190,7 +10194,7 @@
       <c r="O163" s="3" t="n"/>
       <c r="P163" s="3" t="n"/>
       <c r="Q163" s="3" t="n">
-        <v>38.95</v>
+        <v>38.65</v>
       </c>
       <c r="R163" s="3" t="n"/>
       <c r="S163" s="3">
@@ -10284,7 +10288,7 @@
       <c r="O165" s="3" t="n"/>
       <c r="P165" s="3" t="n"/>
       <c r="Q165" s="3" t="n">
-        <v>105.5</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="R165" s="3" t="n"/>
       <c r="S165" s="3">
@@ -10331,7 +10335,7 @@
       <c r="O166" s="3" t="n"/>
       <c r="P166" s="3" t="n"/>
       <c r="Q166" s="3" t="n">
-        <v>169.5</v>
+        <v>168.5</v>
       </c>
       <c r="R166" s="3" t="n"/>
       <c r="S166" s="3">
@@ -10398,7 +10402,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>219</v>
+        <v>250.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -10447,7 +10451,7 @@
       <c r="O168" s="3" t="n"/>
       <c r="P168" s="3" t="n"/>
       <c r="Q168" s="3" t="n">
-        <v>37.8</v>
+        <v>36.6</v>
       </c>
       <c r="R168" s="3" t="n"/>
       <c r="S168" s="3">
@@ -10494,7 +10498,7 @@
       <c r="O169" s="3" t="n"/>
       <c r="P169" s="3" t="n"/>
       <c r="Q169" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="R169" s="3" t="n"/>
       <c r="S169" s="3">
@@ -10541,7 +10545,7 @@
       <c r="O170" s="3" t="n"/>
       <c r="P170" s="3" t="n"/>
       <c r="Q170" s="3" t="n">
-        <v>49.6</v>
+        <v>52.3</v>
       </c>
       <c r="R170" s="3" t="n"/>
       <c r="S170" s="3">
@@ -10608,7 +10612,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>51.6</v>
+        <v>64.5</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -10671,7 +10675,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>19.9</v>
+        <v>20.5</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -10740,7 +10744,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>90.59999999999999</v>
+        <v>124.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -10809,7 +10813,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>39.9</v>
+        <v>42.65</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -10878,7 +10882,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>25.9</v>
+        <v>26.2</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -10927,7 +10931,7 @@
       <c r="O176" s="3" t="n"/>
       <c r="P176" s="3" t="n"/>
       <c r="Q176" s="3" t="n">
-        <v>68.3</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -10994,7 +10998,7 @@
       </c>
       <c r="P177" s="3" t="n"/>
       <c r="Q177" s="3" t="n">
-        <v>76.09999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="R177" s="3" t="n"/>
       <c r="S177" s="3">
@@ -11061,7 +11065,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>200</v>
+        <v>174</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -11128,7 +11132,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.4</v>
+        <v>21.3</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -11195,7 +11199,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>46.5</v>
+        <v>45.8</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -11264,7 +11268,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>183</v>
+        <v>180.5</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -11315,7 +11319,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>237.5</v>
+        <v>235.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -11382,7 +11386,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.35</v>
+        <v>22.8</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -11443,7 +11447,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.65</v>
+        <v>17.3</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -11512,7 +11516,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>214.5</v>
+        <v>223.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -11575,7 +11579,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>59.5</v>
+        <v>59.7</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -11642,7 +11646,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>25.25</v>
+        <v>24.55</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -11711,7 +11715,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>116.5</v>
+        <v>116</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -11780,7 +11784,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>237</v>
+        <v>282</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -11849,7 +11853,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>4610</v>
+        <v>5385</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -11916,7 +11920,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>126</v>
+        <v>126.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -11985,7 +11989,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>82.90000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -12054,7 +12058,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>130</v>
+        <v>129.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -12123,7 +12127,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>98.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -12192,7 +12196,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3235</v>
+        <v>2855</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -12243,7 +12247,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>135.5</v>
+        <v>133</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -12312,7 +12316,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>90.2</v>
+        <v>93.8</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -12381,7 +12385,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -12450,7 +12454,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -12501,7 +12505,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>67.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -12552,7 +12556,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>111</v>
+        <v>113.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -12620,7 +12624,9 @@
       <c r="P202" s="3" t="n">
         <v>22.35</v>
       </c>
-      <c r="Q202" s="3" t="n"/>
+      <c r="Q202" s="3" t="n">
+        <v>281.5</v>
+      </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
       </c>
@@ -12688,7 +12694,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>45.45</v>
+        <v>46.8</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -12757,7 +12763,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>527</v>
+        <v>542</v>
       </c>
       <c r="R204" s="3" t="n"/>
       <c r="S204" s="3">
@@ -12824,7 +12830,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="R205" s="3" t="n"/>
       <c r="S205" s="3">
@@ -12891,7 +12897,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>206</v>
+        <v>200.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -12960,7 +12966,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>1020</v>
+        <v>1075</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -13009,7 +13015,7 @@
       <c r="O208" s="3" t="n"/>
       <c r="P208" s="3" t="n"/>
       <c r="Q208" s="3" t="n">
-        <v>200.26</v>
+        <v>177.5</v>
       </c>
       <c r="R208" s="3" t="n"/>
       <c r="S208" s="3">
@@ -13076,7 +13082,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>488</v>
+        <v>450</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -13214,7 +13220,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>2540</v>
+        <v>2765</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -13263,7 +13269,7 @@
       <c r="O212" s="3" t="n"/>
       <c r="P212" s="3" t="n"/>
       <c r="Q212" s="3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="R212" s="3" t="n"/>
       <c r="S212" s="3">
@@ -13310,7 +13316,7 @@
       <c r="O213" s="3" t="n"/>
       <c r="P213" s="3" t="n"/>
       <c r="Q213" s="3" t="n">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="R213" s="3" t="n"/>
       <c r="S213" s="3">
@@ -13377,7 +13383,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -13446,7 +13452,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2535</v>
+        <v>2335</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -13495,7 +13501,7 @@
       <c r="O216" s="3" t="n"/>
       <c r="P216" s="3" t="n"/>
       <c r="Q216" s="3" t="n">
-        <v>170.5</v>
+        <v>177</v>
       </c>
       <c r="R216" s="3" t="n"/>
       <c r="S216" s="3">
@@ -13542,7 +13548,7 @@
       <c r="O217" s="3" t="n"/>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>65</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -13609,7 +13615,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>702</v>
+        <v>727</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -13678,7 +13684,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>675</v>
+        <v>665</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -13747,7 +13753,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>862</v>
+        <v>794</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -13816,7 +13822,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>391</v>
+        <v>326</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -13885,7 +13891,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>138.5</v>
+        <v>137</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -13934,7 +13940,7 @@
       <c r="O223" s="3" t="n"/>
       <c r="P223" s="3" t="n"/>
       <c r="Q223" s="3" t="n">
-        <v>235</v>
+        <v>193</v>
       </c>
       <c r="R223" s="3" t="n"/>
       <c r="S223" s="3">
@@ -14001,7 +14007,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>193.5</v>
+        <v>175.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -14068,7 +14074,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>136.5</v>
+        <v>166</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -14137,7 +14143,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>402</v>
+        <v>438.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -14206,7 +14212,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>225.5</v>
+        <v>205.5</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -14275,7 +14281,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -14344,7 +14350,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>137</v>
+        <v>133.5</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -14413,7 +14419,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>750</v>
+        <v>721</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -14462,7 +14468,7 @@
       <c r="O231" s="3" t="n"/>
       <c r="P231" s="3" t="n"/>
       <c r="Q231" s="3" t="n">
-        <v>108</v>
+        <v>107.5</v>
       </c>
       <c r="R231" s="3" t="n"/>
       <c r="S231" s="3">
@@ -14529,7 +14535,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -14598,7 +14604,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>228.5</v>
+        <v>210</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -14665,7 +14671,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>172</v>
+        <v>188.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -14732,7 +14738,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>582</v>
+        <v>567</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -14801,7 +14807,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>325</v>
+        <v>302.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -14870,7 +14876,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>183</v>
+        <v>186.5</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -14919,7 +14925,7 @@
       <c r="O238" s="3" t="n"/>
       <c r="P238" s="3" t="n"/>
       <c r="Q238" s="3" t="n">
-        <v>27.55</v>
+        <v>27.15</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -14983,7 +14989,9 @@
         <v>6.15</v>
       </c>
       <c r="P239" s="3" t="n"/>
-      <c r="Q239" s="3" t="n"/>
+      <c r="Q239" s="3" t="n">
+        <v>657</v>
+      </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
       </c>
@@ -15100,7 +15108,7 @@
       <c r="O241" s="3" t="n"/>
       <c r="P241" s="3" t="n"/>
       <c r="Q241" s="3" t="n">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="R241" s="3" t="n"/>
       <c r="S241" s="3">
@@ -15165,7 +15173,7 @@
       </c>
       <c r="P242" s="3" t="n"/>
       <c r="Q242" s="3" t="n">
-        <v>5465</v>
+        <v>5365</v>
       </c>
       <c r="R242" s="3" t="n"/>
       <c r="S242" s="3">
@@ -15232,7 +15240,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>551</v>
+        <v>507</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -15301,7 +15309,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>46</v>
+        <v>45.45</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -15370,7 +15378,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1375</v>
+        <v>1290</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -15419,7 +15427,7 @@
       <c r="O246" s="3" t="n"/>
       <c r="P246" s="3" t="n"/>
       <c r="Q246" s="3" t="n">
-        <v>218.5</v>
+        <v>221</v>
       </c>
       <c r="R246" s="3" t="n"/>
       <c r="S246" s="3">
@@ -15484,7 +15492,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>289.5</v>
+        <v>279</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -15553,7 +15561,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2655</v>
+        <v>2200</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -15620,7 +15628,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>340</v>
+        <v>376.5</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -15687,7 +15695,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1720</v>
+        <v>1610</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -15736,7 +15744,7 @@
       <c r="O251" s="3" t="n"/>
       <c r="P251" s="3" t="n"/>
       <c r="Q251" s="3" t="n">
-        <v>677</v>
+        <v>665</v>
       </c>
       <c r="R251" s="3" t="n"/>
       <c r="S251" s="3">
@@ -15803,7 +15811,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.3</v>
+        <v>17</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -15850,7 +15858,7 @@
       <c r="O253" s="3" t="n"/>
       <c r="P253" s="3" t="n"/>
       <c r="Q253" s="3" t="n">
-        <v>845</v>
+        <v>688</v>
       </c>
       <c r="R253" s="3" t="n"/>
       <c r="S253" s="3">
@@ -15915,7 +15923,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -15984,7 +15992,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>223.5</v>
+        <v>224.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -16053,7 +16061,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -16102,7 +16110,7 @@
       <c r="O257" s="3" t="n"/>
       <c r="P257" s="3" t="n"/>
       <c r="Q257" s="3" t="n">
-        <v>259.5</v>
+        <v>257.5</v>
       </c>
       <c r="R257" s="3" t="n"/>
       <c r="S257" s="3">
@@ -16169,7 +16177,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5600</v>
+        <v>5155</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -16228,7 +16236,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4210</v>
+        <v>3735</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -16287,7 +16295,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2200</v>
+        <v>2050</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -16336,7 +16344,7 @@
       <c r="O261" s="3" t="n"/>
       <c r="P261" s="3" t="n"/>
       <c r="Q261" s="3" t="n">
-        <v>63.3</v>
+        <v>63.1</v>
       </c>
       <c r="R261" s="3" t="n"/>
       <c r="S261" s="3">
@@ -16403,7 +16411,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="R262" s="3" t="n"/>
       <c r="S262" s="3">
@@ -16470,7 +16478,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>463.5</v>
+        <v>464</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -16539,7 +16547,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -16608,7 +16616,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -16677,7 +16685,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.85</v>
+        <v>19.8</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -16726,7 +16734,7 @@
       <c r="O267" s="3" t="n"/>
       <c r="P267" s="3" t="n"/>
       <c r="Q267" s="3" t="n">
-        <v>45.35</v>
+        <v>41.9</v>
       </c>
       <c r="R267" s="3" t="n"/>
       <c r="S267" s="3">
@@ -16773,7 +16781,7 @@
       <c r="O268" s="3" t="n"/>
       <c r="P268" s="3" t="n"/>
       <c r="Q268" s="3" t="n">
-        <v>54.6</v>
+        <v>55.8</v>
       </c>
       <c r="R268" s="3" t="n"/>
       <c r="S268" s="3">
@@ -16840,7 +16848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>92.7</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -16905,7 +16913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>62</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -16972,7 +16980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>621</v>
+        <v>592</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -17021,7 +17029,7 @@
       <c r="O272" s="3" t="n"/>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>49.42</v>
+        <v>57.2</v>
       </c>
       <c r="R272" s="3" t="n"/>
       <c r="S272" s="3">
@@ -17068,7 +17076,7 @@
       <c r="O273" s="3" t="n"/>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>151</v>
+        <v>108</v>
       </c>
       <c r="R273" s="3" t="n"/>
       <c r="S273" s="3">
@@ -17135,7 +17143,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>79</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -17199,7 +17207,9 @@
       <c r="P275" s="3" t="n">
         <v>18.4</v>
       </c>
-      <c r="Q275" s="3" t="n"/>
+      <c r="Q275" s="3" t="n">
+        <v>30.25</v>
+      </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
       </c>
@@ -17264,7 +17274,9 @@
         <v>-13.93</v>
       </c>
       <c r="P276" s="3" t="n"/>
-      <c r="Q276" s="3" t="n"/>
+      <c r="Q276" s="3" t="n">
+        <v>32.35</v>
+      </c>
       <c r="R276" s="3" t="n"/>
       <c r="S276" s="3">
         <f>IF(OR(Q276="",R276="",Q276=0),"",R276/Q276*100)</f>
@@ -17328,7 +17340,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>64.2</v>
+        <v>63.7</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -17395,7 +17407,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -17444,7 +17456,7 @@
       <c r="O279" s="3" t="n"/>
       <c r="P279" s="3" t="n"/>
       <c r="Q279" s="3" t="n">
-        <v>163.5</v>
+        <v>171.5</v>
       </c>
       <c r="R279" s="3" t="n"/>
       <c r="S279" s="3">
@@ -17491,7 +17503,7 @@
       <c r="O280" s="3" t="n"/>
       <c r="P280" s="3" t="n"/>
       <c r="Q280" s="3" t="n">
-        <v>155.5</v>
+        <v>154</v>
       </c>
       <c r="R280" s="3" t="n"/>
       <c r="S280" s="3">
@@ -17538,7 +17550,7 @@
       <c r="O281" s="3" t="n"/>
       <c r="P281" s="3" t="n"/>
       <c r="Q281" s="3" t="n">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="R281" s="3" t="n"/>
       <c r="S281" s="3">
@@ -17593,7 +17605,7 @@
       <c r="O282" s="3" t="n"/>
       <c r="P282" s="3" t="n"/>
       <c r="Q282" s="3" t="n">
-        <v>488</v>
+        <v>471</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -17642,7 +17654,7 @@
       <c r="O283" s="3" t="n"/>
       <c r="P283" s="3" t="n"/>
       <c r="Q283" s="3" t="n">
-        <v>301.5</v>
+        <v>292.5</v>
       </c>
       <c r="R283" s="3" t="n"/>
       <c r="S283" s="3">
@@ -17709,7 +17721,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>32.55</v>
+        <v>35.8</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -17758,7 +17770,7 @@
       <c r="O285" s="3" t="n"/>
       <c r="P285" s="3" t="n"/>
       <c r="Q285" s="3" t="n">
-        <v>299.27</v>
+        <v>202.5</v>
       </c>
       <c r="R285" s="3" t="n"/>
       <c r="S285" s="3">
@@ -17825,7 +17837,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>395.5</v>
+        <v>401</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -17894,7 +17906,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>48.3</v>
+        <v>47.6</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -17961,7 +17973,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>787</v>
+        <v>746</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -18020,7 +18032,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>50.2</v>
+        <v>46.8</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -18067,7 +18079,7 @@
       <c r="O290" s="3" t="n"/>
       <c r="P290" s="3" t="n"/>
       <c r="Q290" s="3" t="n">
-        <v>279.31</v>
+        <v>206.5</v>
       </c>
       <c r="R290" s="3" t="n"/>
       <c r="S290" s="3">
@@ -18134,7 +18146,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>352.5</v>
+        <v>353.5</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -18201,7 +18213,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -18270,7 +18282,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -18339,7 +18351,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>254</v>
+        <v>264.5</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -18408,7 +18420,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>99</v>
+        <v>101.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -18457,7 +18469,7 @@
       <c r="O296" s="3" t="n"/>
       <c r="P296" s="3" t="n"/>
       <c r="Q296" s="3" t="n">
-        <v>44.85</v>
+        <v>34</v>
       </c>
       <c r="R296" s="3" t="n"/>
       <c r="S296" s="3">
@@ -18504,7 +18516,7 @@
       <c r="O297" s="3" t="n"/>
       <c r="P297" s="3" t="n"/>
       <c r="Q297" s="3" t="n">
-        <v>74.3</v>
+        <v>60.5</v>
       </c>
       <c r="R297" s="3" t="n"/>
       <c r="S297" s="3">
@@ -18569,7 +18581,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>118.5</v>
+        <v>116</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -18630,7 +18642,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -18699,7 +18711,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>94.8</v>
+        <v>89.3</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -18768,7 +18780,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>463</v>
+        <v>435.5</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -18837,7 +18849,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -18906,7 +18918,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>570</v>
+        <v>557</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -18955,7 +18967,7 @@
       <c r="O304" s="3" t="n"/>
       <c r="P304" s="3" t="n"/>
       <c r="Q304" s="3" t="n">
-        <v>250.5</v>
+        <v>278</v>
       </c>
       <c r="R304" s="3" t="n"/>
       <c r="S304" s="3">
@@ -19012,7 +19024,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>480</v>
+        <v>530</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -19081,7 +19093,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>522</v>
+        <v>547</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -19140,7 +19152,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>460</v>
+        <v>435</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -19276,7 +19288,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>32.65</v>
+        <v>34.15</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -19345,7 +19357,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>20.95</v>
+        <v>21.65</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -19414,7 +19426,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>302.5</v>
+        <v>300</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -19473,7 +19485,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>97.8</v>
+        <v>89.3</v>
       </c>
       <c r="R312" s="3" t="n"/>
       <c r="S312" s="3">
@@ -19540,7 +19552,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1380</v>
+        <v>1400</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -19609,7 +19621,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>17690</v>
+        <v>15115</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -19658,7 +19670,7 @@
       <c r="O315" s="3" t="n"/>
       <c r="P315" s="3" t="n"/>
       <c r="Q315" s="3" t="n">
-        <v>373.5</v>
+        <v>318.5</v>
       </c>
       <c r="R315" s="3" t="n"/>
       <c r="S315" s="3">
@@ -19725,7 +19737,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1475</v>
+        <v>1570</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -19794,7 +19806,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>16.2</v>
+        <v>28.6</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -19863,7 +19875,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>76.90000000000001</v>
+        <v>76</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -19932,7 +19944,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>160.5</v>
+        <v>151</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -20001,7 +20013,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -20068,7 +20080,7 @@
         <v>337.2</v>
       </c>
       <c r="Q321" s="3" t="n">
-        <v>90.09999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="R321" s="3" t="n">
         <v>0.3</v>
@@ -20203,7 +20215,9 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="P323" s="3" t="n"/>
-      <c r="Q323" s="3" t="n"/>
+      <c r="Q323" s="3" t="n">
+        <v>86.09999999999999</v>
+      </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
       </c>
@@ -20340,7 +20354,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>241</v>
+        <v>239.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -20409,7 +20423,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>106</v>
+        <v>101.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -20466,7 +20480,7 @@
       <c r="O327" s="3" t="n"/>
       <c r="P327" s="3" t="n"/>
       <c r="Q327" s="3" t="n">
-        <v>70.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R327" s="3" t="n"/>
       <c r="S327" s="3">
@@ -20532,7 +20546,9 @@
       <c r="P328" s="3" t="n">
         <v>132.17</v>
       </c>
-      <c r="Q328" s="3" t="n"/>
+      <c r="Q328" s="3" t="n">
+        <v>159.5</v>
+      </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
         <f>IF(OR(Q328="",R328="",Q328=0),"",R328/Q328*100)</f>
@@ -20578,7 +20594,7 @@
       <c r="O329" s="3" t="n"/>
       <c r="P329" s="3" t="n"/>
       <c r="Q329" s="3" t="n">
-        <v>98.5</v>
+        <v>98.7</v>
       </c>
       <c r="R329" s="3" t="n"/>
       <c r="S329" s="3">
@@ -20645,7 +20661,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>188</v>
+        <v>181.5</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -20713,7 +20729,9 @@
       <c r="P331" s="3" t="n">
         <v>6.19</v>
       </c>
-      <c r="Q331" s="3" t="n"/>
+      <c r="Q331" s="3" t="n">
+        <v>63.5</v>
+      </c>
       <c r="R331" s="3" t="n"/>
       <c r="S331" s="3">
         <f>IF(OR(Q331="",R331="",Q331=0),"",R331/Q331*100)</f>
@@ -20779,7 +20797,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>50.8</v>
+        <v>50.4</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -20826,7 +20844,7 @@
       <c r="O333" s="3" t="n"/>
       <c r="P333" s="3" t="n"/>
       <c r="Q333" s="3" t="n">
-        <v>78.8</v>
+        <v>80.2</v>
       </c>
       <c r="R333" s="3" t="n"/>
       <c r="S333" s="3">
@@ -20893,7 +20911,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>878</v>
+        <v>860</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -20942,7 +20960,7 @@
       <c r="O335" s="3" t="n"/>
       <c r="P335" s="3" t="n"/>
       <c r="Q335" s="3" t="n">
-        <v>50.9</v>
+        <v>55.5</v>
       </c>
       <c r="R335" s="3" t="n"/>
       <c r="S335" s="3">
@@ -20997,7 +21015,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>111.5</v>
+        <v>115.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -21066,7 +21084,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>186</v>
+        <v>185.5</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -21135,7 +21153,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>79</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -21184,7 +21202,7 @@
       <c r="O339" s="3" t="n"/>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>15.55</v>
+        <v>14.2</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -21251,7 +21269,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>412</v>
+        <v>391</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -21320,7 +21338,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.6</v>
+        <v>52.4</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -21389,7 +21407,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>290</v>
+        <v>275.5</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -21458,7 +21476,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>798</v>
+        <v>758</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -21596,7 +21614,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>157.5</v>
+        <v>157</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -21645,7 +21663,7 @@
       <c r="O346" s="3" t="n"/>
       <c r="P346" s="3" t="n"/>
       <c r="Q346" s="3" t="n">
-        <v>118.5</v>
+        <v>119</v>
       </c>
       <c r="R346" s="3" t="n"/>
       <c r="S346" s="3">
@@ -21692,7 +21710,7 @@
       <c r="O347" s="3" t="n"/>
       <c r="P347" s="3" t="n"/>
       <c r="Q347" s="3" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="R347" s="3" t="n"/>
       <c r="S347" s="3">
@@ -21759,7 +21777,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>81.3</v>
+        <v>101.5</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -21828,7 +21846,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.5</v>
+        <v>47.2</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -21893,7 +21911,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>111.5</v>
+        <v>110</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -21962,7 +21980,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1275</v>
+        <v>1205</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -22031,7 +22049,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -22080,7 +22098,7 @@
       <c r="O353" s="3" t="n"/>
       <c r="P353" s="3" t="n"/>
       <c r="Q353" s="3" t="n">
-        <v>84.41</v>
+        <v>65</v>
       </c>
       <c r="R353" s="3" t="n"/>
       <c r="S353" s="3">
@@ -22147,7 +22165,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>82</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -22214,7 +22232,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>510</v>
+        <v>493</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -22263,7 +22281,7 @@
       <c r="O356" s="3" t="n"/>
       <c r="P356" s="3" t="n"/>
       <c r="Q356" s="3" t="n">
-        <v>369</v>
+        <v>290</v>
       </c>
       <c r="R356" s="3" t="n"/>
       <c r="S356" s="3">
@@ -22330,7 +22348,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -22379,7 +22397,7 @@
       <c r="O358" s="3" t="n"/>
       <c r="P358" s="3" t="n"/>
       <c r="Q358" s="3" t="n">
-        <v>138.5</v>
+        <v>139</v>
       </c>
       <c r="R358" s="3" t="n"/>
       <c r="S358" s="3">
@@ -22446,7 +22464,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>510</v>
+        <v>482.5</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -22495,7 +22513,7 @@
       <c r="O360" s="3" t="n"/>
       <c r="P360" s="3" t="n"/>
       <c r="Q360" s="3" t="n">
-        <v>137</v>
+        <v>179.5</v>
       </c>
       <c r="R360" s="3" t="n"/>
       <c r="S360" s="3">
@@ -22559,7 +22577,9 @@
         <v>-0.3</v>
       </c>
       <c r="P361" s="3" t="n"/>
-      <c r="Q361" s="3" t="n"/>
+      <c r="Q361" s="3" t="n">
+        <v>148</v>
+      </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
         <f>IF(OR(Q361="",R361="",Q361=0),"",R361/Q361*100)</f>
@@ -22625,7 +22645,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>6495</v>
+        <v>5565</v>
       </c>
       <c r="R362" s="3" t="n"/>
       <c r="S362" s="3">
@@ -22689,7 +22709,9 @@
         <v>2.99</v>
       </c>
       <c r="P363" s="3" t="n"/>
-      <c r="Q363" s="3" t="n"/>
+      <c r="Q363" s="3" t="n">
+        <v>269.5</v>
+      </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
         <f>IF(OR(Q363="",R363="",Q363=0),"",R363/Q363*100)</f>
@@ -22755,7 +22777,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>199.5</v>
+        <v>197.5</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -22804,7 +22826,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>56.2</v>
+        <v>61.9</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -22851,7 +22873,7 @@
       <c r="O366" s="3" t="n"/>
       <c r="P366" s="3" t="n"/>
       <c r="Q366" s="3" t="n">
-        <v>249.5</v>
+        <v>193</v>
       </c>
       <c r="R366" s="3" t="n"/>
       <c r="S366" s="3">
@@ -22914,7 +22936,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1575</v>
+        <v>1455</v>
       </c>
       <c r="R367" s="3" t="n"/>
       <c r="S367" s="3">
@@ -22961,7 +22983,7 @@
       <c r="O368" s="3" t="n"/>
       <c r="P368" s="3" t="n"/>
       <c r="Q368" s="3" t="n">
-        <v>201.5</v>
+        <v>179</v>
       </c>
       <c r="R368" s="3" t="n"/>
       <c r="S368" s="3">
@@ -23008,7 +23030,7 @@
       <c r="O369" s="3" t="n"/>
       <c r="P369" s="3" t="n"/>
       <c r="Q369" s="3" t="n">
-        <v>58.3</v>
+        <v>44.35</v>
       </c>
       <c r="R369" s="3" t="n"/>
       <c r="S369" s="3">
@@ -23074,7 +23096,9 @@
       <c r="P370" s="3" t="n">
         <v>20.21</v>
       </c>
-      <c r="Q370" s="3" t="n"/>
+      <c r="Q370" s="3" t="n">
+        <v>74.8</v>
+      </c>
       <c r="R370" s="3" t="n"/>
       <c r="S370" s="3">
         <f>IF(OR(Q370="",R370="",Q370=0),"",R370/Q370*100)</f>
@@ -23140,7 +23164,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>245</v>
+        <v>230.5</v>
       </c>
       <c r="R371" s="3" t="n"/>
       <c r="S371" s="3">
@@ -23207,7 +23231,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>214.5</v>
+        <v>229</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -23275,7 +23299,9 @@
       <c r="P373" s="3" t="n">
         <v>33.25</v>
       </c>
-      <c r="Q373" s="3" t="n"/>
+      <c r="Q373" s="3" t="n">
+        <v>366</v>
+      </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
       </c>
@@ -23343,7 +23369,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1040</v>
+        <v>1010</v>
       </c>
       <c r="R374" s="3" t="n"/>
       <c r="S374" s="3">
@@ -23410,7 +23436,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>78</v>
+        <v>77.7</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -23479,7 +23505,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>395</v>
+        <v>395.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -23538,7 +23564,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -23606,7 +23632,9 @@
       <c r="P378" s="3" t="n">
         <v>46.15</v>
       </c>
-      <c r="Q378" s="3" t="n"/>
+      <c r="Q378" s="3" t="n">
+        <v>1460</v>
+      </c>
       <c r="R378" s="3" t="n"/>
       <c r="S378" s="3">
         <f>IF(OR(Q378="",R378="",Q378=0),"",R378/Q378*100)</f>
@@ -23652,7 +23680,7 @@
       <c r="O379" s="3" t="n"/>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>36.4</v>
+        <v>25.85</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -23719,7 +23747,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1500</v>
+        <v>1475</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -23788,7 +23816,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>214</v>
+        <v>210.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -23837,7 +23865,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>400.1</v>
+        <v>400</v>
       </c>
       <c r="R382" s="3" t="n"/>
       <c r="S382" s="3">
@@ -23902,7 +23930,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>68</v>
+        <v>65.5</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -23949,7 +23977,7 @@
       <c r="O384" s="3" t="n"/>
       <c r="P384" s="3" t="n"/>
       <c r="Q384" s="3" t="n">
-        <v>431</v>
+        <v>453</v>
       </c>
       <c r="R384" s="3" t="n"/>
       <c r="S384" s="3">
@@ -24016,7 +24044,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>854</v>
+        <v>1010</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -24065,7 +24093,7 @@
       <c r="O386" s="3" t="n"/>
       <c r="P386" s="3" t="n"/>
       <c r="Q386" s="3" t="n">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -24134,7 +24162,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -24203,7 +24231,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>2990</v>
+        <v>2650</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -24272,7 +24300,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6750</v>
+        <v>6145</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -24321,7 +24349,7 @@
       <c r="O390" s="3" t="n"/>
       <c r="P390" s="3" t="n"/>
       <c r="Q390" s="3" t="n">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="R390" s="3" t="n"/>
       <c r="S390" s="3">
@@ -24388,7 +24416,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>610</v>
+        <v>578</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -24457,7 +24485,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>932</v>
+        <v>845</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -24524,7 +24552,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>86.09999999999999</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -24589,7 +24617,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>51.5</v>
+        <v>55.5</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -24655,7 +24683,9 @@
       <c r="P395" s="3" t="n">
         <v>32.7</v>
       </c>
-      <c r="Q395" s="3" t="n"/>
+      <c r="Q395" s="3" t="n">
+        <v>70.8</v>
+      </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
       </c>
@@ -24719,7 +24749,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="R396" s="3" t="n"/>
       <c r="S396" s="3">
@@ -24766,7 +24796,7 @@
       <c r="O397" s="3" t="n"/>
       <c r="P397" s="3" t="n"/>
       <c r="Q397" s="3" t="n">
-        <v>180.5</v>
+        <v>147</v>
       </c>
       <c r="R397" s="3" t="n"/>
       <c r="S397" s="3">
@@ -24830,7 +24860,9 @@
         <v>3.14</v>
       </c>
       <c r="P398" s="3" t="n"/>
-      <c r="Q398" s="3" t="n"/>
+      <c r="Q398" s="3" t="n">
+        <v>586</v>
+      </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
         <f>IF(OR(Q398="",R398="",Q398=0),"",R398/Q398*100)</f>
@@ -24896,7 +24928,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.3</v>
+        <v>61.2</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -24945,7 +24977,7 @@
       <c r="O400" s="3" t="n"/>
       <c r="P400" s="3" t="n"/>
       <c r="Q400" s="3" t="n">
-        <v>126</v>
+        <v>139.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -25011,7 +25043,9 @@
       <c r="P401" s="3" t="n">
         <v>16.06</v>
       </c>
-      <c r="Q401" s="3" t="n"/>
+      <c r="Q401" s="3" t="n">
+        <v>251</v>
+      </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
       </c>
@@ -25079,7 +25113,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1085</v>
+        <v>968</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -25148,7 +25182,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -25216,7 +25250,9 @@
       <c r="P404" s="3" t="n">
         <v>20.96</v>
       </c>
-      <c r="Q404" s="3" t="n"/>
+      <c r="Q404" s="3" t="n">
+        <v>353</v>
+      </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
       </c>
@@ -25278,7 +25314,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>6325</v>
+        <v>6300</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -25327,7 +25363,7 @@
       <c r="O406" s="3" t="n"/>
       <c r="P406" s="3" t="n"/>
       <c r="Q406" s="3" t="n">
-        <v>263.5</v>
+        <v>265.5</v>
       </c>
       <c r="R406" s="3" t="n"/>
       <c r="S406" s="3">
@@ -25374,7 +25410,7 @@
       <c r="O407" s="3" t="n"/>
       <c r="P407" s="3" t="n"/>
       <c r="Q407" s="3" t="n">
-        <v>260.81</v>
+        <v>259</v>
       </c>
       <c r="R407" s="3" t="n"/>
       <c r="S407" s="3">
@@ -25441,7 +25477,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1370</v>
+        <v>1090</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -25509,7 +25545,9 @@
       <c r="P409" s="3" t="n">
         <v>21.78</v>
       </c>
-      <c r="Q409" s="3" t="n"/>
+      <c r="Q409" s="3" t="n">
+        <v>611</v>
+      </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
       </c>
@@ -25577,7 +25615,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="R410" s="3" t="n"/>
       <c r="S410" s="3">
@@ -25624,7 +25662,7 @@
       <c r="O411" s="3" t="n"/>
       <c r="P411" s="3" t="n"/>
       <c r="Q411" s="3" t="n">
-        <v>386.99</v>
+        <v>403.5</v>
       </c>
       <c r="R411" s="3" t="n"/>
       <c r="S411" s="3">
@@ -25691,7 +25729,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>193.5</v>
+        <v>191.5</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -25760,7 +25798,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>978</v>
+        <v>972</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -25829,10 +25867,10 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>141.5</v>
+        <v>141</v>
       </c>
       <c r="R414" s="3" t="n">
-        <v>1.24935115</v>
+        <v>1.25</v>
       </c>
       <c r="S414" s="3">
         <f>IF(OR(Q414="",R414="",Q414=0),"",R414/Q414*100)</f>
@@ -25878,7 +25916,7 @@
       <c r="O415" s="3" t="n"/>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>56.2</v>
+        <v>56</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -25945,10 +25983,10 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>65.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="R416" s="3" t="n">
-        <v>5.15512584</v>
+        <v>5.16</v>
       </c>
       <c r="S416" s="3">
         <f>IF(OR(Q416="",R416="",Q416=0),"",R416/Q416*100)</f>
@@ -26014,7 +26052,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>78.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -26073,7 +26111,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1120</v>
+        <v>1045</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -26142,7 +26180,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>442.5</v>
+        <v>415</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -26211,7 +26249,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>269.5</v>
+        <v>270</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -26280,7 +26318,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>1805</v>
+        <v>1710</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -26329,7 +26367,7 @@
       <c r="O422" s="3" t="n"/>
       <c r="P422" s="3" t="n"/>
       <c r="Q422" s="3" t="n">
-        <v>498.95</v>
+        <v>446.5</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -26378,7 +26416,7 @@
       <c r="O423" s="3" t="n"/>
       <c r="P423" s="3" t="n"/>
       <c r="Q423" s="3" t="n">
-        <v>782</v>
+        <v>549</v>
       </c>
       <c r="R423" s="3" t="n"/>
       <c r="S423" s="3">
@@ -26435,7 +26473,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>168.5</v>
+        <v>163.5</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -26484,7 +26522,7 @@
       <c r="O425" s="3" t="n"/>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>16.95</v>
+        <v>16.6</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -26551,7 +26589,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>313.5</v>
+        <v>304.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -26618,7 +26656,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>104</v>
+        <v>110.5</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -26665,7 +26703,7 @@
       <c r="O428" s="3" t="n"/>
       <c r="P428" s="3" t="n"/>
       <c r="Q428" s="3" t="n">
-        <v>273.5</v>
+        <v>260.5</v>
       </c>
       <c r="R428" s="3" t="n"/>
       <c r="S428" s="3">
@@ -26732,7 +26770,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -26781,7 +26819,7 @@
       <c r="O430" s="3" t="n"/>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>46.75</v>
+        <v>1235</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -26828,7 +26866,7 @@
       <c r="O431" s="3" t="n"/>
       <c r="P431" s="3" t="n"/>
       <c r="Q431" s="3" t="n">
-        <v>31.2</v>
+        <v>31.35</v>
       </c>
       <c r="R431" s="3" t="n"/>
       <c r="S431" s="3">
@@ -26895,7 +26933,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1685</v>
+        <v>1710</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -26944,7 +26982,7 @@
       <c r="O433" s="3" t="n"/>
       <c r="P433" s="3" t="n"/>
       <c r="Q433" s="3" t="n">
-        <v>461.5</v>
+        <v>497.5</v>
       </c>
       <c r="R433" s="3" t="n"/>
       <c r="S433" s="3">
@@ -26991,7 +27029,7 @@
       <c r="O434" s="3" t="n"/>
       <c r="P434" s="3" t="n"/>
       <c r="Q434" s="3" t="n">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="R434" s="3" t="n"/>
       <c r="S434" s="3">
@@ -27058,7 +27096,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2815</v>
+        <v>2780</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -27127,7 +27165,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>500</v>
+        <v>487</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -27176,7 +27214,7 @@
       <c r="O437" s="3" t="n"/>
       <c r="P437" s="3" t="n"/>
       <c r="Q437" s="3" t="n">
-        <v>347.49</v>
+        <v>382</v>
       </c>
       <c r="R437" s="3" t="n"/>
       <c r="S437" s="3">
@@ -27242,7 +27280,9 @@
       <c r="P438" s="3" t="n">
         <v>40.48</v>
       </c>
-      <c r="Q438" s="3" t="n"/>
+      <c r="Q438" s="3" t="n">
+        <v>2140</v>
+      </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
       </c>
@@ -27310,7 +27350,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1575</v>
+        <v>1665</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -27379,7 +27419,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -27447,7 +27487,9 @@
       <c r="P441" s="3" t="n">
         <v>68.04000000000001</v>
       </c>
-      <c r="Q441" s="3" t="n"/>
+      <c r="Q441" s="3" t="n">
+        <v>6255</v>
+      </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
       </c>
@@ -27495,7 +27537,7 @@
       <c r="O442" s="3" t="n"/>
       <c r="P442" s="3" t="n"/>
       <c r="Q442" s="3" t="n">
-        <v>17.9</v>
+        <v>16.9</v>
       </c>
       <c r="R442" s="3" t="n"/>
       <c r="S442" s="3">
@@ -27562,7 +27604,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>122</v>
+        <v>121.5</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -27611,7 +27653,7 @@
       <c r="O444" s="3" t="n"/>
       <c r="P444" s="3" t="n"/>
       <c r="Q444" s="3" t="n">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="R444" s="3" t="n"/>
       <c r="S444" s="3">
@@ -27658,7 +27700,7 @@
       <c r="O445" s="3" t="n"/>
       <c r="P445" s="3" t="n"/>
       <c r="Q445" s="3" t="n">
-        <v>410</v>
+        <v>568</v>
       </c>
       <c r="R445" s="3" t="n"/>
       <c r="S445" s="3">
@@ -27705,7 +27747,7 @@
       <c r="O446" s="3" t="n"/>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>344.45</v>
+        <v>355</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -27772,7 +27814,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>690</v>
+        <v>514</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -27821,7 +27863,7 @@
       <c r="O448" s="3" t="n"/>
       <c r="P448" s="3" t="n"/>
       <c r="Q448" s="3" t="n">
-        <v>997.98</v>
+        <v>915</v>
       </c>
       <c r="R448" s="3" t="n"/>
       <c r="S448" s="3">
@@ -27868,7 +27910,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>164.07</v>
+        <v>159</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -27935,7 +27977,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1650</v>
+        <v>1550</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -27984,7 +28026,7 @@
       <c r="O451" s="3" t="n"/>
       <c r="P451" s="3" t="n"/>
       <c r="Q451" s="3" t="n">
-        <v>264.5</v>
+        <v>295.5</v>
       </c>
       <c r="R451" s="3" t="n"/>
       <c r="S451" s="3">
@@ -28031,7 +28073,7 @@
       <c r="O452" s="3" t="n"/>
       <c r="P452" s="3" t="n"/>
       <c r="Q452" s="3" t="n">
-        <v>397</v>
+        <v>388.5</v>
       </c>
       <c r="R452" s="3" t="n"/>
       <c r="S452" s="3">
@@ -28095,7 +28137,9 @@
         <v>-0.24</v>
       </c>
       <c r="P453" s="3" t="n"/>
-      <c r="Q453" s="3" t="n"/>
+      <c r="Q453" s="3" t="n">
+        <v>167.5</v>
+      </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
         <f>IF(OR(Q453="",R453="",Q453=0),"",R453/Q453*100)</f>
@@ -28188,7 +28232,7 @@
       <c r="O455" s="3" t="n"/>
       <c r="P455" s="3" t="n"/>
       <c r="Q455" s="3" t="n">
-        <v>183.5</v>
+        <v>185</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -28255,7 +28299,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>282</v>
+        <v>265</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -28324,7 +28368,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1195</v>
+        <v>1135</v>
       </c>
       <c r="R457" s="3" t="n"/>
       <c r="S457" s="3">
@@ -28391,7 +28435,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>98.7</v>
+        <v>97</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -28459,7 +28503,9 @@
       <c r="P459" s="3" t="n">
         <v>16.1</v>
       </c>
-      <c r="Q459" s="3" t="n"/>
+      <c r="Q459" s="3" t="n">
+        <v>158.5</v>
+      </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
       </c>
@@ -28507,7 +28553,7 @@
       <c r="O460" s="3" t="n"/>
       <c r="P460" s="3" t="n"/>
       <c r="Q460" s="3" t="n">
-        <v>52.7</v>
+        <v>49</v>
       </c>
       <c r="R460" s="3" t="n"/>
       <c r="S460" s="3">
@@ -28574,7 +28620,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -28643,7 +28689,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>114.5</v>
+        <v>112</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -28712,7 +28758,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -28781,7 +28827,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>116.5</v>
+        <v>106</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -28848,7 +28894,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>45.2</v>
+        <v>45.55</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -28897,7 +28943,7 @@
       <c r="O466" s="3" t="n"/>
       <c r="P466" s="3" t="n"/>
       <c r="Q466" s="3" t="n">
-        <v>88.14</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="R466" s="3" t="n"/>
       <c r="S466" s="3">
@@ -28944,7 +28990,7 @@
       <c r="O467" s="3" t="n"/>
       <c r="P467" s="3" t="n"/>
       <c r="Q467" s="3" t="n">
-        <v>198.5</v>
+        <v>195.5</v>
       </c>
       <c r="R467" s="3" t="n"/>
       <c r="S467" s="3">
@@ -29080,7 +29126,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>86.7</v>
+        <v>87.7</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -29149,7 +29195,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>320.5</v>
+        <v>318</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -29218,7 +29264,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>1000</v>
+        <v>967</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -29277,7 +29323,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -29326,7 +29372,7 @@
       <c r="O473" s="3" t="n"/>
       <c r="P473" s="3" t="n"/>
       <c r="Q473" s="3" t="n">
-        <v>215</v>
+        <v>177.5</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -29373,7 +29419,7 @@
       <c r="O474" s="3" t="n"/>
       <c r="P474" s="3" t="n"/>
       <c r="Q474" s="3" t="n">
-        <v>171.61</v>
+        <v>235.5</v>
       </c>
       <c r="R474" s="3" t="n"/>
       <c r="S474" s="3">
@@ -29438,7 +29484,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2080</v>
+        <v>2135</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -29507,7 +29553,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>428.5</v>
+        <v>417</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -29576,7 +29622,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.5</v>
+        <v>38.45</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -29643,7 +29689,7 @@
       </c>
       <c r="P478" s="3" t="n"/>
       <c r="Q478" s="3" t="n">
-        <v>28.25</v>
+        <v>27.2</v>
       </c>
       <c r="R478" s="3" t="n"/>
       <c r="S478" s="3">
@@ -29710,7 +29756,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>262.5</v>
+        <v>251</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -29779,7 +29825,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>374.5</v>
+        <v>360.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -29828,7 +29874,7 @@
       <c r="O481" s="3" t="n"/>
       <c r="P481" s="3" t="n"/>
       <c r="Q481" s="3" t="n">
-        <v>154</v>
+        <v>141.5</v>
       </c>
       <c r="R481" s="3" t="n"/>
       <c r="S481" s="3">
@@ -29875,7 +29921,7 @@
       <c r="O482" s="3" t="n"/>
       <c r="P482" s="3" t="n"/>
       <c r="Q482" s="3" t="n">
-        <v>56.6</v>
+        <v>56.5</v>
       </c>
       <c r="R482" s="3" t="n"/>
       <c r="S482" s="3">
@@ -29942,7 +29988,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>112</v>
+        <v>105.5</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -30011,7 +30057,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1135</v>
+        <v>1145</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -30060,7 +30106,7 @@
       <c r="O485" s="3" t="n"/>
       <c r="P485" s="3" t="n"/>
       <c r="Q485" s="3" t="n">
-        <v>74.5</v>
+        <v>72.2</v>
       </c>
       <c r="R485" s="3" t="n"/>
       <c r="S485" s="3">
@@ -30176,7 +30222,7 @@
       <c r="O487" s="3" t="n"/>
       <c r="P487" s="3" t="n"/>
       <c r="Q487" s="3" t="n">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="R487" s="3" t="n"/>
       <c r="S487" s="3">
@@ -30223,7 +30269,7 @@
       <c r="O488" s="3" t="n"/>
       <c r="P488" s="3" t="n"/>
       <c r="Q488" s="3" t="n">
-        <v>29.1</v>
+        <v>29.15</v>
       </c>
       <c r="R488" s="3" t="n"/>
       <c r="S488" s="3">
@@ -30289,7 +30335,9 @@
       <c r="P489" s="3" t="n">
         <v>14.11</v>
       </c>
-      <c r="Q489" s="3" t="n"/>
+      <c r="Q489" s="3" t="n">
+        <v>71</v>
+      </c>
       <c r="R489" s="3" t="n"/>
       <c r="S489" s="3">
         <f>IF(OR(Q489="",R489="",Q489=0),"",R489/Q489*100)</f>
@@ -30335,7 +30383,7 @@
       <c r="O490" s="3" t="n"/>
       <c r="P490" s="3" t="n"/>
       <c r="Q490" s="3" t="n">
-        <v>83.3</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R490" s="3" t="n"/>
       <c r="S490" s="3">
@@ -30382,7 +30430,7 @@
       <c r="O491" s="3" t="n"/>
       <c r="P491" s="3" t="n"/>
       <c r="Q491" s="3" t="n">
-        <v>68.90000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="R491" s="3" t="n"/>
       <c r="S491" s="3">
@@ -30517,7 +30565,9 @@
       <c r="P493" s="3" t="n">
         <v>68.39</v>
       </c>
-      <c r="Q493" s="3" t="n"/>
+      <c r="Q493" s="3" t="n">
+        <v>104</v>
+      </c>
       <c r="R493" s="3" t="n"/>
       <c r="S493" s="3">
         <f>IF(OR(Q493="",R493="",Q493=0),"",R493/Q493*100)</f>
@@ -30581,7 +30631,7 @@
       </c>
       <c r="P494" s="3" t="n"/>
       <c r="Q494" s="3" t="n">
-        <v>41.25</v>
+        <v>40.15</v>
       </c>
       <c r="R494" s="3" t="n"/>
       <c r="S494" s="3">
@@ -30648,7 +30698,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>64</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -30717,7 +30767,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>42.15</v>
+        <v>41.55</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -30784,7 +30834,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.1</v>
+        <v>55</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -30833,7 +30883,7 @@
       <c r="O498" s="3" t="n"/>
       <c r="P498" s="3" t="n"/>
       <c r="Q498" s="3" t="n">
-        <v>124</v>
+        <v>134.5</v>
       </c>
       <c r="R498" s="3" t="n"/>
       <c r="S498" s="3">
@@ -30900,7 +30950,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>85.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -30968,7 +31018,9 @@
       <c r="P500" s="3" t="n">
         <v>5.21</v>
       </c>
-      <c r="Q500" s="3" t="n"/>
+      <c r="Q500" s="3" t="n">
+        <v>29</v>
+      </c>
       <c r="R500" s="3" t="n"/>
       <c r="S500" s="3">
         <f>IF(OR(Q500="",R500="",Q500=0),"",R500/Q500*100)</f>
@@ -31034,7 +31086,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>102</v>
+        <v>97.3</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-08-26
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.6</v>
+        <v>24.3</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>34.9</v>
+        <v>35.2</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>26.65</v>
+        <v>26.8</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.6</v>
+        <v>52.7</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.85</v>
+        <v>28.95</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.7</v>
+        <v>41.95</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.8</v>
+        <v>81.2</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>156.5</v>
+        <v>157.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>57.8</v>
+        <v>60.1</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>188.5</v>
+        <v>207</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>11.85</v>
+        <v>12.3</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.65</v>
+        <v>11.9</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>7.9</v>
+        <v>7.99</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>58</v>
+        <v>60.3</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>29</v>
+        <v>28.55</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.45</v>
+        <v>24.85</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>65.3</v>
+        <v>66.7</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.5</v>
+        <v>13.75</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>199.5</v>
+        <v>202</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>70.8</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>165.5</v>
+        <v>166</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>100.5</v>
+        <v>102</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.6</v>
+        <v>50.1</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2790,7 +2790,7 @@
         <v>59.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>2</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1460</v>
+        <v>1470</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.45</v>
+        <v>39.4</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.6</v>
+        <v>37.6</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.35</v>
+        <v>38</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50.6</v>
+        <v>50.1</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>41.25</v>
+        <v>44.2</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40</v>
+        <v>39.9</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.5</v>
+        <v>16.55</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>71.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.65</v>
+        <v>10.7</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>87.40000000000001</v>
+        <v>88</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>126.5</v>
+        <v>128.5</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>158</v>
+        <v>160.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>102.5</v>
+        <v>103</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>18.95</v>
+        <v>19.05</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>194</v>
+        <v>195.5</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>58</v>
+        <v>59.7</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>36.35</v>
+        <v>35.6</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>30.45</v>
+        <v>30.4</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.05</v>
+        <v>19.35</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>82</v>
+        <v>82.2</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.65</v>
+        <v>22.8</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.2</v>
+        <v>17.25</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>50.6</v>
+        <v>50</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>345.5</v>
+        <v>353</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>14285</v>
+        <v>14510</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>33.15</v>
+        <v>33</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>31.35</v>
+        <v>31.4</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54</v>
+        <v>54.2</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.9</v>
+        <v>63.6</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.1</v>
+        <v>19.2</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48</v>
+        <v>48.35</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31</v>
+        <v>31.55</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>125</v>
+        <v>123.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1710</v>
+        <v>1750</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.4</v>
+        <v>31.9</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>217.5</v>
+        <v>222</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>243</v>
+        <v>246.5</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>40.8</v>
+        <v>40.95</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>544</v>
+        <v>537</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>44.7</v>
+        <v>45.35</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>43.35</v>
+        <v>44.15</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2400</v>
+        <v>2415</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>122</v>
+        <v>125.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>38.55</v>
+        <v>39.65</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>179</v>
+        <v>181.5</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2030</v>
+        <v>2055</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>86.7</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>199.5</v>
+        <v>219</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.15</v>
+        <v>28.1</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.05</v>
+        <v>31.4</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>60.5</v>
+        <v>61.5</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>41.65</v>
+        <v>42.65</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>65.40000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>925</v>
+        <v>971</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>145</v>
+        <v>146.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>1965</v>
+        <v>1980</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>48.55</v>
+        <v>49.2</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>50.4</v>
+        <v>51.3</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>43.05</v>
+        <v>44.8</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>971</v>
+        <v>1040</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>27.7</v>
+        <v>27.65</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>122.5</v>
+        <v>124</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>347.5</v>
+        <v>351.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>328.5</v>
+        <v>332.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5595</v>
+        <v>5895</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>74</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.1</v>
+        <v>45.15</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>65.2</v>
+        <v>66.8</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>670</v>
+        <v>688</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.15</v>
+        <v>25.65</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>55.8</v>
+        <v>56.1</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1070</v>
+        <v>1080</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>25.65</v>
+        <v>25.5</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>136.5</v>
+        <v>136</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>144</v>
+        <v>151.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>90.8</v>
+        <v>99.8</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>249.5</v>
+        <v>252</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>82.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>239.5</v>
+        <v>244</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>3735</v>
+        <v>3945</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>419.5</v>
+        <v>428</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>137.5</v>
+        <v>139.5</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>535</v>
+        <v>570</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>218</v>
+        <v>218.5</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>204.5</v>
+        <v>206.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>120.5</v>
+        <v>125.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>120.5</v>
+        <v>122</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>137</v>
+        <v>150.5</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>258</v>
+        <v>262.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>40.55</v>
+        <v>41.5</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>268</v>
+        <v>269.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>171</v>
+        <v>181.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.5</v>
+        <v>40.7</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.85</v>
+        <v>32.1</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>35.4</v>
+        <v>35.8</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.35</v>
+        <v>19.6</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>90.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>46.6</v>
+        <v>47.2</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47.5</v>
+        <v>48</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.6</v>
+        <v>34.9</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>96.40000000000001</v>
+        <v>96</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>168</v>
+        <v>171.5</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>36.7</v>
+        <v>34.85</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>52.1</v>
+        <v>52.4</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>63.6</v>
+        <v>57.6</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>126.5</v>
+        <v>115</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.2</v>
+        <v>43</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.3</v>
+        <v>26.35</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>66.7</v>
+        <v>69</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>95.5</v>
+        <v>91.2</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>170.5</v>
+        <v>179</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.55</v>
+        <v>46.35</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>180.5</v>
+        <v>181</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.65</v>
+        <v>22.6</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.45</v>
+        <v>17.55</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>59</v>
+        <v>59.3</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>24.65</v>
+        <v>27.1</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>270</v>
+        <v>273.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>5720</v>
+        <v>6290</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>130</v>
+        <v>129.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>85.09999999999999</v>
+        <v>87.2</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>130.5</v>
+        <v>132.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>96.8</v>
+        <v>102</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>2950</v>
+        <v>3155</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>93</v>
+        <v>92.5</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>320.5</v>
+        <v>314.5</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>628</v>
+        <v>614</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>66</v>
+        <v>66.3</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>110.5</v>
+        <v>110</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>282.5</v>
+        <v>288.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>45.95</v>
+        <v>45.4</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>172</v>
+        <v>180.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>198.5</v>
+        <v>196.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>1095</v>
+        <v>1160</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>185</v>
+        <v>185.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>463</v>
+        <v>481</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>2960</v>
+        <v>3255</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>166</v>
+        <v>165.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>379</v>
+        <v>405</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2260</v>
+        <v>2485</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>180</v>
+        <v>185.5</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>674</v>
+        <v>716</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>835</v>
+        <v>881</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>331</v>
+        <v>364</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>135.5</v>
+        <v>136.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>194</v>
+        <v>197.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>178.5</v>
+        <v>182</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>182.5</v>
+        <v>180.5</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>418.5</v>
+        <v>416</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>213</v>
+        <v>217.5</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>168</v>
+        <v>173.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>135</v>
+        <v>140.5</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>711</v>
+        <v>702</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1065</v>
+        <v>1075</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>623</v>
+        <v>650</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>311</v>
+        <v>333.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>27.25</v>
+        <v>27.75</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>690</v>
+        <v>759</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>285.5</v>
+        <v>287.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>175</v>
+        <v>180.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5570</v>
+        <v>6125</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>533</v>
+        <v>574</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>46.8</v>
+        <v>46.4</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1270</v>
+        <v>1345</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2195</v>
+        <v>2410</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1605</v>
+        <v>1625</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>656</v>
+        <v>685</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.1</v>
+        <v>17.05</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>693</v>
+        <v>741</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>251.5</v>
+        <v>255.5</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>225.5</v>
+        <v>227</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>247.5</v>
+        <v>251.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5205</v>
+        <v>5725</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>3865</v>
+        <v>3960</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2075</v>
+        <v>2005</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>66</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>461.5</v>
+        <v>488</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>41.4</v>
+        <v>42</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>55.6</v>
+        <v>55.8</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>62</v>
+        <v>63.6</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>59.6</v>
+        <v>62.7</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>109.5</v>
+        <v>114</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.8</v>
+        <v>78.2</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>32.45</v>
+        <v>32.1</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>63.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>123.5</v>
+        <v>123</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>35.15</v>
+        <v>34.65</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>46.95</v>
+        <v>47.8</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>44.95</v>
+        <v>46.6</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>343.5</v>
+        <v>344.5</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>307</v>
+        <v>324.5</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>206.5</v>
+        <v>209</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>260.5</v>
+        <v>261</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>102.5</v>
+        <v>101</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>34.55</v>
+        <v>37.3</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>59.8</v>
+        <v>60.2</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>245</v>
+        <v>255.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>88.8</v>
+        <v>89.3</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>164.5</v>
+        <v>165.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>556</v>
+        <v>576</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>445</v>
+        <v>489.5</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56</v>
+        <v>56.5</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.75</v>
+        <v>33.55</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.4</v>
+        <v>21.45</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>89.09999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1415</v>
+        <v>1455</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>15400</v>
+        <v>15690</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1510</v>
+        <v>1500</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>31.45</v>
+        <v>34.55</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>77</v>
+        <v>80.8</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>150.5</v>
+        <v>152</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>115.5</v>
+        <v>117</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>87.90000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>521</v>
+        <v>536</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>241.5</v>
+        <v>248</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>102.5</v>
+        <v>105.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>71.40000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.7</v>
+        <v>64</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.3</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>53.9</v>
+        <v>54.3</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>74.90000000000001</v>
+        <v>74.8</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>398</v>
+        <v>399.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.6</v>
+        <v>51.3</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>768</v>
+        <v>800</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>195</v>
+        <v>192.5</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>169</v>
+        <v>185.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>203.5</v>
+        <v>198</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>99.90000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>48.05</v>
+        <v>48.35</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1270</v>
+        <v>1300</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>67.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>66.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>80.90000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>477</v>
+        <v>500</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>56.7</v>
+        <v>58.6</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>139.5</v>
+        <v>142.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>530</v>
+        <v>583</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>181.5</v>
+        <v>181</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>154</v>
+        <v>161.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5600</v>
+        <v>5040</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>273.5</v>
+        <v>286</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>198.5</v>
+        <v>204</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>61.9</v>
+        <v>66.3</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>199.5</v>
+        <v>208</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1485</v>
+        <v>1530</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>181.5</v>
+        <v>199.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>44</v>
+        <v>45.3</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>77</v>
+        <v>78.2</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>233.5</v>
+        <v>242</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>383.5</v>
+        <v>400</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1020</v>
+        <v>1030</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>451.5</v>
+        <v>469</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1605</v>
+        <v>1610</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>26.45</v>
+        <v>26.3</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1490</v>
+        <v>1585</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>423</v>
+        <v>454.5</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>67.7</v>
+        <v>69</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>470</v>
+        <v>457</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>980</v>
+        <v>949</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>372.5</v>
+        <v>379</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>71</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>2680</v>
+        <v>2620</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6255</v>
+        <v>6025</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>136</v>
+        <v>141.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>876</v>
+        <v>916</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>77.5</v>
+        <v>82.5</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>56.3</v>
+        <v>61.9</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>70.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>145.5</v>
+        <v>146.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>594</v>
+        <v>604</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>61.6</v>
+        <v>62.1</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>138.5</v>
+        <v>139.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>247.5</v>
+        <v>260.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>980</v>
+        <v>1005</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>414.5</v>
+        <v>433</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>346</v>
+        <v>355.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>6440</v>
+        <v>6785</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>264</v>
+        <v>264.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>270.5</v>
+        <v>276.5</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1130</v>
+        <v>1135</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>363.5</v>
+        <v>363</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>960</v>
+        <v>999</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>139.5</v>
+        <v>144</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.8</v>
+        <v>56.3</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>65.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>69</v>
+        <v>70.2</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1065</v>
+        <v>1040</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>420.5</v>
+        <v>458.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>269</v>
+        <v>268.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>1845</v>
+        <v>2025</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>491</v>
+        <v>526</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>562</v>
+        <v>576</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>159.5</v>
+        <v>175</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>16.35</v>
+        <v>16.7</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>306</v>
+        <v>313.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>105.5</v>
+        <v>106</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>712</v>
+        <v>727</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>1355</v>
+        <v>1490</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.25</v>
+        <v>31.7</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1635</v>
+        <v>1610</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>515</v>
+        <v>493</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2890</v>
+        <v>3100</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>505</v>
+        <v>490</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>382</v>
+        <v>376.5</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2350</v>
+        <v>2370</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1810</v>
+        <v>1805</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>283</v>
+        <v>291.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6210</v>
+        <v>6335</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.85</v>
+        <v>16.9</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>258.5</v>
+        <v>273.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>551</v>
+        <v>580</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>356.5</v>
+        <v>366</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>925</v>
+        <v>928</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1520</v>
+        <v>1580</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>292.5</v>
+        <v>296</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>404</v>
+        <v>418.5</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>169.5</v>
+        <v>178</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>242</v>
+        <v>246.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>179</v>
+        <v>192.5</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>291.5</v>
+        <v>320.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1160</v>
+        <v>1180</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>96.90000000000001</v>
+        <v>103.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>158.5</v>
+        <v>160</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>49.3</v>
+        <v>51.3</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>115.5</v>
+        <v>117</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>215</v>
+        <v>216.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>107.5</v>
+        <v>108</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>45.65</v>
+        <v>45.8</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>94</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>61.5</v>
+        <v>62.8</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>87.5</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>324</v>
+        <v>350.5</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>965</v>
+        <v>974</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>177.5</v>
+        <v>186</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2085</v>
+        <v>2125</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>429</v>
+        <v>449.5</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>38.15</v>
+        <v>37.7</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>27.2</v>
+        <v>27.25</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>251.5</v>
+        <v>255</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>367.5</v>
+        <v>373.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57</v>
+        <v>57.1</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1215</v>
+        <v>1195</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>73</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>25.1</v>
+        <v>25.05</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29</v>
+        <v>29.15</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>70</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>83</v>
+        <v>83.2</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>86.2</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33853,7 +33853,7 @@
         <v>15.67</v>
       </c>
       <c r="Q492" s="3" t="n">
-        <v>110.5</v>
+        <v>111</v>
       </c>
       <c r="R492" s="3" t="n">
         <v>5.7</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.9</v>
+        <v>39.95</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63.2</v>
+        <v>63.7</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>42.2</v>
+        <v>42</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55</v>
+        <v>55.3</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>132.5</v>
+        <v>133</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>86.8</v>
+        <v>85.8</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.75</v>
+        <v>28.9</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>94.8</v>
+        <v>95.3</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-08-27
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.3</v>
+        <v>24.1</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.2</v>
+        <v>35.1</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>26.8</v>
+        <v>26.6</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.7</v>
+        <v>52.4</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>109</v>
+        <v>108.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>77.7</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.95</v>
+        <v>28.85</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.95</v>
+        <v>42.15</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>81.2</v>
+        <v>81</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157.5</v>
+        <v>157</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>60.1</v>
+        <v>63.1</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>207</v>
+        <v>227.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.9</v>
+        <v>12.15</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>7.99</v>
+        <v>8.16</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>82.3</v>
+        <v>81.7</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.55</v>
+        <v>28.4</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.85</v>
+        <v>25</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>17.9</v>
+        <v>18.05</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.75</v>
+        <v>13.85</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>197</v>
+        <v>198.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>202</v>
+        <v>212.5</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>71.40000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>166</v>
+        <v>170.5</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>717</v>
+        <v>770</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>50.1</v>
+        <v>51.1</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1470</v>
+        <v>1480</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>39.4</v>
+        <v>38.9</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>37.6</v>
+        <v>38.2</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>38</v>
+        <v>37.75</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50.1</v>
+        <v>50.7</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>44.2</v>
+        <v>43.5</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>39.9</v>
+        <v>39.85</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>88</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>128.5</v>
+        <v>128</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>160.5</v>
+        <v>160</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>195.5</v>
+        <v>194</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>59.7</v>
+        <v>59.2</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>35.6</v>
+        <v>35.95</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>118</v>
+        <v>116.5</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>25.35</v>
+        <v>25.45</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.55</v>
+        <v>13.5</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>30.4</v>
+        <v>30.6</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.35</v>
+        <v>19.15</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>82.2</v>
+        <v>80.8</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.25</v>
+        <v>17.15</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.90000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>50</v>
+        <v>48.65</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>353</v>
+        <v>359.5</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>14510</v>
+        <v>14340</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>149</v>
+        <v>149.5</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>33</v>
+        <v>32.9</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.2</v>
+        <v>27.75</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>31.4</v>
+        <v>31.1</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.25</v>
+        <v>17.1</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>28.8</v>
+        <v>28.65</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.6</v>
+        <v>63.5</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.7</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48.35</v>
+        <v>47.85</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.55</v>
+        <v>31.6</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>123.5</v>
+        <v>118.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1750</v>
+        <v>1770</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.9</v>
+        <v>31.7</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>161</v>
+        <v>160.5</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>246.5</v>
+        <v>252</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>40.95</v>
+        <v>39.75</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>537</v>
+        <v>555</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>45.35</v>
+        <v>46.7</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>44.15</v>
+        <v>43.8</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2415</v>
+        <v>2410</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>125.5</v>
+        <v>127.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>39.65</v>
+        <v>39.2</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>181.5</v>
+        <v>186</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2055</v>
+        <v>2090</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>87.09999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>61.5</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>42.65</v>
+        <v>44.4</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>66.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>146.5</v>
+        <v>147.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>1980</v>
+        <v>1990</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>49.2</v>
+        <v>48.55</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51.3</v>
+        <v>50.7</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>44.8</v>
+        <v>45.55</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1040</v>
+        <v>1030</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>27.65</v>
+        <v>29.2</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>70.09999999999999</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>124</v>
+        <v>130.5</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>351.5</v>
+        <v>345</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>332.5</v>
+        <v>333.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5895</v>
+        <v>5500</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>74</v>
+        <v>72.5</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.15</v>
+        <v>46.65</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>66.8</v>
+        <v>66.5</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>688</v>
+        <v>675</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.65</v>
+        <v>25.75</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>56.1</v>
+        <v>56.7</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1080</v>
+        <v>1075</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>517</v>
+        <v>541</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>25.5</v>
+        <v>25.25</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>136</v>
+        <v>135.5</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>151.5</v>
+        <v>159.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>99.8</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>244</v>
+        <v>247.5</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>3945</v>
+        <v>3865</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>105</v>
+        <v>105.5</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>570</v>
+        <v>585</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>218.5</v>
+        <v>229</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>206.5</v>
+        <v>207.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>125.5</v>
+        <v>126.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>156</v>
+        <v>156.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>150.5</v>
+        <v>146.5</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>262.5</v>
+        <v>259</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>41.5</v>
+        <v>40.05</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>269.5</v>
+        <v>285</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>181.5</v>
+        <v>185</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.7</v>
+        <v>40.5</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>32.1</v>
+        <v>31.95</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12</v>
+        <v>12.05</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>35.8</v>
+        <v>35.65</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.6</v>
+        <v>19.35</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>90.40000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>34.9</v>
+        <v>34.5</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>47.2</v>
+        <v>48</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>48</v>
+        <v>47.75</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.9</v>
+        <v>35.25</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>96</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>231</v>
+        <v>232.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>34.85</v>
+        <v>34.4</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>72</v>
+        <v>74.3</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.6</v>
+        <v>57.9</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>115</v>
+        <v>113.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>43</v>
+        <v>42.75</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>69</v>
+        <v>70.3</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>91.2</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>179</v>
+        <v>178.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>46.35</v>
+        <v>45.85</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>235</v>
+        <v>233.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.6</v>
+        <v>22.35</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.55</v>
+        <v>17.4</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>223</v>
+        <v>220.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>59.3</v>
+        <v>58.6</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>273.5</v>
+        <v>274</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6290</v>
+        <v>6915</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>129.5</v>
+        <v>129</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>87.2</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>132.5</v>
+        <v>132</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>102</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3155</v>
+        <v>3340</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>92.5</v>
+        <v>91.5</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>314.5</v>
+        <v>320</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>614</v>
+        <v>675</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>66.3</v>
+        <v>65.5</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>288.5</v>
+        <v>296.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>45.4</v>
+        <v>45.2</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>557</v>
+        <v>548</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>180.5</v>
+        <v>176.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>196.5</v>
+        <v>193</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>1160</v>
+        <v>1180</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>185.5</v>
+        <v>192</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3255</v>
+        <v>3370</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>125</v>
+        <v>123.5</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>165.5</v>
+        <v>168.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>405</v>
+        <v>445.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2485</v>
+        <v>2490</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>185.5</v>
+        <v>182.5</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>68</v>
+        <v>67.2</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>716</v>
+        <v>742</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>881</v>
+        <v>914</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>364</v>
+        <v>397.5</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>136.5</v>
+        <v>138</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>197.5</v>
+        <v>198</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>182</v>
+        <v>179.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>180.5</v>
+        <v>180</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>416</v>
+        <v>415.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>217.5</v>
+        <v>219.5</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>173.5</v>
+        <v>176.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>140.5</v>
+        <v>142</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>108</v>
+        <v>111.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1075</v>
+        <v>1060</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>209.5</v>
+        <v>217</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>202</v>
+        <v>204.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>650</v>
+        <v>704</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>333.5</v>
+        <v>351</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>27.75</v>
+        <v>27.85</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>759</v>
+        <v>834</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>180.5</v>
+        <v>182.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>6125</v>
+        <v>5920</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>46.4</v>
+        <v>46.25</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1345</v>
+        <v>1425</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>280</v>
+        <v>281.5</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2410</v>
+        <v>2650</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>741</v>
+        <v>760</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>255.5</v>
+        <v>254</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>159.5</v>
+        <v>160</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>251.5</v>
+        <v>248.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5725</v>
+        <v>5645</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>3960</v>
+        <v>3870</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2005</v>
+        <v>2055</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>68.09999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>283</v>
+        <v>278.5</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>488</v>
+        <v>490.5</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>108</v>
+        <v>101.5</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>42</v>
+        <v>42.45</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>55.8</v>
+        <v>56</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>91.5</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>592</v>
+        <v>605</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>62.7</v>
+        <v>63.5</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>114</v>
+        <v>116.5</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>78.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.9</v>
+        <v>29.85</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>32.1</v>
+        <v>31.85</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>123</v>
+        <v>122.5</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>169.5</v>
+        <v>168</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>203</v>
+        <v>215.5</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>463</v>
+        <v>468.5</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>301</v>
+        <v>302.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>34.65</v>
+        <v>32.2</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>47.8</v>
+        <v>47.15</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>755</v>
+        <v>789</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>46.6</v>
+        <v>45.8</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>344.5</v>
+        <v>345</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>324.5</v>
+        <v>329</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>261</v>
+        <v>265.5</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>101</v>
+        <v>101.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>37.3</v>
+        <v>37.2</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>60.2</v>
+        <v>59.8</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>255.5</v>
+        <v>265.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>89.3</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>453</v>
+        <v>477</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>165.5</v>
+        <v>165</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>576</v>
+        <v>590</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>272.5</v>
+        <v>275.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>552</v>
+        <v>567</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>598</v>
+        <v>617</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>489.5</v>
+        <v>538</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56.5</v>
+        <v>55.9</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.55</v>
+        <v>33.6</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.45</v>
+        <v>21.35</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>91.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1455</v>
+        <v>1465</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>15690</v>
+        <v>15305</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1500</v>
+        <v>1490</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>34.55</v>
+        <v>38</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>80.8</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>117</v>
+        <v>116.5</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>77.40000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>96.59999999999999</v>
+        <v>95.2</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>105.5</v>
+        <v>106.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>72.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>98.7</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>64</v>
+        <v>63.8</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>76.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>54.3</v>
+        <v>52.3</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>117</v>
+        <v>114.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>185.5</v>
+        <v>186</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>74.8</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.4</v>
+        <v>14.85</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>399.5</v>
+        <v>409</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>290</v>
+        <v>295.5</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>800</v>
+        <v>784</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>192.5</v>
+        <v>193</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>185.5</v>
+        <v>187.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>198</v>
+        <v>217.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>98.2</v>
+        <v>95.5</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>48.35</v>
+        <v>47.9</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1300</v>
+        <v>1430</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>68.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>68.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>500</v>
+        <v>497.5</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>58.6</v>
+        <v>59.2</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>142.5</v>
+        <v>140.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>583</v>
+        <v>563</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>181</v>
+        <v>182.5</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>161.5</v>
+        <v>177.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5040</v>
+        <v>5090</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>66.3</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1530</v>
+        <v>1445</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>199.5</v>
+        <v>206</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>45.3</v>
+        <v>45.15</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>78.2</v>
+        <v>77.8</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>241</v>
+        <v>250.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>400</v>
+        <v>417</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1030</v>
+        <v>1045</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>78</v>
+        <v>78.5</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>398</v>
+        <v>393.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>469</v>
+        <v>470.5</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1610</v>
+        <v>1595</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>26.3</v>
+        <v>26.7</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1585</v>
+        <v>1560</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>454.5</v>
+        <v>452</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>69</v>
+        <v>71.8</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>457</v>
+        <v>439.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>949</v>
+        <v>958</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>2620</v>
+        <v>2740</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6025</v>
+        <v>6105</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>595</v>
+        <v>610</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>82.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.9</v>
+        <v>63.1</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>74.09999999999999</v>
+        <v>75</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>146.5</v>
+        <v>148</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>604</v>
+        <v>620</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>62.1</v>
+        <v>61.6</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>139.5</v>
+        <v>142</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>260.5</v>
+        <v>266</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1005</v>
+        <v>1075</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>433</v>
+        <v>442.5</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>355.5</v>
+        <v>355</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>6785</v>
+        <v>6815</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>264.5</v>
+        <v>277.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>276.5</v>
+        <v>281.5</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1135</v>
+        <v>1245</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>363</v>
+        <v>351.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>195</v>
+        <v>194.5</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>999</v>
+        <v>1095</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>144</v>
+        <v>144.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>70.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1040</v>
+        <v>1140</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>458.5</v>
+        <v>462.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>268.5</v>
+        <v>270.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2025</v>
+        <v>2225</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>175</v>
+        <v>173.5</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>16.7</v>
+        <v>16.55</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>313.5</v>
+        <v>314</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>727</v>
+        <v>716</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.7</v>
+        <v>31.35</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1610</v>
+        <v>1595</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>3100</v>
+        <v>2870</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>490</v>
+        <v>503</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>376.5</v>
+        <v>373</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2370</v>
+        <v>2450</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1805</v>
+        <v>1985</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>291.5</v>
+        <v>290</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6335</v>
+        <v>6345</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.9</v>
+        <v>17.05</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>273.5</v>
+        <v>298</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>580</v>
+        <v>545</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>366</v>
+        <v>383.5</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>928</v>
+        <v>957</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1580</v>
+        <v>1650</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>418.5</v>
+        <v>422.5</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>246.5</v>
+        <v>248.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>192.5</v>
+        <v>199</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>320.5</v>
+        <v>352.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1180</v>
+        <v>1295</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>103.5</v>
+        <v>104.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>51.3</v>
+        <v>50.7</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>262</v>
+        <v>261.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>216.5</v>
+        <v>218</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>45.8</v>
+        <v>46.15</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>93.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>198</v>
+        <v>197.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>62.8</v>
+        <v>63.3</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>91.09999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>350.5</v>
+        <v>364.5</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>974</v>
+        <v>960</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2125</v>
+        <v>2155</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>449.5</v>
+        <v>494</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.7</v>
+        <v>37.25</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>27.25</v>
+        <v>27</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>255</v>
+        <v>255.5</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>373.5</v>
+        <v>368.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>144</v>
+        <v>144.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57.1</v>
+        <v>57.4</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1195</v>
+        <v>1310</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>25.05</v>
+        <v>24.8</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.35</v>
+        <v>15.45</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.15</v>
+        <v>29</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>67.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>83.2</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>84.90000000000001</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>104.5</v>
+        <v>105</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.95</v>
+        <v>39.8</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63.7</v>
+        <v>63.1</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>42</v>
+        <v>41.6</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.3</v>
+        <v>55.1</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>85.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.9</v>
+        <v>28.6</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>95.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-08-29
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.1</v>
+        <v>24.3</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.1</v>
+        <v>34.55</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>26.6</v>
+        <v>26.45</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.4</v>
+        <v>52</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.85</v>
+        <v>28.65</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>81</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157</v>
+        <v>156.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>63.1</v>
+        <v>62.7</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>227.5</v>
+        <v>220.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.4</v>
+        <v>12.05</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>12.15</v>
+        <v>11.85</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.16</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>81.7</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>63.2</v>
+        <v>62.1</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.4</v>
+        <v>28.1</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>25</v>
+        <v>24.3</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.40000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.05</v>
+        <v>17.85</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.85</v>
+        <v>13.7</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>314</v>
+        <v>311.5</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>198.5</v>
+        <v>195.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>212.5</v>
+        <v>205.5</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>73.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>170.5</v>
+        <v>168</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>770</v>
+        <v>755</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>51.1</v>
+        <v>50.3</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1480</v>
+        <v>1415</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>38.2</v>
+        <v>37.85</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.75</v>
+        <v>38.1</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50.7</v>
+        <v>51</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>39.85</v>
+        <v>39.8</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.55</v>
+        <v>16.7</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>75.8</v>
+        <v>77.7</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.7</v>
+        <v>10.75</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>86.59999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>128</v>
+        <v>125.5</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>160</v>
+        <v>159.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>103</v>
+        <v>103.5</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19.05</v>
+        <v>19.1</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>59.2</v>
+        <v>60.8</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>35.95</v>
+        <v>34.8</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>116.5</v>
+        <v>125.5</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>25.45</v>
+        <v>25.15</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>30.6</v>
+        <v>29.9</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.15</v>
+        <v>19.05</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>80.8</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.15</v>
+        <v>17.05</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>65.2</v>
+        <v>64.5</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.85</v>
+        <v>13.65</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>48.65</v>
+        <v>48.4</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>359.5</v>
+        <v>354</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>14340</v>
+        <v>14300</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>149.5</v>
+        <v>144</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>32.9</v>
+        <v>31.75</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>27.75</v>
+        <v>28.2</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>31.1</v>
+        <v>30.55</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.1</v>
+        <v>16.85</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>28.65</v>
+        <v>28.4</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54</v>
+        <v>53.4</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.5</v>
+        <v>63.1</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.4</v>
+        <v>19.2</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.40000000000001</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.85</v>
+        <v>48</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.6</v>
+        <v>31.3</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>301</v>
+        <v>317.5</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>118.5</v>
+        <v>130</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1770</v>
+        <v>1830</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.7</v>
+        <v>31.8</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>160.5</v>
+        <v>164</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>39.75</v>
+        <v>39.7</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>555</v>
+        <v>597</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.7</v>
+        <v>46.6</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2410</v>
+        <v>2420</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>127.5</v>
+        <v>126.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>39.2</v>
+        <v>40</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>186</v>
+        <v>181.5</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2090</v>
+        <v>2125</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>86.8</v>
+        <v>86.5</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>240</v>
+        <v>239.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28</v>
+        <v>28.2</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.2</v>
+        <v>30.85</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>63.9</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>44.4</v>
+        <v>44.5</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>147.5</v>
+        <v>145.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>48.55</v>
+        <v>47.75</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>50.7</v>
+        <v>51.8</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>45.55</v>
+        <v>44.8</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1030</v>
+        <v>1130</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>130.5</v>
+        <v>133</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>333.5</v>
+        <v>332.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5500</v>
+        <v>5490</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>72.5</v>
+        <v>73.3</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>46.65</v>
+        <v>44.5</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>66.5</v>
+        <v>66.2</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.75</v>
+        <v>25.9</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>56.7</v>
+        <v>56.6</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>25.25</v>
+        <v>25.85</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>159.5</v>
+        <v>163.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>96.59999999999999</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>78.3</v>
+        <v>78.5</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>114</v>
+        <v>118.5</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>247.5</v>
+        <v>270</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>3865</v>
+        <v>3985</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>139.5</v>
+        <v>138.5</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>211</v>
+        <v>190</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>105.5</v>
+        <v>104.5</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>585</v>
+        <v>610</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>229</v>
+        <v>232.5</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>207.5</v>
+        <v>206.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>126.5</v>
+        <v>125.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>125</v>
+        <v>129.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>156.5</v>
+        <v>157</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>146.5</v>
+        <v>154</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>40.05</v>
+        <v>40.2</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>285</v>
+        <v>313.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>185</v>
+        <v>181.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.5</v>
+        <v>40.55</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.9</v>
+        <v>22.5</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.95</v>
+        <v>31.7</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12.05</v>
+        <v>11.95</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>35.65</v>
+        <v>35.3</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.35</v>
+        <v>19.25</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>91.5</v>
+        <v>91</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>34.5</v>
+        <v>34.35</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>48</v>
+        <v>48.2</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47.75</v>
+        <v>47</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.6</v>
+        <v>38.3</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>35.25</v>
+        <v>34.95</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>95.90000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>171.5</v>
+        <v>172</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>232.5</v>
+        <v>231.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>34.4</v>
+        <v>35.05</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>74.3</v>
+        <v>72.2</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>52.3</v>
+        <v>51.7</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.9</v>
+        <v>56.2</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.8</v>
+        <v>20.35</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>113.5</v>
+        <v>111.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.75</v>
+        <v>41.8</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.35</v>
+        <v>26.25</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>70.3</v>
+        <v>67.8</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>94.59999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>178.5</v>
+        <v>174</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>21.1</v>
+        <v>20.85</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.85</v>
+        <v>45.35</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>181</v>
+        <v>179.5</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>233.5</v>
+        <v>234</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.35</v>
+        <v>22.1</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.4</v>
+        <v>17.45</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>220.5</v>
+        <v>218.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>58.6</v>
+        <v>57.3</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>27.2</v>
+        <v>25.85</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>274</v>
+        <v>269.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6915</v>
+        <v>7065</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>87.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>132</v>
+        <v>131.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>99.90000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3340</v>
+        <v>3360</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>138</v>
+        <v>138.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>91.5</v>
+        <v>90.3</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>675</v>
+        <v>742</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>65.5</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>112</v>
+        <v>111.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>296.5</v>
+        <v>293.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>45.2</v>
+        <v>45.05</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>176.5</v>
+        <v>180.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>1180</v>
+        <v>1110</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>192</v>
+        <v>188.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3370</v>
+        <v>3305</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>123.5</v>
+        <v>124</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>168.5</v>
+        <v>174</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>445.5</v>
+        <v>439</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2490</v>
+        <v>2485</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>182.5</v>
+        <v>181</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>67.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>776</v>
+        <v>754</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>742</v>
+        <v>783</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>914</v>
+        <v>899</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>397.5</v>
+        <v>400</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>138</v>
+        <v>137.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>179.5</v>
+        <v>178</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>180</v>
+        <v>181.5</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>415.5</v>
+        <v>412</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>219.5</v>
+        <v>235</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>176.5</v>
+        <v>186.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>142</v>
+        <v>140.5</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>111.5</v>
+        <v>116.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1060</v>
+        <v>1140</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>204.5</v>
+        <v>199.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>351</v>
+        <v>386</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>27.85</v>
+        <v>28.15</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>834</v>
+        <v>917</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>182.5</v>
+        <v>180.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5920</v>
+        <v>6015</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>578</v>
+        <v>635</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>46.25</v>
+        <v>48.6</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1425</v>
+        <v>1510</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>281.5</v>
+        <v>286</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2650</v>
+        <v>2540</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1625</v>
+        <v>1735</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.05</v>
+        <v>17.5</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>760</v>
+        <v>749</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>254</v>
+        <v>252.5</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>160</v>
+        <v>161.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>248.5</v>
+        <v>243.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5645</v>
+        <v>5785</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>3870</v>
+        <v>4065</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2055</v>
+        <v>2260</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>67.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>278.5</v>
+        <v>277.5</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>490.5</v>
+        <v>500</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>556</v>
+        <v>587</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>101.5</v>
+        <v>100</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.65</v>
+        <v>19.4</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>42.45</v>
+        <v>42</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56</v>
+        <v>55.9</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>63.6</v>
+        <v>63.8</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>605</v>
+        <v>621</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>63.5</v>
+        <v>62.6</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>116.5</v>
+        <v>125</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.85</v>
+        <v>29.9</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>31.85</v>
+        <v>31.7</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>68.09999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>122.5</v>
+        <v>121.5</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>168</v>
+        <v>167.5</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>215.5</v>
+        <v>216</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>468.5</v>
+        <v>467</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>302.5</v>
+        <v>300.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>32.2</v>
+        <v>32.55</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>213</v>
+        <v>213.5</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>47.15</v>
+        <v>46.95</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>45.8</v>
+        <v>45.65</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>228</v>
+        <v>249.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>265.5</v>
+        <v>265</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>101.5</v>
+        <v>100.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>37.2</v>
+        <v>36.4</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>59.8</v>
+        <v>59.6</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>122</v>
+        <v>122.5</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>265.5</v>
+        <v>272.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>89.40000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>477</v>
+        <v>480.5</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>275.5</v>
+        <v>273.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>538</v>
+        <v>520</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>55.9</v>
+        <v>56.4</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.6</v>
+        <v>33.3</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.35</v>
+        <v>21.3</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>302</v>
+        <v>303.5</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>94.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1465</v>
+        <v>1450</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>15305</v>
+        <v>15630</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>323</v>
+        <v>321.5</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1490</v>
+        <v>1470</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>38</v>
+        <v>34.2</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>82.40000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>116.5</v>
+        <v>116</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>95.2</v>
+        <v>96.3</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>262</v>
+        <v>264.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>106.5</v>
+        <v>112</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>73</v>
+        <v>74.8</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>98.59999999999999</v>
+        <v>98.3</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>182</v>
+        <v>183.5</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.8</v>
+        <v>62.8</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>50.6</v>
+        <v>51.2</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.7</v>
+        <v>75.3</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>854</v>
+        <v>871</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>52.3</v>
+        <v>51.5</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>114.5</v>
+        <v>113</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>74.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.85</v>
+        <v>14.5</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>409</v>
+        <v>405.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.3</v>
+        <v>51</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>295.5</v>
+        <v>297</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>784</v>
+        <v>775</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>193</v>
+        <v>192.5</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>187.5</v>
+        <v>182.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>117</v>
+        <v>116.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>217.5</v>
+        <v>239</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>95.5</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.9</v>
+        <v>47.55</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1430</v>
+        <v>1365</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>69.5</v>
+        <v>68.8</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>68.8</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>83.09999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>497.5</v>
+        <v>492.5</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>308</v>
+        <v>309.5</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>59.2</v>
+        <v>59.4</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>140.5</v>
+        <v>138.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>563</v>
+        <v>582</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>182.5</v>
+        <v>181</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>177.5</v>
+        <v>175</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5090</v>
+        <v>5030</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>72.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1445</v>
+        <v>1490</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>206</v>
+        <v>201.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>45.15</v>
+        <v>45.3</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>77.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>250.5</v>
+        <v>248</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>417</v>
+        <v>400.5</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1045</v>
+        <v>1030</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>78.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>393.5</v>
+        <v>390</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>470.5</v>
+        <v>458</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1595</v>
+        <v>1615</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>26.7</v>
+        <v>26.65</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1560</v>
+        <v>1545</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>452</v>
+        <v>453.5</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>71.8</v>
+        <v>74.3</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>439.5</v>
+        <v>435</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>958</v>
+        <v>972</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>72.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>2740</v>
+        <v>2680</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6105</v>
+        <v>6250</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>141.5</v>
+        <v>144.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>917</v>
+        <v>895</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>79.40000000000001</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>63.1</v>
+        <v>65</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>75</v>
+        <v>73.5</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322</v>
+        <v>322.5</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>620</v>
+        <v>682</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>61.6</v>
+        <v>60.5</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>266</v>
+        <v>275.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1075</v>
+        <v>1060</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>442.5</v>
+        <v>437</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>355</v>
+        <v>359.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>6815</v>
+        <v>7200</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>277.5</v>
+        <v>272.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>281.5</v>
+        <v>289.5</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1245</v>
+        <v>1200</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>625</v>
+        <v>618</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>351.5</v>
+        <v>353.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1095</v>
+        <v>1140</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>144.5</v>
+        <v>138.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>56.2</v>
+        <v>55.1</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>64.8</v>
+        <v>64.2</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>69.59999999999999</v>
+        <v>70</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1140</v>
+        <v>1130</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>462.5</v>
+        <v>461</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>270.5</v>
+        <v>271</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2225</v>
+        <v>2345</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>593</v>
+        <v>620</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>173.5</v>
+        <v>169</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>16.55</v>
+        <v>16.15</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>103</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>281</v>
+        <v>292.5</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.35</v>
+        <v>31.15</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1595</v>
+        <v>1495</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2870</v>
+        <v>2995</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2450</v>
+        <v>2300</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1985</v>
+        <v>1790</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>290</v>
+        <v>290.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6345</v>
+        <v>6490</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>17.05</v>
+        <v>16.95</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>298</v>
+        <v>327.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>545</v>
+        <v>564</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>383.5</v>
+        <v>379</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>162</v>
+        <v>159.5</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>422.5</v>
+        <v>454</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>248.5</v>
+        <v>249</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>199</v>
+        <v>189.5</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>352.5</v>
+        <v>343.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1295</v>
+        <v>1240</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>104.5</v>
+        <v>103</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>159</v>
+        <v>160.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>50.7</v>
+        <v>51.4</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>261.5</v>
+        <v>260</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>118</v>
+        <v>117.5</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>218</v>
+        <v>220.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>110</v>
+        <v>109.5</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>46.15</v>
+        <v>46</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>92.2</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>197.5</v>
+        <v>195</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>63.3</v>
+        <v>62.7</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.3</v>
+        <v>90.5</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>364.5</v>
+        <v>372</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>960</v>
+        <v>990</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>185</v>
+        <v>187.5</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>234</v>
+        <v>232.5</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2155</v>
+        <v>2150</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>494</v>
+        <v>543</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.25</v>
+        <v>36.75</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>255.5</v>
+        <v>250</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>368.5</v>
+        <v>366.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>144.5</v>
+        <v>141.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57.4</v>
+        <v>56.8</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>105</v>
+        <v>94.3</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1310</v>
+        <v>1265</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.8</v>
+        <v>24.35</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.45</v>
+        <v>15.35</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29</v>
+        <v>29.05</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.3</v>
+        <v>68.2</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.8</v>
+        <v>39.85</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>41.6</v>
+        <v>40.6</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>87.09999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.6</v>
+        <v>28</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>94.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-01
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>26.45</v>
+        <v>26.65</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52</v>
+        <v>51.4</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>108.5</v>
+        <v>107.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>75.7</v>
+        <v>76.2</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.65</v>
+        <v>28.85</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>42.15</v>
+        <v>41.8</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.59999999999999</v>
+        <v>80.5</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>156.5</v>
+        <v>157</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>62.7</v>
+        <v>66.2</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>220.5</v>
+        <v>242.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.05</v>
+        <v>12.65</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.85</v>
+        <v>12.15</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.050000000000001</v>
+        <v>8.18</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>62.1</v>
+        <v>68.3</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.1</v>
+        <v>28.35</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.3</v>
+        <v>24.6</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>17.85</v>
+        <v>18.15</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>311.5</v>
+        <v>309</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>195.5</v>
+        <v>194.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>205.5</v>
+        <v>200</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>755</v>
+        <v>729</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>50.3</v>
+        <v>49.6</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>695</v>
+        <v>683</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1415</v>
+        <v>1425</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>39</v>
+        <v>39.2</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>37.85</v>
+        <v>37.7</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>38.1</v>
+        <v>37.6</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>51</v>
+        <v>50.6</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>43.9</v>
+        <v>43.35</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>39.8</v>
+        <v>39.95</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.7</v>
+        <v>16.9</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>77.7</v>
+        <v>82.5</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.75</v>
+        <v>10.9</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.6</v>
+        <v>44.55</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>86.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>125.5</v>
+        <v>126</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>159.5</v>
+        <v>164</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>103.5</v>
+        <v>103</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.8</v>
+        <v>34.1</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>125.5</v>
+        <v>126.5</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>25.15</v>
+        <v>25.2</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.9</v>
+        <v>29.85</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.05</v>
+        <v>18.95</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>80.59999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.5</v>
+        <v>63.8</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.65</v>
+        <v>14.15</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>48.4</v>
+        <v>48.8</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>14300</v>
+        <v>14180</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>144</v>
+        <v>141.5</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.75</v>
+        <v>31.25</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.55</v>
+        <v>30.9</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>16.85</v>
+        <v>17.1</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>28.4</v>
+        <v>29.75</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>53.4</v>
+        <v>54</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.2</v>
+        <v>19.3</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48</v>
+        <v>47.4</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>230</v>
+        <v>230.5</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.3</v>
+        <v>31.1</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>317.5</v>
+        <v>305</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1830</v>
+        <v>1840</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.8</v>
+        <v>32.35</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>241</v>
+        <v>248.5</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>164</v>
+        <v>159.5</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>39.7</v>
+        <v>40.35</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>597</v>
+        <v>545</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.6</v>
+        <v>46.8</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>44.1</v>
+        <v>43.5</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2420</v>
+        <v>2405</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>20.4</v>
+        <v>19.9</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>126.5</v>
+        <v>126</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>40</v>
+        <v>39.05</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>181.5</v>
+        <v>182.5</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2125</v>
+        <v>2035</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>86.5</v>
+        <v>87</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>239.5</v>
+        <v>232.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.2</v>
+        <v>28.35</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>30.85</v>
+        <v>31.5</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>63.9</v>
+        <v>64.7</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>44.5</v>
+        <v>43.9</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>64.90000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>965</v>
+        <v>999</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>145.5</v>
+        <v>144.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2010</v>
+        <v>1960</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51.8</v>
+        <v>51.1</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>44.8</v>
+        <v>44.45</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1130</v>
+        <v>1165</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>28.5</v>
+        <v>28.05</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>332.5</v>
+        <v>338.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5490</v>
+        <v>5485</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>108</v>
+        <v>106.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>73.3</v>
+        <v>72.7</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>44.5</v>
+        <v>45</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>66.2</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.9</v>
+        <v>25.25</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>56.6</v>
+        <v>59.7</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1075</v>
+        <v>1060</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>25.85</v>
+        <v>26.65</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>135.5</v>
+        <v>136</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>163.5</v>
+        <v>179.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>96.09999999999999</v>
+        <v>97.8</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>78.5</v>
+        <v>78.8</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>118.5</v>
+        <v>115.5</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>294</v>
+        <v>294.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>3985</v>
+        <v>3925</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>434</v>
+        <v>477</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>138.5</v>
+        <v>135.5</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>104.5</v>
+        <v>99</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>232.5</v>
+        <v>224</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>206.5</v>
+        <v>208.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>129.5</v>
+        <v>123.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>40.2</v>
+        <v>42.2</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>313.5</v>
+        <v>295</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>181.5</v>
+        <v>179.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.55</v>
+        <v>40.2</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.5</v>
+        <v>22.35</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.7</v>
+        <v>31.2</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>11.95</v>
+        <v>12.05</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>35.3</v>
+        <v>36.45</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.25</v>
+        <v>18.8</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>91</v>
+        <v>90.3</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>34.35</v>
+        <v>36.15</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>48.2</v>
+        <v>49.9</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47</v>
+        <v>46.65</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.3</v>
+        <v>39.8</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.95</v>
+        <v>34.25</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>93.8</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>231.5</v>
+        <v>233.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>35.05</v>
+        <v>35.35</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>72.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>51.7</v>
+        <v>52.7</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>56.2</v>
+        <v>59.5</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.35</v>
+        <v>20.25</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>111.5</v>
+        <v>114</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.25</v>
+        <v>26</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>67.8</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.85</v>
+        <v>20.9</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.35</v>
+        <v>44.4</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>179.5</v>
+        <v>177</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>234</v>
+        <v>235.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.1</v>
+        <v>22.35</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.45</v>
+        <v>17.5</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>218.5</v>
+        <v>216.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>57.3</v>
+        <v>56</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>25.85</v>
+        <v>24.2</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>269.5</v>
+        <v>292.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>7065</v>
+        <v>7650</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>89.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131.5</v>
+        <v>128.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>99.59999999999999</v>
+        <v>103</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3360</v>
+        <v>3425</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>138.5</v>
+        <v>143</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>317</v>
+        <v>312.5</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>111.5</v>
+        <v>113</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>293.5</v>
+        <v>290.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>45.05</v>
+        <v>44.55</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>545</v>
+        <v>540</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>180.5</v>
+        <v>175</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>1110</v>
+        <v>999</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>188.5</v>
+        <v>185.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>490</v>
+        <v>496.5</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>115.5</v>
+        <v>116</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3305</v>
+        <v>3530</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>439</v>
+        <v>447.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2485</v>
+        <v>2410</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>181</v>
+        <v>182.5</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>66.40000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>754</v>
+        <v>741</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>783</v>
+        <v>794</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>899</v>
+        <v>819</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>400</v>
+        <v>386.5</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>137.5</v>
+        <v>136.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>181.5</v>
+        <v>185</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>412</v>
+        <v>413.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>186.5</v>
+        <v>178</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>140.5</v>
+        <v>138</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>707</v>
+        <v>730</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>116.5</v>
+        <v>112</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1140</v>
+        <v>1250</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>223</v>
+        <v>215.5</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>199.5</v>
+        <v>202</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>701</v>
+        <v>747</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>386</v>
+        <v>422.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>28.15</v>
+        <v>28.5</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>917</v>
+        <v>1005</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>287.5</v>
+        <v>279</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>180.5</v>
+        <v>182</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>6015</v>
+        <v>6100</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>48.6</v>
+        <v>49.85</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1510</v>
+        <v>1380</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>220</v>
+        <v>222.5</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2540</v>
+        <v>2400</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>399</v>
+        <v>379</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1735</v>
+        <v>1690</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>697</v>
+        <v>682</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.5</v>
+        <v>18.2</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>749</v>
+        <v>724</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>252.5</v>
+        <v>247</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>161.5</v>
+        <v>158</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>243.5</v>
+        <v>254</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5785</v>
+        <v>5990</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4065</v>
+        <v>4075</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2260</v>
+        <v>2170</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>67.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>277.5</v>
+        <v>272.5</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>100</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.4</v>
+        <v>19.55</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>42</v>
+        <v>41.65</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>92.5</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>63.8</v>
+        <v>62.5</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>621</v>
+        <v>584</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>62.6</v>
+        <v>61.6</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>125</v>
+        <v>120.5</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.9</v>
+        <v>29.8</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>31.7</v>
+        <v>31.25</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>167.5</v>
+        <v>162</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>162</v>
+        <v>159.5</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>216</v>
+        <v>216.5</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>300.5</v>
+        <v>293.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>32.55</v>
+        <v>33.4</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>213.5</v>
+        <v>208</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>0</v>
+        <v>402</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>46.95</v>
+        <v>46.5</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>790</v>
+        <v>769</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>45.65</v>
+        <v>46.3</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>249.5</v>
+        <v>241</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>313</v>
+        <v>310.5</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>215</v>
+        <v>212.5</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>100.5</v>
+        <v>101</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.4</v>
+        <v>36.2</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>59.6</v>
+        <v>59.4</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>122.5</v>
+        <v>120</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>272.5</v>
+        <v>259</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>88.5</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>480.5</v>
+        <v>500</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>161</v>
+        <v>162.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>273.5</v>
+        <v>276</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>568</v>
+        <v>600</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.3</v>
+        <v>33.15</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.3</v>
+        <v>21.1</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>303.5</v>
+        <v>295.5</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>91.3</v>
+        <v>90.3</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1450</v>
+        <v>1425</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>15630</v>
+        <v>16065</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>321.5</v>
+        <v>323</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1470</v>
+        <v>1450</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>34.2</v>
+        <v>36</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>84.8</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>153</v>
+        <v>151.5</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>77.5</v>
+        <v>77.2</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>96.3</v>
+        <v>94.8</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>529</v>
+        <v>515</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>264.5</v>
+        <v>267.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>74.8</v>
+        <v>74</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>201</v>
+        <v>204.5</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>183.5</v>
+        <v>178</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>62.8</v>
+        <v>61.7</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>51.2</v>
+        <v>50.5</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.3</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>871</v>
+        <v>864</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>74.2</v>
+        <v>75</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>405.5</v>
+        <v>404</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>775</v>
+        <v>755</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>182.5</v>
+        <v>175.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>116.5</v>
+        <v>115.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>93.09999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.55</v>
+        <v>47.1</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>110</v>
+        <v>105.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1365</v>
+        <v>1345</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>68.8</v>
+        <v>67.2</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>84.7</v>
+        <v>83.7</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>492.5</v>
+        <v>485</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>309.5</v>
+        <v>302.5</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>59.4</v>
+        <v>57.9</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>138.5</v>
+        <v>138</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>582</v>
+        <v>548</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>181</v>
+        <v>183.5</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>175</v>
+        <v>172.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5030</v>
+        <v>5130</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>219</v>
+        <v>208.5</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>75</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1490</v>
+        <v>1435</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>201.5</v>
+        <v>199.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>45.3</v>
+        <v>44.9</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>81.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>248</v>
+        <v>253.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>400.5</v>
+        <v>405</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>79.09999999999999</v>
+        <v>79</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>390</v>
+        <v>389.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>458</v>
+        <v>412.5</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1615</v>
+        <v>1630</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>26.65</v>
+        <v>26</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1545</v>
+        <v>1395</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>453.5</v>
+        <v>456</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>74.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>972</v>
+        <v>912</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>377</v>
+        <v>399.5</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>71.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>2680</v>
+        <v>2845</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6250</v>
+        <v>6285</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>144.5</v>
+        <v>139.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>620</v>
+        <v>607</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>895</v>
+        <v>927</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>78.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>65</v>
+        <v>63.9</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>73.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322.5</v>
+        <v>321</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>147</v>
+        <v>146.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>682</v>
+        <v>629</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.5</v>
+        <v>60.2</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>139</v>
+        <v>138.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>275.5</v>
+        <v>278.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1060</v>
+        <v>1140</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>437</v>
+        <v>411.5</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>359.5</v>
+        <v>347.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>7200</v>
+        <v>7095</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>272.5</v>
+        <v>287.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>289.5</v>
+        <v>275</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1200</v>
+        <v>1210</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>353.5</v>
+        <v>318.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>194.5</v>
+        <v>188</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1140</v>
+        <v>1180</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>138.5</v>
+        <v>140.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.1</v>
+        <v>56.1</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>64.2</v>
+        <v>65</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1130</v>
+        <v>1125</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>461</v>
+        <v>467.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>271</v>
+        <v>270.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2345</v>
+        <v>2305</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>16.15</v>
+        <v>15.85</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>99.59999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>292.5</v>
+        <v>282</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.15</v>
+        <v>31.55</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1495</v>
+        <v>1505</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>487</v>
+        <v>535</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2995</v>
+        <v>2825</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2300</v>
+        <v>2270</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1790</v>
+        <v>1615</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>290.5</v>
+        <v>291.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6490</v>
+        <v>5860</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.95</v>
+        <v>16.75</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>327.5</v>
+        <v>316</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>564</v>
+        <v>508</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>379</v>
+        <v>367.5</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>953</v>
+        <v>914</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>159.5</v>
+        <v>154.5</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1800</v>
+        <v>1765</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>454</v>
+        <v>435</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>185</v>
+        <v>179.5</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>189.5</v>
+        <v>187</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>343.5</v>
+        <v>327</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1240</v>
+        <v>1230</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>160.5</v>
+        <v>156.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>51.4</v>
+        <v>50.2</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>260</v>
+        <v>255.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>117.5</v>
+        <v>118</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>220.5</v>
+        <v>217.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>109.5</v>
+        <v>109</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>46</v>
+        <v>45.65</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>90.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>62.7</v>
+        <v>63.7</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.5</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>990</v>
+        <v>969</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>152</v>
+        <v>147.5</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>187.5</v>
+        <v>178.5</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>232.5</v>
+        <v>227.5</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2150</v>
+        <v>2165</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>27.1</v>
+        <v>26.8</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>366.5</v>
+        <v>374</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>141.5</v>
+        <v>141</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>56.8</v>
+        <v>55.9</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>94.3</v>
+        <v>96</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1265</v>
+        <v>1175</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>71.7</v>
+        <v>71.5</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.35</v>
+        <v>24.85</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.35</v>
+        <v>15.25</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.05</v>
+        <v>29</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.2</v>
+        <v>67.7</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>82.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>83.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33853,7 +33853,7 @@
         <v>15.67</v>
       </c>
       <c r="Q492" s="3" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="R492" s="3" t="n">
         <v>5.7</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.85</v>
+        <v>39.3</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63.1</v>
+        <v>63</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.6</v>
+        <v>40.5</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.1</v>
+        <v>55</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>132</v>
+        <v>131.5</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>86.59999999999999</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28</v>
+        <v>27.8</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>92.2</v>
+        <v>90.3</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-02
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>25.3</v>
+        <v>24.8</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.15</v>
+        <v>35</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.1</v>
+        <v>27.05</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>51.7</v>
+        <v>51.8</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>108</v>
+        <v>109.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>76.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.45</v>
+        <v>28.6</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.6</v>
+        <v>41.95</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.3</v>
+        <v>80.2</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157</v>
+        <v>156.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>67.8</v>
+        <v>66.8</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>234.5</v>
+        <v>237.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.65</v>
+        <v>12.6</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>12.15</v>
+        <v>12.05</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.26</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>83.2</v>
+        <v>83</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>74.3</v>
+        <v>72.8</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>29.4</v>
+        <v>29.1</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>25.65</v>
+        <v>25.35</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>67.2</v>
+        <v>67</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.35</v>
+        <v>18.25</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.85</v>
+        <v>14.2</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>314.5</v>
+        <v>314</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>195.5</v>
+        <v>196</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>208.5</v>
+        <v>206</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>73.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>103.5</v>
+        <v>103</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>761</v>
+        <v>741</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.35</v>
+        <v>49.55</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>744</v>
+        <v>704</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1445</v>
+        <v>1395</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.75</v>
+        <v>38.2</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>37.35</v>
+        <v>36.8</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.25</v>
+        <v>37.5</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>51.3</v>
+        <v>50.6</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>44</v>
+        <v>43.4</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.15</v>
+        <v>41.05</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>18.55</v>
+        <v>17.35</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>84.7</v>
+        <v>80.8</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>11.15</v>
+        <v>10.8</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.65</v>
+        <v>44.6</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>85.59999999999999</v>
+        <v>87</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>171.5</v>
+        <v>163.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>186.5</v>
+        <v>184</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>61.3</v>
+        <v>60.8</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.85</v>
+        <v>35.45</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>24.85</v>
+        <v>24.55</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.7</v>
+        <v>13.85</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.85</v>
+        <v>30.1</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>81.2</v>
+        <v>82.7</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.05</v>
+        <v>16.95</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.2</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.7</v>
+        <v>13.85</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>49.8</v>
+        <v>49.55</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>14150</v>
+        <v>13865</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>141.5</v>
+        <v>139</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.4</v>
+        <v>31.65</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.8</v>
+        <v>28.3</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>31.15</v>
+        <v>30.95</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.45</v>
+        <v>17.4</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>31.5</v>
+        <v>31.95</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54.8</v>
+        <v>54.4</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.2</v>
+        <v>63.3</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.15</v>
+        <v>19.05</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48.05</v>
+        <v>47.9</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>231</v>
+        <v>231.5</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.5</v>
+        <v>31</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>300.5</v>
+        <v>315</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>132.5</v>
+        <v>126</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1865</v>
+        <v>1730</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>33.05</v>
+        <v>33.15</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>166.5</v>
+        <v>161.5</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>39.9</v>
+        <v>39.7</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>568</v>
+        <v>540</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>47.5</v>
+        <v>47.8</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>43.7</v>
+        <v>43.35</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2440</v>
+        <v>2385</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>19.85</v>
+        <v>19.3</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>122.5</v>
+        <v>123</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>39.25</v>
+        <v>39.15</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2205</v>
+        <v>2140</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>86</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.4</v>
+        <v>28.7</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.75</v>
+        <v>32.15</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>65.90000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>44.2</v>
+        <v>44</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>144</v>
+        <v>144.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2030</v>
+        <v>1975</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>47.7</v>
+        <v>48.7</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>44.65</v>
+        <v>44.05</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1225</v>
+        <v>1175</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>28.65</v>
+        <v>28.2</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>68.7</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>359</v>
+        <v>361.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5640</v>
+        <v>5445</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>107</v>
+        <v>109.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>73.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.9</v>
+        <v>45.5</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>711</v>
+        <v>692</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.45</v>
+        <v>25.5</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>62.2</v>
+        <v>59.3</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1100</v>
+        <v>1025</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>136</v>
+        <v>137.5</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>107.5</v>
+        <v>104.5</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>256</v>
+        <v>250.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>78.59999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>119.5</v>
+        <v>116</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>279</v>
+        <v>270.5</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>295</v>
+        <v>296.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4315</v>
+        <v>4275</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>524</v>
+        <v>542</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>184.5</v>
+        <v>202</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>99.5</v>
+        <v>104</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>624</v>
+        <v>609</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>213.5</v>
+        <v>211</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>127.5</v>
+        <v>125.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>123.5</v>
+        <v>121</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>155.5</v>
+        <v>156.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>42.8</v>
+        <v>42.25</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>302.5</v>
+        <v>293</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.9</v>
+        <v>41.65</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.45</v>
+        <v>31.4</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12.05</v>
+        <v>12.1</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.1</v>
+        <v>35.85</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.75</v>
+        <v>19.25</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>89.2</v>
+        <v>89.5</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.55</v>
+        <v>34.95</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>48.1</v>
+        <v>46.9</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47.9</v>
+        <v>47.95</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.65</v>
+        <v>38.3</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.55</v>
+        <v>34.25</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>93.2</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>170.5</v>
+        <v>170</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>238</v>
+        <v>234.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>34.75</v>
+        <v>35.05</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.6</v>
+        <v>53.3</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.6</v>
+        <v>57.5</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.35</v>
+        <v>20.45</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>114.5</v>
+        <v>112</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.4</v>
+        <v>42.15</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.25</v>
+        <v>26.2</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>67</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>95.59999999999999</v>
+        <v>96.3</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45</v>
+        <v>45.15</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>232.5</v>
+        <v>234.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.2</v>
+        <v>22.35</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.4</v>
+        <v>17.8</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>56.7</v>
+        <v>57.2</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>24.75</v>
+        <v>24.05</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>118.5</v>
+        <v>116</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>278.5</v>
+        <v>281.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>7580</v>
+        <v>7810</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>128</v>
+        <v>129.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>92.40000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131.5</v>
+        <v>131</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3410</v>
+        <v>3310</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>143.5</v>
+        <v>157.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>92.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>731</v>
+        <v>686</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>64.59999999999999</v>
+        <v>66</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>297.5</v>
+        <v>288.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>44.25</v>
+        <v>44.65</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>183.5</v>
+        <v>184.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>115.5</v>
+        <v>116</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3425</v>
+        <v>3395</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>125.5</v>
+        <v>123</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>173</v>
+        <v>168.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>492</v>
+        <v>469.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2480</v>
+        <v>2405</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>64.2</v>
+        <v>63.4</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>800</v>
+        <v>774</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>874</v>
+        <v>847</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>138</v>
+        <v>135.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>196.5</v>
+        <v>195.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>182</v>
+        <v>185.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>412</v>
+        <v>412.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>237.5</v>
+        <v>233.5</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>182.5</v>
+        <v>178.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>143</v>
+        <v>141.5</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>114.5</v>
+        <v>112</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1375</v>
+        <v>1435</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>215.5</v>
+        <v>209</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>786</v>
+        <v>780</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>421.5</v>
+        <v>419.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>28.35</v>
+        <v>30.05</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1005</v>
+        <v>1050</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>284</v>
+        <v>285.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>177</v>
+        <v>172.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5995</v>
+        <v>5895</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>625</v>
+        <v>602</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>49.3</v>
+        <v>49.05</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1480</v>
+        <v>1445</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>224.5</v>
+        <v>228.5</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>285</v>
+        <v>284.5</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2640</v>
+        <v>2395</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>402</v>
+        <v>386</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1745</v>
+        <v>1705</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>773</v>
+        <v>757</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>253.5</v>
+        <v>265</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>224.5</v>
+        <v>226.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>159.5</v>
+        <v>161</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>251.5</v>
+        <v>249</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5885</v>
+        <v>5770</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4275</v>
+        <v>4200</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2315</v>
+        <v>2170</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>67.8</v>
+        <v>67</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>278.5</v>
+        <v>274</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>542</v>
+        <v>520</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>624</v>
+        <v>642</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>100.5</v>
+        <v>102</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.55</v>
+        <v>19.4</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>41.7</v>
+        <v>42.1</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>55.9</v>
+        <v>56</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>95.7</v>
+        <v>94.7</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>63.2</v>
+        <v>62.2</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>610</v>
+        <v>589</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>62.5</v>
+        <v>62</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>132.5</v>
+        <v>124.5</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.8</v>
+        <v>29.7</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>31.05</v>
+        <v>30.85</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>62.4</v>
+        <v>63.4</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>167.5</v>
+        <v>166</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>230.5</v>
+        <v>242</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>467.5</v>
+        <v>478.5</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>32.25</v>
+        <v>31.45</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>208</v>
+        <v>201.5</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>405</v>
+        <v>0</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>46.45</v>
+        <v>46.65</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>799</v>
+        <v>787</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>50</v>
+        <v>51.5</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>350</v>
+        <v>346.5</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>307.5</v>
+        <v>298</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>221.5</v>
+        <v>216</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>261.5</v>
+        <v>256</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>101</v>
+        <v>102.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>38.2</v>
+        <v>36.95</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>59.8</v>
+        <v>60.3</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>124</v>
+        <v>120.5</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>260.5</v>
+        <v>250</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>91</v>
+        <v>91.7</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>535</v>
+        <v>507</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>167.5</v>
+        <v>169.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>660</v>
+        <v>669</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>600</v>
+        <v>624</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>544</v>
+        <v>530</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56.3</v>
+        <v>55.9</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>34.15</v>
+        <v>33.55</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>91.90000000000001</v>
+        <v>91.8</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1470</v>
+        <v>1460</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>17120</v>
+        <v>17725</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1450</v>
+        <v>1420</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>35.3</v>
+        <v>34.2</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>84.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>153.5</v>
+        <v>149.5</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>119.5</v>
+        <v>117</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>95.2</v>
+        <v>92.5</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>540</v>
+        <v>535</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>275</v>
+        <v>269.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>111.5</v>
+        <v>112</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>74</v>
+        <v>73.7</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>200.5</v>
+        <v>190</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>183.5</v>
+        <v>179</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>62.4</v>
+        <v>63.2</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>883</v>
+        <v>823</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>51.7</v>
+        <v>55.6</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>185.5</v>
+        <v>185</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>73.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.3</v>
+        <v>14.15</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>408.5</v>
+        <v>404</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>50.8</v>
+        <v>51.7</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>293.5</v>
+        <v>288</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>770</v>
+        <v>721</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>194</v>
+        <v>192.5</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>183.5</v>
+        <v>182.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>117.5</v>
+        <v>117</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>261.5</v>
+        <v>260.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.55</v>
+        <v>47.2</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>116</v>
+        <v>110.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1375</v>
+        <v>1340</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>71.59999999999999</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>84.3</v>
+        <v>83.5</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>507</v>
+        <v>492</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>317</v>
+        <v>313.5</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>59</v>
+        <v>58.5</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>550</v>
+        <v>536</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>182.5</v>
+        <v>183</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>189.5</v>
+        <v>195.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5410</v>
+        <v>5290</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>221.5</v>
+        <v>216</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>75.2</v>
+        <v>71.7</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1450</v>
+        <v>1410</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>200</v>
+        <v>199.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>44.9</v>
+        <v>44.5</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>80.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>249</v>
+        <v>245.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>259.5</v>
+        <v>256.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1030</v>
+        <v>1005</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>79.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>396</v>
+        <v>391.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>418.5</v>
+        <v>426</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1635</v>
+        <v>1795</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>25.75</v>
+        <v>25.1</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1310</v>
+        <v>1305</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>455</v>
+        <v>500</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>420</v>
+        <v>422.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>994</v>
+        <v>967</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>396.5</v>
+        <v>394</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>76.7</v>
+        <v>78.7</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3125</v>
+        <v>3435</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>6910</v>
+        <v>7050</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>667</v>
+        <v>646</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>74.8</v>
+        <v>82.2</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.3</v>
+        <v>61.5</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>72.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322.5</v>
+        <v>325</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>150</v>
+        <v>148.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>667</v>
+        <v>658</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.2</v>
+        <v>61.2</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>138</v>
+        <v>137.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>274</v>
+        <v>264.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1120</v>
+        <v>1210</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>365</v>
+        <v>362.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>7800</v>
+        <v>2610</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>277.5</v>
+        <v>278.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>278.5</v>
+        <v>272</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1330</v>
+        <v>1460</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>631</v>
+        <v>607</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>335.5</v>
+        <v>341.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1150</v>
+        <v>1120</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>142.5</v>
+        <v>139</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.5</v>
+        <v>55.3</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>64.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>70.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1155</v>
+        <v>1115</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>490</v>
+        <v>483.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>270</v>
+        <v>269.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2285</v>
+        <v>2110</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>572</v>
+        <v>598</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>168</v>
+        <v>166.5</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>15.45</v>
+        <v>15.25</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>91.2</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>289</v>
+        <v>293.5</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>719</v>
+        <v>709</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>32.45</v>
+        <v>32.3</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1605</v>
+        <v>1520</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>280.5</v>
+        <v>277</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2880</v>
+        <v>2795</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2345</v>
+        <v>2300</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1660</v>
+        <v>1555</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>292.5</v>
+        <v>286</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>5870</v>
+        <v>5710</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.85</v>
+        <v>17.05</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>117.5</v>
+        <v>116.5</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>320.5</v>
+        <v>316</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>538</v>
+        <v>515</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>510</v>
+        <v>523</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>940</v>
+        <v>930</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1810</v>
+        <v>1760</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>297.5</v>
+        <v>295</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>255</v>
+        <v>245.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>185.5</v>
+        <v>181</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>319</v>
+        <v>313.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1225</v>
+        <v>1200</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>105</v>
+        <v>104.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>158</v>
+        <v>154.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>50.3</v>
+        <v>50.6</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>259.5</v>
+        <v>257.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>221</v>
+        <v>220.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>111.5</v>
+        <v>109.5</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>45.15</v>
+        <v>44.7</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>91.3</v>
+        <v>91.2</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>196</v>
+        <v>198.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>63.5</v>
+        <v>62.6</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>93.2</v>
+        <v>90.2</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>369.5</v>
+        <v>369</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>990</v>
+        <v>968</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>150</v>
+        <v>146.5</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>226</v>
+        <v>225.5</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2125</v>
+        <v>2065</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>526</v>
+        <v>503</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.15</v>
+        <v>37.25</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.75</v>
+        <v>26.65</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>142</v>
+        <v>144.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>93.7</v>
+        <v>90.8</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1175</v>
+        <v>1265</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>71.7</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.9</v>
+        <v>24.75</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.45</v>
+        <v>15.5</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>82.8</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>102.5</v>
+        <v>101.5</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>40.05</v>
+        <v>40</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63.2</v>
+        <v>63</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>41</v>
+        <v>40.75</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.1</v>
+        <v>55</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>132.5</v>
+        <v>131.5</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>80</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.05</v>
+        <v>28.3</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>90.59999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-03
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.8</v>
+        <v>24.45</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35</v>
+        <v>35.2</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.05</v>
+        <v>27.8</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>109.5</v>
+        <v>110</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>76.59999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.6</v>
+        <v>28.55</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.95</v>
+        <v>42.1</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.2</v>
+        <v>80</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>156.5</v>
+        <v>155.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>66.8</v>
+        <v>65.7</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>237.5</v>
+        <v>221</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.6</v>
+        <v>12.45</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>12.05</v>
+        <v>11.9</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.220000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>83</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>72.8</v>
+        <v>69.7</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>25.35</v>
+        <v>24.6</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>67</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.25</v>
+        <v>18.1</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>314</v>
+        <v>313.5</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>165</v>
+        <v>162.5</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>103</v>
+        <v>100.5</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>741</v>
+        <v>722</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.55</v>
+        <v>49.2</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1395</v>
+        <v>1375</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.2</v>
+        <v>37.6</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.8</v>
+        <v>36.35</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.5</v>
+        <v>37</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>43.4</v>
+        <v>41.55</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>41.05</v>
+        <v>40.6</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>17.35</v>
+        <v>16.55</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>80.8</v>
+        <v>76.8</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.6</v>
+        <v>44.65</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>87</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>163.5</v>
+        <v>161</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>184</v>
+        <v>181.5</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>60.8</v>
+        <v>58.6</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>35.45</v>
+        <v>35.8</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>24.55</v>
+        <v>25.1</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.85</v>
+        <v>13.65</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>30.1</v>
+        <v>30.3</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.05</v>
+        <v>19</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>82.7</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.45</v>
+        <v>22.55</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>16.95</v>
+        <v>16.9</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.85</v>
+        <v>13.8</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>49.55</v>
+        <v>50.2</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>352</v>
+        <v>344.5</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>13865</v>
+        <v>13450</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.65</v>
+        <v>31.4</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.3</v>
+        <v>27.95</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.95</v>
+        <v>30.7</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.4</v>
+        <v>17.2</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>31.95</v>
+        <v>31.4</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.3</v>
+        <v>63.1</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>19.05</v>
+        <v>18.85</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.9</v>
+        <v>47.6</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>231.5</v>
+        <v>229.5</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31</v>
+        <v>30.1</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>315</v>
+        <v>299</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1730</v>
+        <v>1760</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>33.15</v>
+        <v>31.8</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>161.5</v>
+        <v>153</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>251</v>
+        <v>247.5</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>39.7</v>
+        <v>38.75</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>540</v>
+        <v>511</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>47.8</v>
+        <v>45.8</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>43.35</v>
+        <v>42.25</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2385</v>
+        <v>2390</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>19.3</v>
+        <v>18.65</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>39.15</v>
+        <v>38.05</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2140</v>
+        <v>2090</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>87.40000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.7</v>
+        <v>28.5</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>32.15</v>
+        <v>31.25</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>66.3</v>
+        <v>63.7</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>44</v>
+        <v>41.85</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>66.59999999999999</v>
+        <v>65</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>1010</v>
+        <v>971</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>144.5</v>
+        <v>140.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>1975</v>
+        <v>2015</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>48.7</v>
+        <v>47.25</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51</v>
+        <v>50.1</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>44.05</v>
+        <v>42.3</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1175</v>
+        <v>1100</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>28.2</v>
+        <v>27.6</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>70.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>361.5</v>
+        <v>350.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>155</v>
+        <v>150.5</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>744</v>
+        <v>707</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5445</v>
+        <v>5290</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>109.5</v>
+        <v>107.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>76.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.5</v>
+        <v>45.35</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>66</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>692</v>
+        <v>674</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.5</v>
+        <v>24.85</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>59.3</v>
+        <v>57.3</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1025</v>
+        <v>1035</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>518</v>
+        <v>477.5</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>26.4</v>
+        <v>26.55</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>137.5</v>
+        <v>138</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>168</v>
+        <v>164.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>104.5</v>
+        <v>95</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>250.5</v>
+        <v>244.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>78.3</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>116</v>
+        <v>113.5</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>270.5</v>
+        <v>261</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>296.5</v>
+        <v>286</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4275</v>
+        <v>4340</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>542</v>
+        <v>525</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>104</v>
+        <v>94.7</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>609</v>
+        <v>595</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>211</v>
+        <v>206.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>125.5</v>
+        <v>122.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>121</v>
+        <v>114.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>156.5</v>
+        <v>155.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>288</v>
+        <v>259.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>42.25</v>
+        <v>40.9</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>293</v>
+        <v>271.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>41.65</v>
+        <v>41.6</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12.1</v>
+        <v>11.95</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>35.85</v>
+        <v>36.9</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.25</v>
+        <v>19.55</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>89.5</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>34.95</v>
+        <v>35.1</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>46.9</v>
+        <v>47.15</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47.95</v>
+        <v>48.65</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.3</v>
+        <v>38.35</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.25</v>
+        <v>34.65</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>93.40000000000001</v>
+        <v>93.5</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>234.5</v>
+        <v>239</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>35.05</v>
+        <v>35.5</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>75.09999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.3</v>
+        <v>53.4</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.5</v>
+        <v>57.8</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.45</v>
+        <v>20.55</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>112</v>
+        <v>115.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.15</v>
+        <v>42.8</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>66.40000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>96.3</v>
+        <v>99.8</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>176</v>
+        <v>171.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.65</v>
+        <v>20.7</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.15</v>
+        <v>45.25</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>179</v>
+        <v>178.5</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>234.5</v>
+        <v>231.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.35</v>
+        <v>22.3</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>217</v>
+        <v>216.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>57.2</v>
+        <v>56.8</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>24.05</v>
+        <v>23.65</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>281.5</v>
+        <v>277</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>7810</v>
+        <v>7150</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>129.5</v>
+        <v>127.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>89.5</v>
+        <v>86</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131</v>
+        <v>130.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>100</v>
+        <v>98.3</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3310</v>
+        <v>3300</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>157.5</v>
+        <v>143</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>90.40000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>686</v>
+        <v>638</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>112.5</v>
+        <v>109</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>288.5</v>
+        <v>293.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>44.65</v>
+        <v>44.15</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>543</v>
+        <v>527</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>184.5</v>
+        <v>180</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>187</v>
+        <v>190.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>973</v>
+        <v>923</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>502</v>
+        <v>487.5</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3395</v>
+        <v>3120</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>168.5</v>
+        <v>162.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>469.5</v>
+        <v>446.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2405</v>
+        <v>2365</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>176</v>
+        <v>172.5</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>63.4</v>
+        <v>59.5</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>766</v>
+        <v>720</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>774</v>
+        <v>730</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>847</v>
+        <v>775</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>392</v>
+        <v>375</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>135.5</v>
+        <v>134</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>195.5</v>
+        <v>191.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>185.5</v>
+        <v>188.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>211</v>
+        <v>194.5</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>412.5</v>
+        <v>395</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>233.5</v>
+        <v>226</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>178.5</v>
+        <v>173</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>141.5</v>
+        <v>138</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>112</v>
+        <v>108.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1435</v>
+        <v>1350</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>780</v>
+        <v>774</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>419.5</v>
+        <v>400</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>30.05</v>
+        <v>29</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1050</v>
+        <v>991</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>285.5</v>
+        <v>280</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>172.5</v>
+        <v>165</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5895</v>
+        <v>5800</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>602</v>
+        <v>554</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>49.05</v>
+        <v>48.1</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1445</v>
+        <v>1405</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>228.5</v>
+        <v>220</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>284.5</v>
+        <v>280</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2395</v>
+        <v>2330</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1705</v>
+        <v>1670</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>710</v>
+        <v>676</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.3</v>
+        <v>17.05</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>757</v>
+        <v>742</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>265</v>
+        <v>249.5</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>226.5</v>
+        <v>221</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>249</v>
+        <v>241.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5770</v>
+        <v>5615</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4200</v>
+        <v>4050</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2170</v>
+        <v>2100</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>67</v>
+        <v>64.7</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.4</v>
+        <v>19.95</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>42.1</v>
+        <v>40</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56</v>
+        <v>55.9</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>94.7</v>
+        <v>91.5</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>62.2</v>
+        <v>60.5</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>62</v>
+        <v>61.5</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>124.5</v>
+        <v>118</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.7</v>
+        <v>77.3</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.85</v>
+        <v>30.55</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>63.4</v>
+        <v>63.2</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>164.5</v>
+        <v>163.5</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>478.5</v>
+        <v>462</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>294.5</v>
+        <v>288</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>31.45</v>
+        <v>30.4</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>201.5</v>
+        <v>195.5</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>46.65</v>
+        <v>44.75</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>787</v>
+        <v>759</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>51.5</v>
+        <v>49.1</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>240</v>
+        <v>217.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>346.5</v>
+        <v>342</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>298</v>
+        <v>290.5</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>102.5</v>
+        <v>103.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.95</v>
+        <v>35.5</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>60.3</v>
+        <v>59.6</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>120.5</v>
+        <v>115</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>250</v>
+        <v>239.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>91.7</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>507</v>
+        <v>464</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>169.5</v>
+        <v>166</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>579</v>
+        <v>558</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>278</v>
+        <v>272.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>669</v>
+        <v>611</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>624</v>
+        <v>572</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>530</v>
+        <v>484.5</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.55</v>
+        <v>33.35</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21</v>
+        <v>20.9</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>297</v>
+        <v>289.5</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>91.8</v>
+        <v>88.3</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1460</v>
+        <v>1440</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>17725</v>
+        <v>17850</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>355</v>
+        <v>323</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1420</v>
+        <v>1345</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>34.2</v>
+        <v>31</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>149.5</v>
+        <v>147</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>76.8</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>92.5</v>
+        <v>91.2</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>269.5</v>
+        <v>261</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>73.7</v>
+        <v>71.2</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>190</v>
+        <v>182.5</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>98.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.2</v>
+        <v>63.8</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>50.2</v>
+        <v>49.8</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>76.3</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>823</v>
+        <v>817</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>55.6</v>
+        <v>57.2</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>113</v>
+        <v>111.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>185</v>
+        <v>184.5</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>73.40000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.15</v>
+        <v>13.9</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>404</v>
+        <v>394.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.7</v>
+        <v>51.9</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>721</v>
+        <v>712</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>192.5</v>
+        <v>185</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>182.5</v>
+        <v>189</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>260.5</v>
+        <v>241</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>92.3</v>
+        <v>90.3</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.2</v>
+        <v>48.75</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>110.5</v>
+        <v>104.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1340</v>
+        <v>1300</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>67.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>83.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>492</v>
+        <v>500</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>313.5</v>
+        <v>299</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>58.5</v>
+        <v>57</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>138</v>
+        <v>134.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>536</v>
+        <v>512</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5290</v>
+        <v>5045</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>71.7</v>
+        <v>65</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>223</v>
+        <v>215.5</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1410</v>
+        <v>1345</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>199.5</v>
+        <v>191.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>44.5</v>
+        <v>43.2</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>78</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>245.5</v>
+        <v>233.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>256.5</v>
+        <v>245.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>1005</v>
+        <v>972</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>79.2</v>
+        <v>77.3</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>391.5</v>
+        <v>381</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1795</v>
+        <v>1770</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>25.1</v>
+        <v>24.55</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1305</v>
+        <v>1350</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>225</v>
+        <v>216.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>70.09999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>422.5</v>
+        <v>411.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>967</v>
+        <v>927</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>394</v>
+        <v>380.5</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>78.7</v>
+        <v>76.5</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3435</v>
+        <v>3350</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7050</v>
+        <v>7000</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>137</v>
+        <v>135.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>646</v>
+        <v>630</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>957</v>
+        <v>912</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>82.2</v>
+        <v>75.5</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.5</v>
+        <v>61.8</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>325</v>
+        <v>322.5</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>148.5</v>
+        <v>142.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>658</v>
+        <v>629</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>61.2</v>
+        <v>60.9</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>137.5</v>
+        <v>137</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>264.5</v>
+        <v>257</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1210</v>
+        <v>1185</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>416</v>
+        <v>403</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>362.5</v>
+        <v>363</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2610</v>
+        <v>2475</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>278.5</v>
+        <v>275</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1460</v>
+        <v>1385</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>157.5</v>
+        <v>156.5</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>341.5</v>
+        <v>307.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1120</v>
+        <v>1075</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.3</v>
+        <v>55.9</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1115</v>
+        <v>1060</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>483.5</v>
+        <v>465.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>269.5</v>
+        <v>271</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2110</v>
+        <v>2095</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>598</v>
+        <v>590</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>609</v>
+        <v>585</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>166.5</v>
+        <v>169</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>15.25</v>
+        <v>14.9</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>310</v>
+        <v>305.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>88.09999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>293.5</v>
+        <v>278</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>709</v>
+        <v>695</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>32.3</v>
+        <v>31.8</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1520</v>
+        <v>1655</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>610</v>
+        <v>575</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>277</v>
+        <v>274.5</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2795</v>
+        <v>2710</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>540</v>
+        <v>521</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>370</v>
+        <v>363.5</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2300</v>
+        <v>2200</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1555</v>
+        <v>1465</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>5710</v>
+        <v>5870</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>17.05</v>
+        <v>16.65</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>515</v>
+        <v>489</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>523</v>
+        <v>502</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>930</v>
+        <v>898</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>152</v>
+        <v>151.5</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1760</v>
+        <v>1755</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>459</v>
+        <v>413.5</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>245.5</v>
+        <v>236.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>313.5</v>
+        <v>293</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1200</v>
+        <v>1080</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>104.5</v>
+        <v>102</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>154.5</v>
+        <v>147</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>50.6</v>
+        <v>49.2</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>257.5</v>
+        <v>251.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>220.5</v>
+        <v>214.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>109.5</v>
+        <v>104</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>44.7</v>
+        <v>43.25</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>91.2</v>
+        <v>89.3</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>198.5</v>
+        <v>189</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>62.6</v>
+        <v>60.5</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>369</v>
+        <v>348</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>968</v>
+        <v>948</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>146.5</v>
+        <v>145</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>225.5</v>
+        <v>217</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2065</v>
+        <v>2000</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>503</v>
+        <v>470</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.25</v>
+        <v>37.35</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.65</v>
+        <v>26.15</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>372.5</v>
+        <v>367.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>144.5</v>
+        <v>141</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>56.3</v>
+        <v>56.6</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>90.8</v>
+        <v>89.7</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1265</v>
+        <v>1185</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.75</v>
+        <v>24.55</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.5</v>
+        <v>15.35</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29</v>
+        <v>29.05</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68</v>
+        <v>67.7</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>81</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>101.5</v>
+        <v>100.5</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>40</v>
+        <v>39.7</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63</v>
+        <v>62.4</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.75</v>
+        <v>40.8</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55</v>
+        <v>55.1</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.3</v>
+        <v>28.25</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>90.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-04
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.45</v>
+        <v>24.6</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.2</v>
+        <v>35.1</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>51.8</v>
+        <v>52.2</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>110</v>
+        <v>110.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>42.1</v>
+        <v>41.85</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>155.5</v>
+        <v>157</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>65.7</v>
+        <v>66</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>221</v>
+        <v>225.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.45</v>
+        <v>12.35</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>81.40000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>69.7</v>
+        <v>69.8</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>29.1</v>
+        <v>29.15</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.6</v>
+        <v>24.55</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.40000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>313.5</v>
+        <v>313</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>194</v>
+        <v>196.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>201</v>
+        <v>207.5</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>71</v>
+        <v>72.2</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>162.5</v>
+        <v>165.5</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>100.5</v>
+        <v>102</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>722</v>
+        <v>746</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.2</v>
+        <v>49.8</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>711</v>
+        <v>695</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1375</v>
+        <v>1395</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>37.6</v>
+        <v>38.4</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.35</v>
+        <v>36.5</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37</v>
+        <v>37.35</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50.6</v>
+        <v>51.2</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>41.55</v>
+        <v>42.3</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.6</v>
+        <v>40.65</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.55</v>
+        <v>16.65</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>76.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.65</v>
+        <v>44.8</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>86.90000000000001</v>
+        <v>86</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>122</v>
+        <v>125.5</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>161</v>
+        <v>162.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>181.5</v>
+        <v>182</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>58.6</v>
+        <v>59.1</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>35.8</v>
+        <v>34.7</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>120</v>
+        <v>118.5</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>25.1</v>
+        <v>24.8</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.65</v>
+        <v>13.5</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>30.3</v>
+        <v>29.85</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.8</v>
+        <v>13.85</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>344.5</v>
+        <v>363</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>13450</v>
+        <v>13860</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.4</v>
+        <v>31.35</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>27.95</v>
+        <v>28.25</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.7</v>
+        <v>30.95</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>31.4</v>
+        <v>31.1</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54.4</v>
+        <v>54.1</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.1</v>
+        <v>63.4</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>521</v>
+        <v>539</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>18.85</v>
+        <v>18.8</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.59999999999999</v>
+        <v>83</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.6</v>
+        <v>47.65</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>229.5</v>
+        <v>231.5</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>30.1</v>
+        <v>30.3</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1760</v>
+        <v>1825</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.8</v>
+        <v>32.85</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>236</v>
+        <v>249.5</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>247.5</v>
+        <v>256</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>38.75</v>
+        <v>41.6</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>511</v>
+        <v>562</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>45.8</v>
+        <v>46.6</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>42.25</v>
+        <v>42.9</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2390</v>
+        <v>2410</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>18.65</v>
+        <v>19.55</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>117</v>
+        <v>121.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>38.05</v>
+        <v>38.6</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2090</v>
+        <v>2100</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>86.40000000000001</v>
+        <v>88</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>223</v>
+        <v>239.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.5</v>
+        <v>29.25</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.25</v>
+        <v>32.7</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>63.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>41.85</v>
+        <v>42.8</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>65</v>
+        <v>67.5</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>971</v>
+        <v>1025</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>140.5</v>
+        <v>142</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2015</v>
+        <v>2030</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>47.25</v>
+        <v>49.3</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>50.1</v>
+        <v>51.1</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>42.3</v>
+        <v>43.1</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1100</v>
+        <v>1045</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>27.6</v>
+        <v>28.15</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>67.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>350.5</v>
+        <v>361</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>150.5</v>
+        <v>161.5</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5290</v>
+        <v>5415</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>107.5</v>
+        <v>110.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>75</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.35</v>
+        <v>45.6</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>64.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>674</v>
+        <v>711</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>24.85</v>
+        <v>25.7</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>57.3</v>
+        <v>57.1</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1035</v>
+        <v>1070</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>477.5</v>
+        <v>496</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>26.55</v>
+        <v>26.8</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>138</v>
+        <v>137.5</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>164.5</v>
+        <v>178</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>95</v>
+        <v>104.5</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>244.5</v>
+        <v>260</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>113.5</v>
+        <v>116</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>286</v>
+        <v>284.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4340</v>
+        <v>4415</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>94.7</v>
+        <v>97.2</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>206.5</v>
+        <v>209.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>122.5</v>
+        <v>121</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>114.5</v>
+        <v>125.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>155.5</v>
+        <v>156</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>259.5</v>
+        <v>256</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>271.5</v>
+        <v>298.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>179</v>
+        <v>181.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.5</v>
+        <v>22.55</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.5</v>
+        <v>31.25</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>11.95</v>
+        <v>12.15</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.9</v>
+        <v>37.1</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.55</v>
+        <v>20.15</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>88.59999999999999</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.1</v>
+        <v>35</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>48.65</v>
+        <v>48.55</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.35</v>
+        <v>38.45</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.65</v>
+        <v>34.85</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>93.5</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>35.5</v>
+        <v>35.85</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.4</v>
+        <v>53.5</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.8</v>
+        <v>58.2</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.55</v>
+        <v>20.45</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>115.5</v>
+        <v>115</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.8</v>
+        <v>42.5</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>65</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>171.5</v>
+        <v>173.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.7</v>
+        <v>20.65</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.25</v>
+        <v>45.5</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>178.5</v>
+        <v>179</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>231.5</v>
+        <v>232</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>18.2</v>
+        <v>18.15</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>216.5</v>
+        <v>216</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>56.8</v>
+        <v>57.6</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>23.65</v>
+        <v>25.6</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>277</v>
+        <v>278.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>7150</v>
+        <v>7400</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>127.5</v>
+        <v>129</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>130.5</v>
+        <v>131.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>98.3</v>
+        <v>101</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3300</v>
+        <v>3570</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>143</v>
+        <v>144.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>87.2</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>638</v>
+        <v>701</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>64</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>109</v>
+        <v>111.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>293.5</v>
+        <v>284</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>44.15</v>
+        <v>43.95</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>180</v>
+        <v>179.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>190.5</v>
+        <v>192.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>923</v>
+        <v>902</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>174</v>
+        <v>173.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>487.5</v>
+        <v>488.5</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3120</v>
+        <v>3170</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>162.5</v>
+        <v>176.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>446.5</v>
+        <v>449.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2365</v>
+        <v>2385</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>172.5</v>
+        <v>173</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>59.5</v>
+        <v>60.6</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>720</v>
+        <v>775</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>730</v>
+        <v>803</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>775</v>
+        <v>819</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>375</v>
+        <v>386</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>191.5</v>
+        <v>192</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>188.5</v>
+        <v>198</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>194.5</v>
+        <v>206</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>395</v>
+        <v>400.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>173</v>
+        <v>176.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>108.5</v>
+        <v>111</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1350</v>
+        <v>1485</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>774</v>
+        <v>735</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>400</v>
+        <v>430</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>991</v>
+        <v>1055</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>280</v>
+        <v>282.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>165</v>
+        <v>172.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5800</v>
+        <v>5810</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>554</v>
+        <v>580</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>48.1</v>
+        <v>48.5</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1405</v>
+        <v>1505</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2330</v>
+        <v>2385</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>381</v>
+        <v>399</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1670</v>
+        <v>1685</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>676</v>
+        <v>693</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.05</v>
+        <v>17.15</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>742</v>
+        <v>711</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>249.5</v>
+        <v>255</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>157</v>
+        <v>159.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>241.5</v>
+        <v>248</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5615</v>
+        <v>5875</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4050</v>
+        <v>4220</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2100</v>
+        <v>2145</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>64.7</v>
+        <v>65.5</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>648</v>
+        <v>663</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.95</v>
+        <v>20</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>40</v>
+        <v>40.1</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>55.9</v>
+        <v>56.1</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>91.5</v>
+        <v>92.5</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>60.5</v>
+        <v>62</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>61.5</v>
+        <v>66.8</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.3</v>
+        <v>77</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.6</v>
+        <v>29.8</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.55</v>
+        <v>30.15</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>63.2</v>
+        <v>63.6</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>122</v>
+        <v>121.5</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>163.5</v>
+        <v>164.5</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>161</v>
+        <v>171.5</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>462</v>
+        <v>473.5</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>288</v>
+        <v>294.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>30.4</v>
+        <v>30.1</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>195.5</v>
+        <v>200.5</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>44.75</v>
+        <v>44.65</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>759</v>
+        <v>776</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>49.1</v>
+        <v>50.3</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>217.5</v>
+        <v>231.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>290.5</v>
+        <v>306</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>217</v>
+        <v>226.5</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>103.5</v>
+        <v>104</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>35.5</v>
+        <v>36.9</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>59.6</v>
+        <v>60.8</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>239.5</v>
+        <v>251</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>90.40000000000001</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>166</v>
+        <v>165.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>272.5</v>
+        <v>276</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>611</v>
+        <v>624</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>572</v>
+        <v>629</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>484.5</v>
+        <v>497</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>55.8</v>
+        <v>56.4</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.35</v>
+        <v>33.2</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>289.5</v>
+        <v>293</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>88.3</v>
+        <v>90</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1440</v>
+        <v>1430</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>17850</v>
+        <v>17470</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1345</v>
+        <v>1360</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>79.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>110</v>
+        <v>112.5</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>75.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>91.2</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>261</v>
+        <v>261.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>110</v>
+        <v>112.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>71.2</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>182.5</v>
+        <v>190</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>176</v>
+        <v>183.5</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.8</v>
+        <v>64</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>49.8</v>
+        <v>50</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>817</v>
+        <v>853</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>57.2</v>
+        <v>56.8</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>184.5</v>
+        <v>185</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>13.9</v>
+        <v>14.05</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>394.5</v>
+        <v>397</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.9</v>
+        <v>51.5</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>280</v>
+        <v>286.5</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>712</v>
+        <v>736</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>185</v>
+        <v>182.5</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>189</v>
+        <v>182.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>114</v>
+        <v>121.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>241</v>
+        <v>260.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>90.3</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>48.75</v>
+        <v>49.2</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>104.5</v>
+        <v>111</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1300</v>
+        <v>1305</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>67.3</v>
+        <v>68</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>81.40000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>500</v>
+        <v>516</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>57</v>
+        <v>58.8</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>134.5</v>
+        <v>138.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>183</v>
+        <v>185.5</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>195.5</v>
+        <v>188.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5045</v>
+        <v>5155</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>275</v>
+        <v>276.5</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>65</v>
+        <v>67.7</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>215.5</v>
+        <v>237</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1345</v>
+        <v>1365</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>191.5</v>
+        <v>200</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>43.2</v>
+        <v>44</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>233.5</v>
+        <v>243.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>245.5</v>
+        <v>270</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>458</v>
+        <v>456.5</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>972</v>
+        <v>965</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>77.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>381</v>
+        <v>395</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>411</v>
+        <v>428.5</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1770</v>
+        <v>1755</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>24.55</v>
+        <v>24.95</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1350</v>
+        <v>1310</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>216.5</v>
+        <v>237.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>67.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>411.5</v>
+        <v>416</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>927</v>
+        <v>981</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>380.5</v>
+        <v>385</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>76.5</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7000</v>
+        <v>7075</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>135.5</v>
+        <v>138</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>75.5</v>
+        <v>79.7</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.8</v>
+        <v>61.5</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>71.3</v>
+        <v>75.2</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322.5</v>
+        <v>322</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>142.5</v>
+        <v>150.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.9</v>
+        <v>61</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>137</v>
+        <v>138.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>257</v>
+        <v>258.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1185</v>
+        <v>1250</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>403</v>
+        <v>407.5</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>363</v>
+        <v>355.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2475</v>
+        <v>2565</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>275</v>
+        <v>275.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>263</v>
+        <v>289</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1385</v>
+        <v>1360</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>603</v>
+        <v>619</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>156.5</v>
+        <v>157</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>307.5</v>
+        <v>320</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1075</v>
+        <v>1135</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>137</v>
+        <v>137.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>64</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>67.8</v>
+        <v>68.5</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1060</v>
+        <v>1115</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>465.5</v>
+        <v>468</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>271</v>
+        <v>270.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2095</v>
+        <v>2200</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>585</v>
+        <v>605</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>169</v>
+        <v>169.5</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>14.9</v>
+        <v>14.95</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>305.5</v>
+        <v>312.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>84.5</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.8</v>
+        <v>31.95</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1655</v>
+        <v>1820</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>575</v>
+        <v>632</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>274.5</v>
+        <v>280</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2710</v>
+        <v>2890</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>521</v>
+        <v>545</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>363.5</v>
+        <v>368.5</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2200</v>
+        <v>2415</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1465</v>
+        <v>1610</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>278</v>
+        <v>282.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>5870</v>
+        <v>5980</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.65</v>
+        <v>16.7</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>315</v>
+        <v>335</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>489</v>
+        <v>505</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>898</v>
+        <v>922</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>151.5</v>
+        <v>151</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1755</v>
+        <v>1930</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>290</v>
+        <v>293.5</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>413.5</v>
+        <v>420</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>177</v>
+        <v>181.5</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>236.5</v>
+        <v>239</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>293</v>
+        <v>297.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1080</v>
+        <v>1055</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>147</v>
+        <v>148.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>49.2</v>
+        <v>50.5</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>251.5</v>
+        <v>254.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>112</v>
+        <v>112.5</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>214.5</v>
+        <v>215</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>104</v>
+        <v>104.5</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>43.25</v>
+        <v>43.55</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>89.3</v>
+        <v>90.5</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>189</v>
+        <v>194.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>60.5</v>
+        <v>61.4</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>89.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>348</v>
+        <v>348.5</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>948</v>
+        <v>986</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>173</v>
+        <v>180.5</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2000</v>
+        <v>2015</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>470</v>
+        <v>500</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.35</v>
+        <v>37.55</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.15</v>
+        <v>26.1</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>367.5</v>
+        <v>373.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>56.6</v>
+        <v>57.5</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>89.7</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1185</v>
+        <v>1300</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72.2</v>
+        <v>72.3</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.55</v>
+        <v>24.6</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.35</v>
+        <v>15.25</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>67.7</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>82.09999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>79.59999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33853,7 +33853,7 @@
         <v>15.67</v>
       </c>
       <c r="Q492" s="3" t="n">
-        <v>106</v>
+        <v>106.5</v>
       </c>
       <c r="R492" s="3" t="n">
         <v>5.7</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>100.5</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.7</v>
+        <v>39.55</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>62.4</v>
+        <v>63.1</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.8</v>
+        <v>40.4</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.1</v>
+        <v>55.2</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>80.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.25</v>
+        <v>28.45</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>88.40000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-07
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.6</v>
+        <v>24.3</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.1</v>
+        <v>35.05</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.7</v>
+        <v>27.5</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.2</v>
+        <v>52.1</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>110.5</v>
+        <v>111</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>75.2</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.55</v>
+        <v>28.4</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.85</v>
+        <v>41.65</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.59999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157</v>
+        <v>157.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>66</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>225.5</v>
+        <v>230.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.35</v>
+        <v>12.2</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.119999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>69.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>29.15</v>
+        <v>28.7</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.55</v>
+        <v>24.35</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.9</v>
+        <v>13.5</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>196.5</v>
+        <v>195</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>72.2</v>
+        <v>71.7</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>165.5</v>
+        <v>167</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102</v>
+        <v>102.5</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>49.8</v>
+        <v>48.95</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>695</v>
+        <v>730</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2790,7 +2790,7 @@
         <v>59.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>66</v>
+        <v>79.5</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>2</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1395</v>
+        <v>1370</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.4</v>
+        <v>37.9</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.5</v>
+        <v>36.05</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.35</v>
+        <v>37.2</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>51.2</v>
+        <v>50</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>42.3</v>
+        <v>40.9</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.65</v>
+        <v>40.3</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.65</v>
+        <v>16.45</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>76.09999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.6</v>
+        <v>10.45</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.8</v>
+        <v>44.6</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>125.5</v>
+        <v>126</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>162.5</v>
+        <v>160.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19.1</v>
+        <v>19.4</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>182</v>
+        <v>180.5</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>59.1</v>
+        <v>60.7</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.7</v>
+        <v>34.25</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>118.5</v>
+        <v>130</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>24.8</v>
+        <v>24.45</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.5</v>
+        <v>13.2</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.85</v>
+        <v>29.1</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>81.59999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.55</v>
+        <v>22.3</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.85</v>
+        <v>13.95</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>50.2</v>
+        <v>49.1</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>363</v>
+        <v>364.5</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>13860</v>
+        <v>13905</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.35</v>
+        <v>31.1</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>28.25</v>
+        <v>27.4</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.95</v>
+        <v>30.7</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.3</v>
+        <v>16.95</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>31.1</v>
+        <v>30.8</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>54.1</v>
+        <v>53.6</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.65</v>
+        <v>48.3</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>231.5</v>
+        <v>234</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>30.3</v>
+        <v>31.5</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1825</v>
+        <v>1850</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>32.85</v>
+        <v>32.3</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>249.5</v>
+        <v>240</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>41.6</v>
+        <v>40.05</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>562</v>
+        <v>589</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.6</v>
+        <v>46</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>42.9</v>
+        <v>43.3</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2410</v>
+        <v>2460</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>19.55</v>
+        <v>19.45</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>121.5</v>
+        <v>124.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>38.6</v>
+        <v>38.55</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>88</v>
+        <v>89.3</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>239.5</v>
+        <v>233.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>29.25</v>
+        <v>29</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>32.7</v>
+        <v>32.3</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>42.8</v>
+        <v>42.2</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>67.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>1025</v>
+        <v>999</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2030</v>
+        <v>2230</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>49.3</v>
+        <v>47.95</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51.1</v>
+        <v>52.5</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>43.1</v>
+        <v>42.4</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1045</v>
+        <v>1120</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>68.3</v>
+        <v>67.5</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>361</v>
+        <v>364.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>161.5</v>
+        <v>158.5</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>713</v>
+        <v>729</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>345</v>
+        <v>347.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5415</v>
+        <v>5495</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>81.40000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>45.6</v>
+        <v>44.35</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>64.8</v>
+        <v>63.5</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>711</v>
+        <v>680</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.7</v>
+        <v>25.55</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>57.1</v>
+        <v>56.1</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1070</v>
+        <v>1080</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>496</v>
+        <v>517</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>26.8</v>
+        <v>28.7</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>137.5</v>
+        <v>138</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>178</v>
+        <v>171.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>104.5</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>260</v>
+        <v>259.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>284.5</v>
+        <v>289.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4415</v>
+        <v>4760</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>528</v>
+        <v>500</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>97.2</v>
+        <v>100.5</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>603</v>
+        <v>619</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>209.5</v>
+        <v>208.5</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>125.5</v>
+        <v>127</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>156</v>
+        <v>157.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>256</v>
+        <v>254.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>41</v>
+        <v>40.9</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>298.5</v>
+        <v>323</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>181.5</v>
+        <v>184</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>41.6</v>
+        <v>41</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.55</v>
+        <v>22.3</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.25</v>
+        <v>31.3</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12.15</v>
+        <v>11.9</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>37.1</v>
+        <v>36.6</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>20.15</v>
+        <v>19.75</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>89.40000000000001</v>
+        <v>89.2</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35</v>
+        <v>35.15</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>47.15</v>
+        <v>46.9</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>48.55</v>
+        <v>48</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.45</v>
+        <v>38.65</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.85</v>
+        <v>34.5</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>94.59999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>35.85</v>
+        <v>36.35</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>78.2</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.5</v>
+        <v>53.1</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>115</v>
+        <v>114.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.5</v>
+        <v>42.1</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>65</v>
+        <v>66.3</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>99.8</v>
+        <v>99.2</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>173.5</v>
+        <v>174</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.65</v>
+        <v>20.5</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.3</v>
+        <v>22.25</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>18.15</v>
+        <v>17.9</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>57.6</v>
+        <v>56.7</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>25.6</v>
+        <v>27.1</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>278.5</v>
+        <v>297</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>7400</v>
+        <v>6660</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>129</v>
+        <v>129.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>88</v>
+        <v>86.3</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131.5</v>
+        <v>132</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>101</v>
+        <v>100.5</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3570</v>
+        <v>3420</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>144.5</v>
+        <v>142</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>95.90000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>340</v>
+        <v>339.5</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>701</v>
+        <v>771</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>63.4</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>111.5</v>
+        <v>109.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>43.95</v>
+        <v>43.25</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>524</v>
+        <v>540</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>179.5</v>
+        <v>179</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>902</v>
+        <v>949</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>173.5</v>
+        <v>176.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>488.5</v>
+        <v>493</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3170</v>
+        <v>3070</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>176.5</v>
+        <v>171.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>449.5</v>
+        <v>450.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2385</v>
+        <v>2555</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>60.6</v>
+        <v>60.8</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>775</v>
+        <v>752</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>803</v>
+        <v>883</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>819</v>
+        <v>813</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>192</v>
+        <v>190.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>206</v>
+        <v>199.5</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>400.5</v>
+        <v>412</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>176.5</v>
+        <v>176</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>140</v>
+        <v>140.5</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>111</v>
+        <v>109.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1485</v>
+        <v>1440</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>214</v>
+        <v>213.5</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>735</v>
+        <v>723</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>430</v>
+        <v>469.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>211</v>
+        <v>206.5</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>30</v>
+        <v>29.85</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1055</v>
+        <v>987</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>282.5</v>
+        <v>284</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>172.5</v>
+        <v>169.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5810</v>
+        <v>5935</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>48.5</v>
+        <v>49.95</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1505</v>
+        <v>1510</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2385</v>
+        <v>2570</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1685</v>
+        <v>1695</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.15</v>
+        <v>17.05</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>711</v>
+        <v>722</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>255</v>
+        <v>252.5</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>224</v>
+        <v>221.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>248</v>
+        <v>248.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5875</v>
+        <v>5655</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4220</v>
+        <v>4040</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2145</v>
+        <v>2070</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>65.5</v>
+        <v>65.8</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>663</v>
+        <v>682</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>20</v>
+        <v>19.75</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>40.1</v>
+        <v>39.7</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56.1</v>
+        <v>56.4</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>92.5</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>62</v>
+        <v>61.2</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>588</v>
+        <v>621</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>66.8</v>
+        <v>67.2</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>118</v>
+        <v>119.5</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77</v>
+        <v>76.5</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.8</v>
+        <v>29.65</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.15</v>
+        <v>29.55</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>63.6</v>
+        <v>62.7</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>121.5</v>
+        <v>122.5</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>164.5</v>
+        <v>163</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>171.5</v>
+        <v>167.5</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>473.5</v>
+        <v>462</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>294.5</v>
+        <v>297.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>30.1</v>
+        <v>28.3</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>200.5</v>
+        <v>200</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>44.65</v>
+        <v>45.6</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>776</v>
+        <v>787</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>50.3</v>
+        <v>50.6</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>231.5</v>
+        <v>228</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>346</v>
+        <v>344.5</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>226.5</v>
+        <v>239</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>248</v>
+        <v>250.5</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.9</v>
+        <v>36.8</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>60.8</v>
+        <v>60.2</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>120</v>
+        <v>122.5</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>251</v>
+        <v>247.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>95.40000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>463</v>
+        <v>501</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>276</v>
+        <v>277.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>624</v>
+        <v>610</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>629</v>
+        <v>590</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56.4</v>
+        <v>56.6</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>33.2</v>
+        <v>32.75</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>20.9</v>
+        <v>20.85</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>90</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1430</v>
+        <v>1440</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>17470</v>
+        <v>19215</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>330</v>
+        <v>318.5</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1360</v>
+        <v>1405</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>32</v>
+        <v>35.2</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>79.2</v>
+        <v>81.2</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>112.5</v>
+        <v>118.5</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>92.90000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>261.5</v>
+        <v>262.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>112.5</v>
+        <v>120</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>71.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>64</v>
+        <v>63.3</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>50</v>
+        <v>49.45</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>76.59999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>853</v>
+        <v>874</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>56.8</v>
+        <v>55.2</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>111.5</v>
+        <v>112.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>72.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.05</v>
+        <v>14.2</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>397</v>
+        <v>386.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>51.5</v>
+        <v>50.8</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>286.5</v>
+        <v>288</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>182.5</v>
+        <v>181</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>182.5</v>
+        <v>191</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>121.5</v>
+        <v>116</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>260.5</v>
+        <v>286.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>91.90000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>49.2</v>
+        <v>47.4</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>111</v>
+        <v>111.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1305</v>
+        <v>1370</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>66.59999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>68</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>82.5</v>
+        <v>82.8</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>58.8</v>
+        <v>59</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>138.5</v>
+        <v>136</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>185.5</v>
+        <v>185</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>188.5</v>
+        <v>181.5</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5155</v>
+        <v>5490</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>276.5</v>
+        <v>280</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>67.7</v>
+        <v>67.8</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>237</v>
+        <v>232.5</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1365</v>
+        <v>1370</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>44</v>
+        <v>44.35</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>79.09999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>243.5</v>
+        <v>239.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>270</v>
+        <v>269.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>456.5</v>
+        <v>442.5</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>965</v>
+        <v>977</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>77.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>395</v>
+        <v>389.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>428.5</v>
+        <v>418</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1755</v>
+        <v>1700</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>24.95</v>
+        <v>24.6</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1310</v>
+        <v>1325</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>237.5</v>
+        <v>231.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>449</v>
+        <v>448.5</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>981</v>
+        <v>971</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>385</v>
+        <v>379.5</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>78.09999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3350</v>
+        <v>3470</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7075</v>
+        <v>7000</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>138</v>
+        <v>133.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>635</v>
+        <v>644</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>911</v>
+        <v>960</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>79.7</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.5</v>
+        <v>63.4</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>75.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>150.5</v>
+        <v>152</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>634</v>
+        <v>619</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>61</v>
+        <v>60.6</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>138.5</v>
+        <v>137.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>258.5</v>
+        <v>265</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1250</v>
+        <v>1300</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>407.5</v>
+        <v>411</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>355.5</v>
+        <v>356.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2565</v>
+        <v>2490</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>275.5</v>
+        <v>276</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>289</v>
+        <v>299.5</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1360</v>
+        <v>1410</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1135</v>
+        <v>1110</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.9</v>
+        <v>55.5</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>68.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1115</v>
+        <v>1080</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>270.5</v>
+        <v>271.5</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2200</v>
+        <v>2265</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>597</v>
+        <v>582</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>605</v>
+        <v>568</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>169.5</v>
+        <v>166</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>312.5</v>
+        <v>315</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>86.40000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>283</v>
+        <v>286.5</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>696</v>
+        <v>719</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>1490</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.95</v>
+        <v>31.8</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>1820</v>
+        <v>2000</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>632</v>
+        <v>660</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2890</v>
+        <v>2915</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>368.5</v>
+        <v>354</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2415</v>
+        <v>2375</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1610</v>
+        <v>1590</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>282.5</v>
+        <v>283</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>5980</v>
+        <v>6565</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.7</v>
+        <v>16.65</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>116.5</v>
+        <v>115.5</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>335</v>
+        <v>316.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>505</v>
+        <v>536</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>370</v>
+        <v>395</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>922</v>
+        <v>930</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1930</v>
+        <v>1870</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>293.5</v>
+        <v>291.5</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>420</v>
+        <v>462</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>181.5</v>
+        <v>185.5</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>239</v>
+        <v>249.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>297.5</v>
+        <v>327</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1055</v>
+        <v>1050</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>112</v>
+        <v>122.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>148.5</v>
+        <v>150.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>50.5</v>
+        <v>49.9</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>254.5</v>
+        <v>253</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>215</v>
+        <v>216.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>104.5</v>
+        <v>105</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>43.55</v>
+        <v>43.85</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>90.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>194.5</v>
+        <v>189.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>61.4</v>
+        <v>61.9</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.09999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>348.5</v>
+        <v>347</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>986</v>
+        <v>937</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>180.5</v>
+        <v>181</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2015</v>
+        <v>2095</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.55</v>
+        <v>37.2</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.1</v>
+        <v>26.05</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>373.5</v>
+        <v>361</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>142</v>
+        <v>142.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57.5</v>
+        <v>57.9</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1300</v>
+        <v>1240</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72.3</v>
+        <v>72</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.25</v>
+        <v>15.3</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.05</v>
+        <v>29.2</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.90000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>81.2</v>
+        <v>81.7</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>79.3</v>
+        <v>77.8</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>98.90000000000001</v>
+        <v>97.3</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.4</v>
+        <v>40.3</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.2</v>
+        <v>55.7</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>131.5</v>
+        <v>129</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>81.3</v>
+        <v>80.5</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.45</v>
+        <v>27.9</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>88.09999999999999</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-08
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.05</v>
+        <v>35.2</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.5</v>
+        <v>27.45</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.1</v>
+        <v>52.5</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>75.2</v>
+        <v>76.7</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.4</v>
+        <v>28.55</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.65</v>
+        <v>41.7</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.09999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157.5</v>
+        <v>157</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>66.59999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>230.5</v>
+        <v>235</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.2</v>
+        <v>12.35</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.1</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>81.7</v>
+        <v>79</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.7</v>
+        <v>28.65</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.35</v>
+        <v>24.45</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>68.3</v>
+        <v>67.5</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.1</v>
+        <v>17.8</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>207.5</v>
+        <v>204.5</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>71.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102.5</v>
+        <v>102</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>48.95</v>
+        <v>47.9</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>730</v>
+        <v>717</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2790,7 +2790,7 @@
         <v>59.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>79.5</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>2</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1370</v>
+        <v>1335</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>37.9</v>
+        <v>38.1</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.05</v>
+        <v>36.65</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.2</v>
+        <v>37.6</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50</v>
+        <v>50.2</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>40.9</v>
+        <v>39.5</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.3</v>
+        <v>40.85</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.45</v>
+        <v>16.25</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>73.5</v>
+        <v>72.3</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.45</v>
+        <v>10.4</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.6</v>
+        <v>44.55</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>84</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>126</v>
+        <v>126.5</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>160.5</v>
+        <v>164</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19.4</v>
+        <v>19.15</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>60.7</v>
+        <v>59.9</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.25</v>
+        <v>34.85</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.1</v>
+        <v>29.15</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>80.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>49.1</v>
+        <v>49.35</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>364.5</v>
+        <v>350</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>13905</v>
+        <v>12520</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>31.1</v>
+        <v>30.65</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>27.4</v>
+        <v>25.75</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.7</v>
+        <v>30.6</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>30.8</v>
+        <v>30.45</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>53.6</v>
+        <v>53.3</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.4</v>
+        <v>63.7</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83</v>
+        <v>83.2</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48.3</v>
+        <v>48</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.5</v>
+        <v>31.85</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1850</v>
+        <v>1805</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>32.3</v>
+        <v>31.3</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>256</v>
+        <v>251.5</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>40.05</v>
+        <v>39.05</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>589</v>
+        <v>567</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>43.3</v>
+        <v>42.7</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2460</v>
+        <v>2470</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>19.45</v>
+        <v>18.75</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>124.5</v>
+        <v>126</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>38.55</v>
+        <v>37.75</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2100</v>
+        <v>1955</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>89.3</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>233.5</v>
+        <v>227.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>29</v>
+        <v>28.65</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>32.3</v>
+        <v>31.05</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>65.7</v>
+        <v>64.5</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>42.2</v>
+        <v>41.9</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>66.09999999999999</v>
+        <v>64</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>999</v>
+        <v>968</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>142</v>
+        <v>135.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2230</v>
+        <v>2265</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>47.95</v>
+        <v>47.55</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>52.5</v>
+        <v>51.8</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>42.4</v>
+        <v>41.5</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1120</v>
+        <v>1075</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>28.15</v>
+        <v>27.8</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>364.5</v>
+        <v>357</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>158.5</v>
+        <v>152.5</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>729</v>
+        <v>692</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>347.5</v>
+        <v>328</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5495</v>
+        <v>5340</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>110.5</v>
+        <v>105.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>77.7</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>44.35</v>
+        <v>42.8</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>63.5</v>
+        <v>62.6</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>680</v>
+        <v>657</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.55</v>
+        <v>24.85</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>56.1</v>
+        <v>54.6</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1080</v>
+        <v>1055</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>517</v>
+        <v>531</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>28.7</v>
+        <v>29.6</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>171.5</v>
+        <v>168</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>99.09999999999999</v>
+        <v>97.5</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>259.5</v>
+        <v>253.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>76.90000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>118</v>
+        <v>114.5</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>273</v>
+        <v>268.5</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>289.5</v>
+        <v>286</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4760</v>
+        <v>4710</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>131</v>
+        <v>130.5</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>203</v>
+        <v>194.5</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>100.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>226</v>
+        <v>215.5</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>208.5</v>
+        <v>205</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>122</v>
+        <v>119.5</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>157.5</v>
+        <v>155.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>158</v>
+        <v>152.5</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>254.5</v>
+        <v>245.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>40.9</v>
+        <v>39.15</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>323</v>
+        <v>318.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>184</v>
+        <v>179.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>41</v>
+        <v>40.2</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.3</v>
+        <v>31.6</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.6</v>
+        <v>36.8</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.75</v>
+        <v>19.85</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>89.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.15</v>
+        <v>35.25</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>46.9</v>
+        <v>48.2</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>48</v>
+        <v>47.7</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>38.65</v>
+        <v>39.05</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.5</v>
+        <v>34.8</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>94.2</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>36.35</v>
+        <v>36.5</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>78.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>58.1</v>
+        <v>57.3</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.45</v>
+        <v>20.6</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>114.5</v>
+        <v>112</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.1</v>
+        <v>42.45</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>66.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>99.2</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>174</v>
+        <v>172.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.6</v>
+        <v>45.55</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.25</v>
+        <v>22.45</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>17.9</v>
+        <v>18.25</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>56.7</v>
+        <v>57.4</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>27.1</v>
+        <v>26.7</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>113</v>
+        <v>112.5</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>297</v>
+        <v>298.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6660</v>
+        <v>6500</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>129.5</v>
+        <v>127</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>86.3</v>
+        <v>83.8</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>100.5</v>
+        <v>101.5</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3420</v>
+        <v>3285</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>142</v>
+        <v>138.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>91.5</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>339.5</v>
+        <v>323</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>771</v>
+        <v>747</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>63.4</v>
+        <v>62.3</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>109.5</v>
+        <v>111.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>43.25</v>
+        <v>43.3</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>192.5</v>
+        <v>189.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>176.5</v>
+        <v>172</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>493</v>
+        <v>484</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>3070</v>
+        <v>2865</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>171.5</v>
+        <v>167.5</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>450.5</v>
+        <v>441.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2555</v>
+        <v>2635</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>60.8</v>
+        <v>60.2</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>752</v>
+        <v>726</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>883</v>
+        <v>938</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>813</v>
+        <v>800</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>384</v>
+        <v>375.5</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>136</v>
+        <v>133.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>190.5</v>
+        <v>186.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>197</v>
+        <v>186.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>199.5</v>
+        <v>197</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>176</v>
+        <v>166.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>140.5</v>
+        <v>138</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>109.5</v>
+        <v>103.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1440</v>
+        <v>1340</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>213.5</v>
+        <v>206.5</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>190</v>
+        <v>187.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>723</v>
+        <v>711</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>469.5</v>
+        <v>475</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>206.5</v>
+        <v>203.5</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>29.85</v>
+        <v>29.9</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>987</v>
+        <v>1010</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>284</v>
+        <v>281.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>169.5</v>
+        <v>160.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5935</v>
+        <v>5960</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>585</v>
+        <v>527</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>49.95</v>
+        <v>48.8</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1510</v>
+        <v>1490</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>231</v>
+        <v>221.5</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2570</v>
+        <v>2825</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1695</v>
+        <v>1620</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>17.05</v>
+        <v>16.9</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>722</v>
+        <v>740</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>252.5</v>
+        <v>246</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>221.5</v>
+        <v>218.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>159.5</v>
+        <v>155.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>248.5</v>
+        <v>245</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5655</v>
+        <v>5550</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4040</v>
+        <v>4030</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2070</v>
+        <v>1935</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>65.8</v>
+        <v>63.9</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>682</v>
+        <v>669</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>105</v>
+        <v>104.5</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.75</v>
+        <v>19.85</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>39.7</v>
+        <v>38.9</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56.4</v>
+        <v>56.1</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>92.59999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>61.2</v>
+        <v>60</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>67.2</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>119.5</v>
+        <v>126.5</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>76.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.65</v>
+        <v>29.6</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>29.55</v>
+        <v>30.4</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>62.7</v>
+        <v>65.3</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>122.5</v>
+        <v>122</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>163</v>
+        <v>162.5</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>167.5</v>
+        <v>163</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>247</v>
+        <v>235.5</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>297.5</v>
+        <v>297</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>394</v>
+        <v>392.5</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>45.6</v>
+        <v>46.95</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>50.6</v>
+        <v>49.15</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>228</v>
+        <v>218.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>344.5</v>
+        <v>346</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>250.5</v>
+        <v>249.5</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.8</v>
+        <v>36.1</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>60.2</v>
+        <v>60.5</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>122.5</v>
+        <v>118</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>247.5</v>
+        <v>241.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>93.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>165.5</v>
+        <v>177.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>566</v>
+        <v>547</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>277.5</v>
+        <v>280.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>590</v>
+        <v>605</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>32.75</v>
+        <v>32.8</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>20.85</v>
+        <v>21.15</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>95.40000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1440</v>
+        <v>1400</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>19215</v>
+        <v>19220</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>318.5</v>
+        <v>309.5</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1405</v>
+        <v>1370</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>35.2</v>
+        <v>38.7</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>81.2</v>
+        <v>82.5</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>118.5</v>
+        <v>117</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>75.3</v>
+        <v>73.5</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>92.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>541</v>
+        <v>532</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>262.5</v>
+        <v>257.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>120</v>
+        <v>114.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>72.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>97.90000000000001</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>183.5</v>
+        <v>180</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.3</v>
+        <v>63.6</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>49.45</v>
+        <v>49.4</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>874</v>
+        <v>851</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>55.2</v>
+        <v>54.9</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>112.5</v>
+        <v>115</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>386.5</v>
+        <v>378.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>50.8</v>
+        <v>50.1</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>191</v>
+        <v>186.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>116</v>
+        <v>114.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>286.5</v>
+        <v>273.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.4</v>
+        <v>47.75</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>111.5</v>
+        <v>109</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1370</v>
+        <v>1385</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>65.5</v>
+        <v>65</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>67.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>82.8</v>
+        <v>81.7</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>514</v>
+        <v>503</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>308</v>
+        <v>300.5</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>59</v>
+        <v>56.9</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>181.5</v>
+        <v>178</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5490</v>
+        <v>5795</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>280</v>
+        <v>275.5</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>67.8</v>
+        <v>65.8</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>232.5</v>
+        <v>223</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1370</v>
+        <v>1345</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>195</v>
+        <v>188.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>44.35</v>
+        <v>43.25</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>79.90000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>239.5</v>
+        <v>236</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>269.5</v>
+        <v>264.5</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>442.5</v>
+        <v>463.5</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>977</v>
+        <v>958</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>77</v>
+        <v>74.7</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>389.5</v>
+        <v>376</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1700</v>
+        <v>1695</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1325</v>
+        <v>1405</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>231.5</v>
+        <v>225</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>448.5</v>
+        <v>435</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>68.8</v>
+        <v>66.8</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>416</v>
+        <v>412.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>971</v>
+        <v>955</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>379.5</v>
+        <v>376</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>79.7</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3470</v>
+        <v>3620</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7000</v>
+        <v>7700</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>133.5</v>
+        <v>130.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>960</v>
+        <v>931</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>78.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>63.4</v>
+        <v>64</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>73.59999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>152</v>
+        <v>147.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.6</v>
+        <v>60.3</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>137.5</v>
+        <v>135.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>265</v>
+        <v>258.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1300</v>
+        <v>1215</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>411</v>
+        <v>438</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2490</v>
+        <v>2340</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>299.5</v>
+        <v>294</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1410</v>
+        <v>1405</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>190</v>
+        <v>183.5</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1110</v>
+        <v>1145</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>137.5</v>
+        <v>134.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>63.8</v>
+        <v>63.7</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>72.90000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1080</v>
+        <v>1065</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>271.5</v>
+        <v>271</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2265</v>
+        <v>2155</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>14.95</v>
+        <v>15.25</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>85.2</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>286.5</v>
+        <v>287.5</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>719</v>
+        <v>706</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>67.09999999999999</v>
+        <v>60.4</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.8</v>
+        <v>31.25</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>2000</v>
+        <v>2065</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>660</v>
+        <v>594</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>279</v>
+        <v>272.5</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2915</v>
+        <v>2910</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>561</v>
+        <v>523</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2375</v>
+        <v>2315</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1590</v>
+        <v>1545</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>283</v>
+        <v>275.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6565</v>
+        <v>6970</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.65</v>
+        <v>16.55</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>115.5</v>
+        <v>115</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>316.5</v>
+        <v>291.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>395</v>
+        <v>382.5</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>930</v>
+        <v>899</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>1870</v>
+        <v>2035</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>291.5</v>
+        <v>278</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>462</v>
+        <v>450</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>185.5</v>
+        <v>177</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>249.5</v>
+        <v>236.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>177</v>
+        <v>174.5</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>327</v>
+        <v>294.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1050</v>
+        <v>1025</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>122.5</v>
+        <v>134.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>150.5</v>
+        <v>147</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>49.9</v>
+        <v>50</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>253</v>
+        <v>248.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>112.5</v>
+        <v>110</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>216.5</v>
+        <v>213.5</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>43.85</v>
+        <v>43.75</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>90.40000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>189.5</v>
+        <v>180</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>91.3</v>
+        <v>90.3</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>347</v>
+        <v>341.5</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>937</v>
+        <v>907</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>143</v>
+        <v>139.5</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>181</v>
+        <v>170.5</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>222</v>
+        <v>219.5</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2095</v>
+        <v>2085</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.2</v>
+        <v>37.05</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.05</v>
+        <v>26.6</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>242</v>
+        <v>239.5</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>361</v>
+        <v>371.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>142.5</v>
+        <v>141.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57.9</v>
+        <v>57.2</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>94.2</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1240</v>
+        <v>1225</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>72</v>
+        <v>71.2</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.6</v>
+        <v>24.7</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.3</v>
+        <v>15.25</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>69.8</v>
+        <v>71.8</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>77.8</v>
+        <v>77</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>97.3</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.55</v>
+        <v>39.6</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>63.1</v>
+        <v>62.7</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.3</v>
+        <v>39.1</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.7</v>
+        <v>55.2</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>129</v>
+        <v>128.5</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>80.5</v>
+        <v>81</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>27.9</v>
+        <v>28.05</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>91.59999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-09
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.3</v>
+        <v>24.75</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.2</v>
+        <v>35.4</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>110</v>
+        <v>110.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>76.7</v>
+        <v>76</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.7</v>
+        <v>41.95</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.40000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>157</v>
+        <v>156.5</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>235</v>
+        <v>236.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.35</v>
+        <v>12.8</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.8</v>
+        <v>12.15</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.109999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>79</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.65</v>
+        <v>28.7</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>24.45</v>
+        <v>26.85</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>67.5</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>17.8</v>
+        <v>18.15</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.6</v>
+        <v>13.75</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>300</v>
+        <v>295.5</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>198</v>
+        <v>197.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>204.5</v>
+        <v>206</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102</v>
+        <v>103.5</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>47.9</v>
+        <v>48</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>717</v>
+        <v>730</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2790,7 +2790,7 @@
         <v>59.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>2</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1335</v>
+        <v>1330</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.1</v>
+        <v>38.35</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.65</v>
+        <v>37</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.6</v>
+        <v>38.1</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>39.5</v>
+        <v>39.85</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.25</v>
+        <v>16.8</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.4</v>
+        <v>10.85</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.55</v>
+        <v>44.2</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>83.90000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>126.5</v>
+        <v>126</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>164</v>
+        <v>164.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>100</v>
+        <v>101.5</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>180.5</v>
+        <v>179</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>59.9</v>
+        <v>60.2</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.85</v>
+        <v>35.1</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>24.45</v>
+        <v>24.55</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.2</v>
+        <v>13.45</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.15</v>
+        <v>29.2</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.1</v>
+        <v>19.25</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>81.90000000000001</v>
+        <v>82</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.4</v>
+        <v>22.55</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17</v>
+        <v>17.05</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>13.95</v>
+        <v>14</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>49.35</v>
+        <v>48.6</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>350</v>
+        <v>370.5</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>12520</v>
+        <v>12400</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>30.65</v>
+        <v>30.85</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>25.75</v>
+        <v>26.5</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.6</v>
+        <v>30.8</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>16.95</v>
+        <v>17.05</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>30.45</v>
+        <v>30.5</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>53.3</v>
+        <v>53.4</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>63.7</v>
+        <v>64.2</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.2</v>
+        <v>84</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>48</v>
+        <v>47.85</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>233</v>
+        <v>232.5</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.85</v>
+        <v>31.8</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>291</v>
+        <v>292.5</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>137</v>
+        <v>141.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1805</v>
+        <v>1795</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.3</v>
+        <v>31.8</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>251.5</v>
+        <v>252</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>39.05</v>
+        <v>38.9</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46</v>
+        <v>46.3</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>42.7</v>
+        <v>42.65</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2470</v>
+        <v>2465</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>18.75</v>
+        <v>19.15</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>126</v>
+        <v>126.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>37.75</v>
+        <v>41.5</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>1955</v>
+        <v>2015</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>88.90000000000001</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>227.5</v>
+        <v>237.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.65</v>
+        <v>28.8</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.05</v>
+        <v>31.8</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>41.9</v>
+        <v>42.65</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>64</v>
+        <v>64.3</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>968</v>
+        <v>979</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>135.5</v>
+        <v>133.5</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2265</v>
+        <v>2335</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>47.55</v>
+        <v>48.3</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>51.8</v>
+        <v>52.6</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>41.5</v>
+        <v>42.2</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>27.8</v>
+        <v>28.05</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>357</v>
+        <v>349.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>152.5</v>
+        <v>156.5</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>692</v>
+        <v>705</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5340</v>
+        <v>5375</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>105.5</v>
+        <v>106.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>76.09999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>62.6</v>
+        <v>62.7</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>24.85</v>
+        <v>25.15</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1055</v>
+        <v>1065</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>29.6</v>
+        <v>30.5</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>139</v>
+        <v>139.5</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>168</v>
+        <v>167.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>97.5</v>
+        <v>99.5</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>253.5</v>
+        <v>248.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>76.09999999999999</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>268.5</v>
+        <v>270</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>286</v>
+        <v>287.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4710</v>
+        <v>4625</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>515</v>
+        <v>533</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>130.5</v>
+        <v>130</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>194.5</v>
+        <v>197.5</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>98.59999999999999</v>
+        <v>103.5</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>610</v>
+        <v>581</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>215.5</v>
+        <v>215</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>119.5</v>
+        <v>120</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>121</v>
+        <v>122.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>152.5</v>
+        <v>152</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>245.5</v>
+        <v>249.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>39.15</v>
+        <v>39.45</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>318.5</v>
+        <v>319.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>179.5</v>
+        <v>180</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.2</v>
+        <v>40.5</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.6</v>
+        <v>31.55</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>11.9</v>
+        <v>12.05</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.85</v>
+        <v>19.8</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>89.09999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.25</v>
+        <v>35.75</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>48.2</v>
+        <v>49.1</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>47.7</v>
+        <v>48.2</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>39.05</v>
+        <v>39.4</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.8</v>
+        <v>34.6</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>94.59999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>36.5</v>
+        <v>36.95</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>77.8</v>
+        <v>79.7</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.2</v>
+        <v>53.5</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>57.3</v>
+        <v>58.5</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.6</v>
+        <v>20.45</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.45</v>
+        <v>42.55</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>65.90000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>98.09999999999999</v>
+        <v>100.5</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>172.5</v>
+        <v>174.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.6</v>
+        <v>20.55</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>45.55</v>
+        <v>46.3</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.45</v>
+        <v>22.4</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>18.25</v>
+        <v>18.05</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>217</v>
+        <v>217.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>26.7</v>
+        <v>27.8</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>112.5</v>
+        <v>115</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>298.5</v>
+        <v>306.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6500</v>
+        <v>6870</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>83.8</v>
+        <v>87</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>101.5</v>
+        <v>100</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3285</v>
+        <v>3380</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>138.5</v>
+        <v>142.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>86.40000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>62.3</v>
+        <v>62</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>111.5</v>
+        <v>111</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>43.3</v>
+        <v>41.85</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>534</v>
+        <v>543</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>175</v>
+        <v>176.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>189.5</v>
+        <v>191.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>954</v>
+        <v>993</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>172</v>
+        <v>184.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>484</v>
+        <v>509</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>118</v>
+        <v>119.5</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>2865</v>
+        <v>2850</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>121</v>
+        <v>126.5</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>167.5</v>
+        <v>166</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>441.5</v>
+        <v>464</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2635</v>
+        <v>2555</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>60.2</v>
+        <v>62.5</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>938</v>
+        <v>900</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>800</v>
+        <v>812</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>375.5</v>
+        <v>367</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>133.5</v>
+        <v>128.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>186.5</v>
+        <v>185.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>186.5</v>
+        <v>189</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>414</v>
+        <v>414.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>166.5</v>
+        <v>167.5</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>103.5</v>
+        <v>104.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1340</v>
+        <v>1385</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>206.5</v>
+        <v>208</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>187.5</v>
+        <v>189.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>475</v>
+        <v>478.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>203.5</v>
+        <v>206</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>29.9</v>
+        <v>30.4</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1010</v>
+        <v>1110</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>281.5</v>
+        <v>282</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5960</v>
+        <v>5925</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>48.8</v>
+        <v>50.1</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1490</v>
+        <v>1455</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>221.5</v>
+        <v>225.5</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2825</v>
+        <v>2780</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>398</v>
+        <v>424</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1620</v>
+        <v>1625</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>16.9</v>
+        <v>16.95</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>740</v>
+        <v>730</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>218.5</v>
+        <v>222</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>155.5</v>
+        <v>157.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5550</v>
+        <v>5760</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4030</v>
+        <v>3905</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>1935</v>
+        <v>1975</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>63.9</v>
+        <v>64.2</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>274</v>
+        <v>271.5</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>521</v>
+        <v>566</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>669</v>
+        <v>700</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>104.5</v>
+        <v>105</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.85</v>
+        <v>19.95</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>38.9</v>
+        <v>39.4</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56.1</v>
+        <v>56.3</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>91.3</v>
+        <v>81.8</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>60</v>
+        <v>60.1</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>618</v>
+        <v>640</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>64.90000000000001</v>
+        <v>63.7</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>126.5</v>
+        <v>135</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>76.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.6</v>
+        <v>29.95</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.4</v>
+        <v>30.55</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>65.3</v>
+        <v>62.8</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>122</v>
+        <v>121.5</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>162.5</v>
+        <v>166</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>235.5</v>
+        <v>244</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>28.3</v>
+        <v>27.2</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>392.5</v>
+        <v>0</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>46.95</v>
+        <v>45.8</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>49.15</v>
+        <v>48.3</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>218.5</v>
+        <v>226.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>346</v>
+        <v>340.5</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>234</v>
+        <v>249.5</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>249.5</v>
+        <v>246</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.1</v>
+        <v>36.6</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>60.5</v>
+        <v>61.4</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>241.5</v>
+        <v>252.5</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>91.7</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>177.5</v>
+        <v>177</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>280.5</v>
+        <v>281.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>605</v>
+        <v>621</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>32.8</v>
+        <v>32.55</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.15</v>
+        <v>21.05</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>296</v>
+        <v>296.5</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>91.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1400</v>
+        <v>1395</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>19220</v>
+        <v>18605</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>309.5</v>
+        <v>314</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1370</v>
+        <v>1355</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>38.7</v>
+        <v>42.55</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>82.5</v>
+        <v>84.8</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>73.5</v>
+        <v>73</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>89.59999999999999</v>
+        <v>90</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>257.5</v>
+        <v>264.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>114.5</v>
+        <v>111.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>71.09999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.6</v>
+        <v>63.5</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>49.4</v>
+        <v>49</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.90000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>851</v>
+        <v>862</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>54.9</v>
+        <v>55.8</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>185</v>
+        <v>184.5</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>71.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.3</v>
+        <v>14.65</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>378.5</v>
+        <v>383</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>276</v>
+        <v>272.5</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>186.5</v>
+        <v>198</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>114.5</v>
+        <v>115.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>273.5</v>
+        <v>268.5</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>91.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>47.75</v>
+        <v>48.45</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>109</v>
+        <v>110.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1385</v>
+        <v>1330</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>65</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>81.7</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>503</v>
+        <v>534</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>300.5</v>
+        <v>302.5</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>56.9</v>
+        <v>57.2</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>134</v>
+        <v>137.5</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>510</v>
+        <v>523</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>185</v>
+        <v>187.5</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5795</v>
+        <v>5615</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>275.5</v>
+        <v>281</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>65.8</v>
+        <v>69.3</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>223</v>
+        <v>226.5</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>188.5</v>
+        <v>193.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>43.25</v>
+        <v>43.7</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>236</v>
+        <v>233.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>264.5</v>
+        <v>275</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>463.5</v>
+        <v>480</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>958</v>
+        <v>926</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>376</v>
+        <v>378.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1695</v>
+        <v>1700</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>24</v>
+        <v>23.95</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1405</v>
+        <v>1345</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>66.8</v>
+        <v>67.5</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>412.5</v>
+        <v>407.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>79.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3620</v>
+        <v>3610</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7700</v>
+        <v>7280</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>931</v>
+        <v>999</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>77.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>64</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>320</v>
+        <v>317.5</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>147.5</v>
+        <v>149</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>602</v>
+        <v>586</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.3</v>
+        <v>60.5</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>135.5</v>
+        <v>136</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>258.5</v>
+        <v>264.5</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1215</v>
+        <v>1200</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>356.5</v>
+        <v>353.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2340</v>
+        <v>2325</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>279</v>
+        <v>279.5</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>294</v>
+        <v>299.5</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1405</v>
+        <v>1370</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>325</v>
+        <v>354.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>183.5</v>
+        <v>182.5</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1145</v>
+        <v>1200</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>134.5</v>
+        <v>135</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>55.4</v>
+        <v>54.9</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>63.7</v>
+        <v>63.4</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>463</v>
+        <v>475.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2155</v>
+        <v>2295</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>560</v>
+        <v>575</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>15.25</v>
+        <v>15.1</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>81.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>287.5</v>
+        <v>291</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>706</v>
+        <v>715</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>60.4</v>
+        <v>54.9</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.25</v>
+        <v>31.1</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>2065</v>
+        <v>2030</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>594</v>
+        <v>610</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>272.5</v>
+        <v>272</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2910</v>
+        <v>2980</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>355</v>
+        <v>355.5</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2315</v>
+        <v>2270</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1545</v>
+        <v>1610</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>275.5</v>
+        <v>276.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6970</v>
+        <v>6720</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.55</v>
+        <v>16.65</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>115</v>
+        <v>115.5</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>291.5</v>
+        <v>320.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>382.5</v>
+        <v>386.5</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>151</v>
+        <v>151.5</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>2035</v>
+        <v>2080</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>450</v>
+        <v>442.5</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>236.5</v>
+        <v>236</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>294.5</v>
+        <v>289.5</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1025</v>
+        <v>1110</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>134.5</v>
+        <v>134</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>147</v>
+        <v>149.5</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>50</v>
+        <v>49.85</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>248.5</v>
+        <v>251</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>110</v>
+        <v>113.5</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>213.5</v>
+        <v>212</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>101</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>43.75</v>
+        <v>43.3</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>89.5</v>
+        <v>86.5</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>61.9</v>
+        <v>63.5</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.3</v>
+        <v>91.5</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>341.5</v>
+        <v>348</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>907</v>
+        <v>916</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>139.5</v>
+        <v>138.5</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>219.5</v>
+        <v>217.5</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>37.05</v>
+        <v>36.7</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.6</v>
+        <v>26.25</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>239.5</v>
+        <v>238.5</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>371.5</v>
+        <v>375</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>141.5</v>
+        <v>141</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>57.2</v>
+        <v>59.3</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>92.40000000000001</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1225</v>
+        <v>1345</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.7</v>
+        <v>24.55</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.25</v>
+        <v>15.35</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.1</v>
+        <v>29.05</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>71.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>81.7</v>
+        <v>82</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>77</v>
+        <v>79.2</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33853,7 +33853,7 @@
         <v>15.67</v>
       </c>
       <c r="Q492" s="3" t="n">
-        <v>106.5</v>
+        <v>106</v>
       </c>
       <c r="R492" s="3" t="n">
         <v>5.7</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>95.59999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.6</v>
+        <v>39.75</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>62.7</v>
+        <v>62.6</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>39.1</v>
+        <v>40.15</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.2</v>
+        <v>55.7</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>128.5</v>
+        <v>127.5</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34334,7 +34334,7 @@
         <v>12.04</v>
       </c>
       <c r="Q499" s="3" t="n">
-        <v>81</v>
+        <v>80.3</v>
       </c>
       <c r="R499" s="3" t="n">
         <v>4.38</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.05</v>
+        <v>28.2</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>90.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-10
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.75</v>
+        <v>24.8</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.4</v>
+        <v>35.45</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.45</v>
+        <v>27.25</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.5</v>
+        <v>52.3</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>110.5</v>
+        <v>111</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>76</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.55</v>
+        <v>28.35</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.95</v>
+        <v>41.75</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.5</v>
+        <v>80.2</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>66.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>236.5</v>
+        <v>244</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.8</v>
+        <v>12.45</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>12.15</v>
+        <v>11.85</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.210000000000001</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>79.59999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>71.8</v>
+        <v>71.3</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n">
-        <v>28.7</v>
+        <v>28.65</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>1.25</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>26.85</v>
+        <v>25.15</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>67.90000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18.15</v>
+        <v>18</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.75</v>
+        <v>13.5</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>295.5</v>
+        <v>290</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>167</v>
+        <v>165.5</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>103.5</v>
+        <v>102</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>735</v>
+        <v>718</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>48</v>
+        <v>47.8</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1330</v>
+        <v>1305</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>38.35</v>
+        <v>37.8</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>37</v>
+        <v>36.45</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>38.1</v>
+        <v>37.75</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>50.2</v>
+        <v>49.4</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>39.85</v>
+        <v>39.05</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.85</v>
+        <v>40.8</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.8</v>
+        <v>16.5</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>72.3</v>
+        <v>71.7</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.85</v>
+        <v>10.6</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>44.2</v>
+        <v>43.75</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>83.59999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>164.5</v>
+        <v>161.5</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>101.5</v>
+        <v>98.3</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>19.15</v>
+        <v>18.6</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>60.2</v>
+        <v>59.6</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>35.1</v>
+        <v>34.4</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>24.55</v>
+        <v>25.55</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.45</v>
+        <v>13.3</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.2</v>
+        <v>29.15</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.25</v>
+        <v>19.1</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>82</v>
+        <v>81.2</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.55</v>
+        <v>22.4</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>17.05</v>
+        <v>16.9</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>48.6</v>
+        <v>48.2</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>370.5</v>
+        <v>363</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>12400</v>
+        <v>12600</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>133</v>
+        <v>130.5</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>30.85</v>
+        <v>30.4</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>26.5</v>
+        <v>25.85</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.8</v>
+        <v>30.6</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>17.05</v>
+        <v>16.85</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>30.5</v>
+        <v>30.2</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>53.4</v>
+        <v>53.1</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>18.9</v>
+        <v>18.7</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>84</v>
+        <v>83.5</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.85</v>
+        <v>47.05</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5871,7 +5871,7 @@
         <v>16.2</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>232.5</v>
+        <v>230</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>14.5</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.8</v>
+        <v>31.1</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>292.5</v>
+        <v>291</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>141.5</v>
+        <v>142.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1795</v>
+        <v>1675</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.8</v>
+        <v>31.15</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>228</v>
+        <v>225.5</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>38.9</v>
+        <v>38.65</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.3</v>
+        <v>46.1</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>42.65</v>
+        <v>42.2</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2465</v>
+        <v>2450</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>19.15</v>
+        <v>18.85</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>126.5</v>
+        <v>122.5</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>41.5</v>
+        <v>45.65</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>183</v>
+        <v>179.5</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>2015</v>
+        <v>1965</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>88.59999999999999</v>
+        <v>88.8</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>237.5</v>
+        <v>235.5</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.8</v>
+        <v>31.5</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>64.5</v>
+        <v>65</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>42.65</v>
+        <v>41.85</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>64.3</v>
+        <v>62.6</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>979</v>
+        <v>989</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>133.5</v>
+        <v>130</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2335</v>
+        <v>2180</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>48.3</v>
+        <v>47.6</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>42.2</v>
+        <v>41.15</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1100</v>
+        <v>1045</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>28.05</v>
+        <v>27.85</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8185,7 +8185,7 @@
         <v>20.71</v>
       </c>
       <c r="Q112" s="3" t="n">
-        <v>67.7</v>
+        <v>67.3</v>
       </c>
       <c r="R112" s="3" t="n">
         <v>1.99</v>
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>349.5</v>
+        <v>351.5</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8386,7 +8386,7 @@
         <v>12.14</v>
       </c>
       <c r="Q115" s="3" t="n">
-        <v>156.5</v>
+        <v>149</v>
       </c>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3">
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>705</v>
+        <v>696</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>106.5</v>
+        <v>103.5</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>42.8</v>
+        <v>43.4</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>62.7</v>
+        <v>61.8</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>25.15</v>
+        <v>24.9</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>54.6</v>
+        <v>54.2</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1065</v>
+        <v>1060</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>30.5</v>
+        <v>31.2</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>167.5</v>
+        <v>165</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>99.5</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>248.5</v>
+        <v>250.5</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>74.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>114.5</v>
+        <v>115</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>270</v>
+        <v>271.5</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>287.5</v>
+        <v>282.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4625</v>
+        <v>4720</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>197.5</v>
+        <v>193.5</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>103.5</v>
+        <v>101.5</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10375,7 +10375,7 @@
         <v>13.61</v>
       </c>
       <c r="Q144" s="3" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="R144" s="3" t="n">
         <v>7.11</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>122.5</v>
+        <v>124</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>155.5</v>
+        <v>156.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>152</v>
+        <v>154.5</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>249.5</v>
+        <v>242</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>39.45</v>
+        <v>38.6</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>319.5</v>
+        <v>334</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>180</v>
+        <v>174.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.5</v>
+        <v>40.15</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.4</v>
+        <v>22.25</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.55</v>
+        <v>31.45</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11163,7 +11163,7 @@
         <v>25</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>12.05</v>
+        <v>12</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.9</v>
+        <v>36.75</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.8</v>
+        <v>19.55</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>88.7</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.75</v>
+        <v>35.35</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>49.1</v>
+        <v>49.45</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11553,7 +11553,7 @@
         <v>10.69</v>
       </c>
       <c r="Q162" s="3" t="n">
-        <v>48.2</v>
+        <v>46.5</v>
       </c>
       <c r="R162" s="3" t="n">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>39.4</v>
+        <v>39.1</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.6</v>
+        <v>34.4</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>95.59999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>36.95</v>
+        <v>36.25</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>79.7</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53.5</v>
+        <v>53</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>58.5</v>
+        <v>58</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.45</v>
+        <v>20.2</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>116</v>
+        <v>110.5</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>42.55</v>
+        <v>41.8</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12485,7 +12485,7 @@
         <v>33.48</v>
       </c>
       <c r="Q176" s="3" t="n">
-        <v>65.3</v>
+        <v>63.8</v>
       </c>
       <c r="R176" s="3" t="n">
         <v>0.78</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>174.5</v>
+        <v>172.5</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.55</v>
+        <v>20.3</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>46.3</v>
+        <v>46</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12826,7 +12826,7 @@
         <v>12.67</v>
       </c>
       <c r="Q181" s="3" t="n">
-        <v>178</v>
+        <v>177.5</v>
       </c>
       <c r="R181" s="3" t="n">
         <v>10.75</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>229</v>
+        <v>229.5</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>18.05</v>
+        <v>18.35</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>217.5</v>
+        <v>218.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>57.4</v>
+        <v>56.9</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>27.8</v>
+        <v>27.3</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>306.5</v>
+        <v>312</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6870</v>
+        <v>6720</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="P191" s="3" t="n"/>
       <c r="Q191" s="3" t="n">
-        <v>125</v>
+        <v>124.5</v>
       </c>
       <c r="R191" s="3" t="n">
         <v>5.3</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>87</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131</v>
+        <v>131.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3380</v>
+        <v>3460</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>142.5</v>
+        <v>139</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>85.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>758</v>
+        <v>803</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>62</v>
+        <v>62.3</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>271</v>
+        <v>266.5</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>41.85</v>
+        <v>42.05</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>176.5</v>
+        <v>179</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>191.5</v>
+        <v>192.5</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>184.5</v>
+        <v>180.5</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>119.5</v>
+        <v>120</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>2850</v>
+        <v>2830</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>126.5</v>
+        <v>126</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>464</v>
+        <v>461.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2555</v>
+        <v>2460</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>62.5</v>
+        <v>61.4</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>724</v>
+        <v>707</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>900</v>
+        <v>848</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>812</v>
+        <v>827</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>128.5</v>
+        <v>127.5</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>185.5</v>
+        <v>183.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>414.5</v>
+        <v>407</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>167.5</v>
+        <v>171</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>104.5</v>
+        <v>101.5</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1385</v>
+        <v>1440</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>189.5</v>
+        <v>182.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>478.5</v>
+        <v>488</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>206</v>
+        <v>189.5</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>30.4</v>
+        <v>30.65</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1110</v>
+        <v>1070</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>282</v>
+        <v>283.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>160.5</v>
+        <v>161</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>5925</v>
+        <v>6225</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>50.1</v>
+        <v>49.35</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1455</v>
+        <v>1355</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>225.5</v>
+        <v>221.5</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2780</v>
+        <v>2730</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>424</v>
+        <v>410</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1625</v>
+        <v>1575</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>688</v>
+        <v>668</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>16.95</v>
+        <v>16.65</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>730</v>
+        <v>713</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>222</v>
+        <v>221.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>157.5</v>
+        <v>154.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5760</v>
+        <v>5790</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>3905</v>
+        <v>4055</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>1975</v>
+        <v>1930</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>64.2</v>
+        <v>62.6</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>271.5</v>
+        <v>269</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>700</v>
+        <v>691</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.95</v>
+        <v>19.9</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56.3</v>
+        <v>56</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>81.8</v>
+        <v>82</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>60.1</v>
+        <v>61.8</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>640</v>
+        <v>650</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>63.7</v>
+        <v>62</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.2</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.95</v>
+        <v>29.75</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.55</v>
+        <v>30.35</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>62.8</v>
+        <v>61.6</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>121.5</v>
+        <v>121</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>166</v>
+        <v>164.5</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>455</v>
+        <v>442</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>292</v>
+        <v>290.5</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>27.2</v>
+        <v>26.75</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>0</v>
+        <v>391</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>45.8</v>
+        <v>45.55</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>770</v>
+        <v>757</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>48.3</v>
+        <v>48.35</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>226.5</v>
+        <v>220.5</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>340.5</v>
+        <v>339</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>249.5</v>
+        <v>239</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>104</v>
+        <v>104.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.6</v>
+        <v>36.35</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>61.4</v>
+        <v>62.1</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>119</v>
+        <v>116.5</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>252.5</v>
+        <v>244</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -20939,7 +20939,7 @@
         <v>15.99</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>91.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>4.01</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>502</v>
+        <v>494.5</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>177</v>
+        <v>172.5</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>281.5</v>
+        <v>276.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>621</v>
+        <v>600</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>610</v>
+        <v>571</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>499</v>
+        <v>488</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56.6</v>
+        <v>56.2</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>21.05</v>
+        <v>20.85</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>296.5</v>
+        <v>290</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>92.2</v>
+        <v>90.2</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1395</v>
+        <v>1360</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>18605</v>
+        <v>18700</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1355</v>
+        <v>1290</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>42.55</v>
+        <v>46.8</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>84.8</v>
+        <v>85.7</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>157</v>
+        <v>161.5</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>118</v>
+        <v>115.5</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>73</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>90</v>
+        <v>89.3</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22549,7 +22549,7 @@
         <v>19.69</v>
       </c>
       <c r="Q324" s="3" t="n">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="R324" s="3" t="n">
         <v>13.42</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>264.5</v>
+        <v>258</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>111.5</v>
+        <v>108</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>72.40000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>193</v>
+        <v>184.5</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>97.40000000000001</v>
+        <v>97</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>63.5</v>
+        <v>62.7</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>49</v>
+        <v>49.4</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>75.8</v>
+        <v>74.5</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>55.8</v>
+        <v>52.3</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>112</v>
+        <v>112.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>184.5</v>
+        <v>185</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>72.90000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.65</v>
+        <v>14.7</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>383</v>
+        <v>378.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>50</v>
+        <v>49.8</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>272.5</v>
+        <v>271.5</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>198</v>
+        <v>190.5</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24053,7 +24053,7 @@
         <v>22.62</v>
       </c>
       <c r="Q346" s="3" t="n">
-        <v>115.5</v>
+        <v>112.5</v>
       </c>
       <c r="R346" s="3" t="n">
         <v>1.2</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>268.5</v>
+        <v>295</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>90.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24260,7 +24260,7 @@
         <v>5.24</v>
       </c>
       <c r="Q349" s="3" t="n">
-        <v>48.45</v>
+        <v>47.5</v>
       </c>
       <c r="R349" s="3" t="n">
         <v>3</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>110.5</v>
+        <v>108.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1330</v>
+        <v>1280</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>69</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>83.09999999999999</v>
+        <v>82</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>302.5</v>
+        <v>301</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>57.2</v>
+        <v>56.6</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>137.5</v>
+        <v>135</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25145,7 +25145,7 @@
         <v>120.99</v>
       </c>
       <c r="Q362" s="3" t="n">
-        <v>5615</v>
+        <v>5620</v>
       </c>
       <c r="R362" s="3" t="n">
         <v>22</v>
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>281</v>
+        <v>283.5</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>69.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>226.5</v>
+        <v>227</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1345</v>
+        <v>1395</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>193.5</v>
+        <v>191.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>43.7</v>
+        <v>43.2</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>233.5</v>
+        <v>227</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>926</v>
+        <v>876</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26012,7 +26012,7 @@
         <v>12.85</v>
       </c>
       <c r="Q375" s="3" t="n">
-        <v>74.7</v>
+        <v>73.7</v>
       </c>
       <c r="R375" s="3" t="n">
         <v>3.7</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>378.5</v>
+        <v>372.5</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>23.95</v>
+        <v>23.65</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1345</v>
+        <v>1320</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>225.5</v>
+        <v>226.5</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>67.5</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>407.5</v>
+        <v>405.5</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>955</v>
+        <v>917</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>373</v>
+        <v>366.5</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>87.5</v>
+        <v>86.2</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3610</v>
+        <v>3670</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7280</v>
+        <v>7195</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>130.5</v>
+        <v>129.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>999</v>
+        <v>1030</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>81.90000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>68.09999999999999</v>
+        <v>61.4</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>71.7</v>
+        <v>70.8</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>149</v>
+        <v>148.5</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>586</v>
+        <v>554</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60.5</v>
+        <v>60</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>136</v>
+        <v>135.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>264.5</v>
+        <v>265</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1200</v>
+        <v>1210</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>433</v>
+        <v>423.5</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>353.5</v>
+        <v>346.5</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2325</v>
+        <v>2345</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>279.5</v>
+        <v>276</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>299.5</v>
+        <v>299</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28199,7 +28199,7 @@
         <v>61.16</v>
       </c>
       <c r="Q408" s="3" t="n">
-        <v>1370</v>
+        <v>1290</v>
       </c>
       <c r="R408" s="3" t="n">
         <v>9</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>158</v>
+        <v>156.5</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>354.5</v>
+        <v>336.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>182.5</v>
+        <v>184.5</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1200</v>
+        <v>1320</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>135</v>
+        <v>135.5</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28676,7 +28676,7 @@
       </c>
       <c r="P415" s="3" t="n"/>
       <c r="Q415" s="3" t="n">
-        <v>54.9</v>
+        <v>54.2</v>
       </c>
       <c r="R415" s="3" t="n"/>
       <c r="S415" s="3">
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>63.4</v>
+        <v>62.4</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>72.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1065</v>
+        <v>1030</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>475.5</v>
+        <v>469.5</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2295</v>
+        <v>2190</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>576</v>
+        <v>591</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>575</v>
+        <v>552</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>316</v>
+        <v>300.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>82.40000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>54.9</v>
+        <v>58.8</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>31.1</v>
+        <v>30.8</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>2030</v>
+        <v>2035</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>610</v>
+        <v>590</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>272</v>
+        <v>267.5</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2980</v>
+        <v>2810</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2270</v>
+        <v>2215</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1610</v>
+        <v>1500</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>276.5</v>
+        <v>271.5</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6720</v>
+        <v>6475</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.65</v>
+        <v>16.55</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>115.5</v>
+        <v>114.5</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>320.5</v>
+        <v>308</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>548</v>
+        <v>534</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>386.5</v>
+        <v>425</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>902</v>
+        <v>866</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>151.5</v>
+        <v>153</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>2080</v>
+        <v>2055</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>442.5</v>
+        <v>438</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>236</v>
+        <v>229.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>174.5</v>
+        <v>171.5</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>289.5</v>
+        <v>275</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1110</v>
+        <v>1070</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>134</v>
+        <v>126.5</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>149.5</v>
+        <v>147</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>49.85</v>
+        <v>49.45</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>251</v>
+        <v>247.5</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>113.5</v>
+        <v>109.5</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>99.90000000000001</v>
+        <v>91.8</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>43.3</v>
+        <v>42.75</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>86.5</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>180</v>
+        <v>178.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>63.5</v>
+        <v>62</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>91.5</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>916</v>
+        <v>910</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>138.5</v>
+        <v>137</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>170.5</v>
+        <v>168</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>217.5</v>
+        <v>211</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2085</v>
+        <v>2065</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>36.7</v>
+        <v>36.35</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.25</v>
+        <v>26.3</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>238.5</v>
+        <v>234</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>375</v>
+        <v>368.5</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>59.3</v>
+        <v>58.7</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>93.40000000000001</v>
+        <v>92.3</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1345</v>
+        <v>1300</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>71.2</v>
+        <v>66</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.55</v>
+        <v>24.1</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.35</v>
+        <v>15.3</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.59999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33715,7 +33715,7 @@
         <v>12.87</v>
       </c>
       <c r="Q490" s="3" t="n">
-        <v>82</v>
+        <v>81.8</v>
       </c>
       <c r="R490" s="3" t="n">
         <v>5</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>79.2</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33853,7 +33853,7 @@
         <v>15.67</v>
       </c>
       <c r="Q492" s="3" t="n">
-        <v>106</v>
+        <v>105.5</v>
       </c>
       <c r="R492" s="3" t="n">
         <v>5.7</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>98.5</v>
+        <v>97.3</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.75</v>
+        <v>39.7</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>62.6</v>
+        <v>62.2</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.15</v>
+        <v>40.35</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.7</v>
+        <v>55.6</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>127.5</v>
+        <v>128</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>28.2</v>
+        <v>27.75</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>91.7</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>

<commit_message>
Daily refresh: price/yield 2026-09-11
</commit_message>
<xml_diff>
--- a/taiwan_stocks_top500.xlsx
+++ b/taiwan_stocks_top500.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n">
-        <v>24.8</v>
+        <v>24.5</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -742,7 +742,7 @@
         <v>9.24</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>35.45</v>
+        <v>35.3</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>2.3</v>
@@ -811,7 +811,7 @@
         <v>9.94</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>27.25</v>
+        <v>27.2</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>1.85</v>
@@ -880,7 +880,7 @@
         <v>12.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>52.3</v>
+        <v>52.1</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>12.9</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>111</v>
+        <v>110.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>7</v>
@@ -1018,7 +1018,7 @@
         <v>18.31</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>3</v>
@@ -1087,7 +1087,7 @@
         <v>18.26</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>28.35</v>
+        <v>28.45</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>1.34</v>
@@ -1156,7 +1156,7 @@
         <v>16.39</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>41.75</v>
+        <v>40.7</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>1.8</v>
@@ -1225,7 +1225,7 @@
         <v>18.27</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>80.2</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>1.5</v>
@@ -1294,7 +1294,7 @@
         <v>17.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>156.5</v>
+        <v>156</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>7.2</v>
@@ -1363,7 +1363,7 @@
         <v>35.24</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.5</v>
@@ -1432,7 +1432,7 @@
         <v>30</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>244</v>
+        <v>234.5</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0.8</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="n">
-        <v>12.45</v>
+        <v>12.35</v>
       </c>
       <c r="R14" s="3" t="n"/>
       <c r="S14" s="3">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n">
-        <v>11.85</v>
+        <v>11.95</v>
       </c>
       <c r="R15" s="3" t="n"/>
       <c r="S15" s="3">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n">
-        <v>8.130000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="R16" s="3" t="n"/>
       <c r="S16" s="3">
@@ -1696,7 +1696,7 @@
         <v>13.47</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>78.40000000000001</v>
+        <v>79</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>5</v>
@@ -1765,7 +1765,7 @@
         <v>24.75</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>71.3</v>
+        <v>70.2</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0.6</v>
@@ -1901,7 +1901,7 @@
         <v>11.48</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>25.15</v>
+        <v>24.45</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0.9</v>
@@ -1970,7 +1970,7 @@
         <v>4.81</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>66.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>1.8</v>
@@ -2039,7 +2039,7 @@
         <v>19.02</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0.5</v>
@@ -2108,7 +2108,7 @@
         <v>466.67</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>0.3</v>
@@ -2177,7 +2177,7 @@
         <v>13.34</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>290</v>
+        <v>288.5</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>15</v>
@@ -2246,7 +2246,7 @@
         <v>14.88</v>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>197.5</v>
+        <v>196.5</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>15</v>
@@ -2315,7 +2315,7 @@
         <v>27.34</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>5</v>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="R27" s="3" t="n">
         <v>2</v>
@@ -2451,7 +2451,7 @@
         <v>18.67</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>165.5</v>
+        <v>165</v>
       </c>
       <c r="R28" s="3" t="n">
         <v>6</v>
@@ -2520,7 +2520,7 @@
         <v>28.08</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>102</v>
+        <v>100.5</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>46.47</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>718</v>
+        <v>712</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>11</v>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n">
-        <v>47.8</v>
+        <v>47.35</v>
       </c>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n">
-        <v>733</v>
+        <v>790</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>3.66</v>
@@ -2790,7 +2790,7 @@
         <v>59.91</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>78.2</v>
+        <v>76</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>2</v>
@@ -2859,7 +2859,7 @@
         <v>31.09</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>1305</v>
+        <v>1285</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>29.11</v>
@@ -2928,7 +2928,7 @@
         <v>11.3</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>37.8</v>
+        <v>37.4</v>
       </c>
       <c r="R35" s="3" t="n">
         <v>0.5</v>
@@ -2997,7 +2997,7 @@
         <v>3.11</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>36.45</v>
+        <v>36.2</v>
       </c>
       <c r="R36" s="3" t="n">
         <v>2</v>
@@ -3066,7 +3066,7 @@
         <v>13.67</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>37.75</v>
+        <v>37.85</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>0.7</v>
@@ -3135,7 +3135,7 @@
         <v>12.45</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>49.4</v>
+        <v>48.5</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>1.6</v>
@@ -3204,7 +3204,7 @@
         <v>308.46</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>39.05</v>
+        <v>38.45</v>
       </c>
       <c r="R39" s="3" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>14.68</v>
       </c>
       <c r="Q40" s="3" t="n">
-        <v>40.8</v>
+        <v>40.25</v>
       </c>
       <c r="R40" s="3" t="n">
         <v>2.5</v>
@@ -3342,7 +3342,7 @@
         <v>14.41</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>16.5</v>
+        <v>15.35</v>
       </c>
       <c r="R41" s="3" t="n">
         <v>0.18</v>
@@ -3411,7 +3411,7 @@
         <v>36.95</v>
       </c>
       <c r="Q42" s="3" t="n">
-        <v>71.7</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="R42" s="3" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>18.14</v>
       </c>
       <c r="Q43" s="3" t="n">
-        <v>10.6</v>
+        <v>10.4</v>
       </c>
       <c r="R43" s="3" t="n"/>
       <c r="S43" s="3">
@@ -3547,7 +3547,7 @@
         <v>55.06</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>43.75</v>
+        <v>43.25</v>
       </c>
       <c r="R44" s="3" t="n">
         <v>2</v>
@@ -3616,7 +3616,7 @@
         <v>28.39</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>82.3</v>
+        <v>81.7</v>
       </c>
       <c r="R45" s="3" t="n">
         <v>1.85</v>
@@ -3685,7 +3685,7 @@
         <v>11.48</v>
       </c>
       <c r="Q46" s="3" t="n">
-        <v>125</v>
+        <v>128.5</v>
       </c>
       <c r="R46" s="3" t="n">
         <v>4.5</v>
@@ -3754,7 +3754,7 @@
         <v>19.89</v>
       </c>
       <c r="Q47" s="3" t="n">
-        <v>161.5</v>
+        <v>159</v>
       </c>
       <c r="R47" s="3" t="n">
         <v>4</v>
@@ -3823,7 +3823,7 @@
         <v>15.1</v>
       </c>
       <c r="Q48" s="3" t="n">
-        <v>98.3</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="R48" s="3" t="n">
         <v>2</v>
@@ -3892,7 +3892,7 @@
         <v>389</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>18.6</v>
+        <v>18.3</v>
       </c>
       <c r="R49" s="3" t="n">
         <v>0.29</v>
@@ -3961,7 +3961,7 @@
         <v>13.89</v>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>177</v>
+        <v>173.5</v>
       </c>
       <c r="R50" s="3" t="n">
         <v>2.57</v>
@@ -4030,7 +4030,7 @@
         <v>66.98</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>59.6</v>
+        <v>58.2</v>
       </c>
       <c r="R51" s="3" t="n">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>8.75</v>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>34.4</v>
+        <v>34.45</v>
       </c>
       <c r="R52" s="3" t="n">
         <v>1.5</v>
@@ -4168,7 +4168,7 @@
         <v>31.01</v>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>126</v>
+        <v>127.5</v>
       </c>
       <c r="R53" s="3" t="n">
         <v>0.5</v>
@@ -4237,7 +4237,7 @@
         <v>11.84</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>25.55</v>
+        <v>24.8</v>
       </c>
       <c r="R54" s="3" t="n">
         <v>0.45</v>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3">
@@ -4371,7 +4371,7 @@
         <v>17.91</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>29.15</v>
+        <v>29.05</v>
       </c>
       <c r="R56" s="3" t="n">
         <v>1</v>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n">
-        <v>19.1</v>
+        <v>18.9</v>
       </c>
       <c r="R57" s="3" t="n">
         <v>0.15</v>
@@ -4503,7 +4503,7 @@
         <v>10.74</v>
       </c>
       <c r="Q58" s="3" t="n">
-        <v>81.2</v>
+        <v>82.5</v>
       </c>
       <c r="R58" s="3" t="n">
         <v>4.3</v>
@@ -4572,7 +4572,7 @@
         <v>9.08</v>
       </c>
       <c r="Q59" s="3" t="n">
-        <v>22.4</v>
+        <v>22.05</v>
       </c>
       <c r="R59" s="3" t="n">
         <v>2</v>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n">
-        <v>16.9</v>
+        <v>16.65</v>
       </c>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3">
@@ -4706,7 +4706,7 @@
         <v>14.86</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>64.7</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="R61" s="3" t="n">
         <v>3.3</v>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="n">
-        <v>14.1</v>
+        <v>13.9</v>
       </c>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3">
@@ -4840,7 +4840,7 @@
         <v>9.390000000000001</v>
       </c>
       <c r="Q63" s="3" t="n">
-        <v>48.2</v>
+        <v>46.5</v>
       </c>
       <c r="R63" s="3" t="n">
         <v>1.5</v>
@@ -4909,7 +4909,7 @@
         <v>52.88</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="R64" s="3" t="n">
         <v>2</v>
@@ -4978,7 +4978,7 @@
         <v>68.91</v>
       </c>
       <c r="Q65" s="3" t="n">
-        <v>12600</v>
+        <v>12080</v>
       </c>
       <c r="R65" s="3" t="n">
         <v>51</v>
@@ -5047,7 +5047,7 @@
         <v>10.49</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>130.5</v>
+        <v>127</v>
       </c>
       <c r="R66" s="3" t="n">
         <v>13.08</v>
@@ -5116,7 +5116,7 @@
         <v>5.72</v>
       </c>
       <c r="Q67" s="3" t="n">
-        <v>30.4</v>
+        <v>30.25</v>
       </c>
       <c r="R67" s="3" t="n">
         <v>1.3</v>
@@ -5183,7 +5183,7 @@
         <v>10.78</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>25.85</v>
+        <v>25.75</v>
       </c>
       <c r="R68" s="3" t="n">
         <v>0.27</v>
@@ -5252,7 +5252,7 @@
         <v>16.7</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>30.6</v>
+        <v>30.4</v>
       </c>
       <c r="R69" s="3" t="n">
         <v>1.8</v>
@@ -5321,7 +5321,7 @@
         <v>37.55</v>
       </c>
       <c r="Q70" s="3" t="n">
-        <v>16.85</v>
+        <v>16.7</v>
       </c>
       <c r="R70" s="3" t="n">
         <v>0.65</v>
@@ -5390,7 +5390,7 @@
         <v>32.92</v>
       </c>
       <c r="Q71" s="3" t="n">
-        <v>30.2</v>
+        <v>30</v>
       </c>
       <c r="R71" s="3" t="n">
         <v>0.5600000000000001</v>
@@ -5459,7 +5459,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="Q72" s="3" t="n">
-        <v>53.1</v>
+        <v>52.8</v>
       </c>
       <c r="R72" s="3" t="n">
         <v>3.6</v>
@@ -5528,7 +5528,7 @@
         <v>10.2</v>
       </c>
       <c r="Q73" s="3" t="n">
-        <v>64</v>
+        <v>63.1</v>
       </c>
       <c r="R73" s="3" t="n">
         <v>3.06</v>
@@ -5597,7 +5597,7 @@
         <v>12.64</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="R74" s="3" t="n">
         <v>20</v>
@@ -5666,7 +5666,7 @@
         <v>39.9</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>18.7</v>
+        <v>19.1</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>0</v>
@@ -5735,7 +5735,7 @@
         <v>11.44</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>83.5</v>
+        <v>82.7</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>6.5</v>
@@ -5802,7 +5802,7 @@
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="n">
-        <v>47.05</v>
+        <v>47.1</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>0.84</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="n">
-        <v>31.1</v>
+        <v>30.55</v>
       </c>
       <c r="R79" s="3" t="n"/>
       <c r="S79" s="3">
@@ -6005,7 +6005,7 @@
         <v>31.23</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>5.5</v>
@@ -6074,7 +6074,7 @@
         <v>18.2</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>142.5</v>
+        <v>140.5</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>2.61</v>
@@ -6143,7 +6143,7 @@
         <v>59.99</v>
       </c>
       <c r="Q82" s="3" t="n">
-        <v>1675</v>
+        <v>1620</v>
       </c>
       <c r="R82" s="3" t="n">
         <v>11.6</v>
@@ -6212,7 +6212,7 @@
         <v>28.36</v>
       </c>
       <c r="Q83" s="3" t="n">
-        <v>31.15</v>
+        <v>30.45</v>
       </c>
       <c r="R83" s="3" t="n">
         <v>0.6</v>
@@ -6281,7 +6281,7 @@
         <v>34.7</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>225.5</v>
+        <v>221.5</v>
       </c>
       <c r="R84" s="3" t="n">
         <v>2.8</v>
@@ -6350,7 +6350,7 @@
         <v>11.08</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>2</v>
@@ -6419,7 +6419,7 @@
         <v>17.11</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>7.17</v>
@@ -6488,7 +6488,7 @@
         <v>21.71</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>38.65</v>
+        <v>37.8</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>1.1</v>
@@ -6557,7 +6557,7 @@
         <v>41.89</v>
       </c>
       <c r="Q88" s="3" t="n">
-        <v>572</v>
+        <v>544</v>
       </c>
       <c r="R88" s="3" t="n">
         <v>6</v>
@@ -6626,7 +6626,7 @@
         <v>104.42</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.1</v>
+        <v>46</v>
       </c>
       <c r="R89" s="3" t="n">
         <v>0.9</v>
@@ -6695,7 +6695,7 @@
         <v>19.26</v>
       </c>
       <c r="Q90" s="3" t="n">
-        <v>42.2</v>
+        <v>41.6</v>
       </c>
       <c r="R90" s="3" t="n">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>32.47</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>2450</v>
+        <v>2410</v>
       </c>
       <c r="R91" s="3" t="n">
         <v>12</v>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="n">
-        <v>18.85</v>
+        <v>19</v>
       </c>
       <c r="R92" s="3" t="n"/>
       <c r="S92" s="3">
@@ -6898,7 +6898,7 @@
         <v>32.46</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>122.5</v>
+        <v>119</v>
       </c>
       <c r="R93" s="3" t="n"/>
       <c r="S93" s="3">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="n">
-        <v>45.65</v>
+        <v>47.75</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>0</v>
@@ -7032,7 +7032,7 @@
         <v>20.23</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>179.5</v>
+        <v>171.5</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>0.5</v>
@@ -7101,7 +7101,7 @@
         <v>36.14</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>1965</v>
+        <v>1885</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>15</v>
@@ -7170,7 +7170,7 @@
         <v>12.44</v>
       </c>
       <c r="Q97" s="3" t="n">
-        <v>88.8</v>
+        <v>89</v>
       </c>
       <c r="R97" s="3" t="n">
         <v>4.2</v>
@@ -7239,7 +7239,7 @@
         <v>46.8</v>
       </c>
       <c r="Q98" s="3" t="n">
-        <v>235.5</v>
+        <v>234</v>
       </c>
       <c r="R98" s="3" t="n">
         <v>1.03</v>
@@ -7308,7 +7308,7 @@
         <v>38.31</v>
       </c>
       <c r="Q99" s="3" t="n">
-        <v>29</v>
+        <v>28.7</v>
       </c>
       <c r="R99" s="3" t="n">
         <v>1</v>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="n">
-        <v>31.5</v>
+        <v>31.1</v>
       </c>
       <c r="R100" s="3" t="n">
         <v>1.3</v>
@@ -7444,7 +7444,7 @@
         <v>25.51</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>65</v>
+        <v>65.7</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>1.5</v>
@@ -7513,7 +7513,7 @@
         <v>21.95</v>
       </c>
       <c r="Q102" s="3" t="n">
-        <v>41.85</v>
+        <v>41.5</v>
       </c>
       <c r="R102" s="3" t="n">
         <v>1</v>
@@ -7582,7 +7582,7 @@
         <v>20.81</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>62.6</v>
+        <v>62</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>2</v>
@@ -7647,7 +7647,7 @@
         <v>13.35</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>989</v>
+        <v>924</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>42</v>
@@ -7716,7 +7716,7 @@
         <v>23.99</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3">
@@ -7779,7 +7779,7 @@
         <v>54.59</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>2180</v>
+        <v>2160</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>19.5</v>
@@ -7848,7 +7848,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>47.6</v>
+        <v>47.15</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>2</v>
@@ -7917,7 +7917,7 @@
         <v>93.89</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>52.6</v>
+        <v>50.7</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>0.61</v>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="P109" s="3" t="n"/>
       <c r="Q109" s="3" t="n">
-        <v>41.15</v>
+        <v>40.7</v>
       </c>
       <c r="R109" s="3" t="n"/>
       <c r="S109" s="3">
@@ -8051,7 +8051,7 @@
         <v>36.79</v>
       </c>
       <c r="Q110" s="3" t="n">
-        <v>1045</v>
+        <v>1030</v>
       </c>
       <c r="R110" s="3" t="n">
         <v>9.800000000000001</v>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n">
-        <v>27.85</v>
+        <v>27.45</v>
       </c>
       <c r="R111" s="3" t="n"/>
       <c r="S111" s="3">
@@ -8254,7 +8254,7 @@
         <v>29.45</v>
       </c>
       <c r="Q113" s="3" t="n">
-        <v>122</v>
+        <v>118.5</v>
       </c>
       <c r="R113" s="3" t="n"/>
       <c r="S113" s="3">
@@ -8317,7 +8317,7 @@
         <v>12.87</v>
       </c>
       <c r="Q114" s="3" t="n">
-        <v>351.5</v>
+        <v>349</v>
       </c>
       <c r="R114" s="3" t="n">
         <v>12</v>
@@ -8453,7 +8453,7 @@
         <v>25.49</v>
       </c>
       <c r="Q116" s="3" t="n">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3">
@@ -8520,7 +8520,7 @@
         <v>14.25</v>
       </c>
       <c r="Q117" s="3" t="n">
-        <v>336</v>
+        <v>336.5</v>
       </c>
       <c r="R117" s="3" t="n">
         <v>15.6</v>
@@ -8589,7 +8589,7 @@
         <v>93.59</v>
       </c>
       <c r="Q118" s="3" t="n">
-        <v>5375</v>
+        <v>5365</v>
       </c>
       <c r="R118" s="3" t="n">
         <v>25</v>
@@ -8658,7 +8658,7 @@
         <v>12.01</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>103.5</v>
+        <v>105</v>
       </c>
       <c r="R119" s="3" t="n">
         <v>7.2</v>
@@ -8727,7 +8727,7 @@
         <v>46.19</v>
       </c>
       <c r="Q120" s="3" t="n">
-        <v>77.7</v>
+        <v>75.2</v>
       </c>
       <c r="R120" s="3" t="n">
         <v>0.05</v>
@@ -8796,7 +8796,7 @@
         <v>5.36</v>
       </c>
       <c r="Q121" s="3" t="n">
-        <v>43.4</v>
+        <v>42.3</v>
       </c>
       <c r="R121" s="3" t="n">
         <v>1</v>
@@ -8865,7 +8865,7 @@
         <v>13.8</v>
       </c>
       <c r="Q122" s="3" t="n">
-        <v>61.8</v>
+        <v>62.1</v>
       </c>
       <c r="R122" s="3" t="n">
         <v>4.14</v>
@@ -8934,7 +8934,7 @@
         <v>43.26</v>
       </c>
       <c r="Q123" s="3" t="n">
-        <v>659</v>
+        <v>674</v>
       </c>
       <c r="R123" s="3" t="n">
         <v>9.17</v>
@@ -9003,7 +9003,7 @@
         <v>255</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>24.9</v>
+        <v>24.1</v>
       </c>
       <c r="R124" s="3" t="n">
         <v>0</v>
@@ -9072,7 +9072,7 @@
         <v>32.81</v>
       </c>
       <c r="Q125" s="3" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="R125" s="3" t="n">
         <v>2</v>
@@ -9141,7 +9141,7 @@
         <v>16.97</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>1060</v>
+        <v>1005</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>40</v>
@@ -9210,7 +9210,7 @@
         <v>19.87</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>515</v>
+        <v>493</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>1.35</v>
@@ -9279,7 +9279,7 @@
         <v>106.67</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>31.2</v>
+        <v>30.2</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>0.4</v>
@@ -9348,7 +9348,7 @@
         <v>26.52</v>
       </c>
       <c r="Q129" s="3" t="n">
-        <v>139.5</v>
+        <v>140.5</v>
       </c>
       <c r="R129" s="3" t="n">
         <v>5.2</v>
@@ -9417,7 +9417,7 @@
         <v>15.32</v>
       </c>
       <c r="Q130" s="3" t="n">
-        <v>165</v>
+        <v>164.5</v>
       </c>
       <c r="R130" s="3" t="n">
         <v>5.24</v>
@@ -9486,7 +9486,7 @@
         <v>822</v>
       </c>
       <c r="Q131" s="3" t="n">
-        <v>96.09999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="R131" s="3" t="n">
         <v>0.1</v>
@@ -9555,7 +9555,7 @@
         <v>18.02</v>
       </c>
       <c r="Q132" s="3" t="n">
-        <v>250.5</v>
+        <v>255</v>
       </c>
       <c r="R132" s="3" t="n">
         <v>5.9</v>
@@ -9624,7 +9624,7 @@
         <v>15.05</v>
       </c>
       <c r="Q133" s="3" t="n">
-        <v>77.2</v>
+        <v>76.5</v>
       </c>
       <c r="R133" s="3" t="n">
         <v>4.084</v>
@@ -9693,7 +9693,7 @@
         <v>20.83</v>
       </c>
       <c r="Q134" s="3" t="n">
-        <v>115</v>
+        <v>111.5</v>
       </c>
       <c r="R134" s="3" t="n">
         <v>3.01</v>
@@ -9762,7 +9762,7 @@
         <v>32.37</v>
       </c>
       <c r="Q135" s="3" t="n">
-        <v>271.5</v>
+        <v>263</v>
       </c>
       <c r="R135" s="3" t="n">
         <v>1</v>
@@ -9831,7 +9831,7 @@
         <v>5.09</v>
       </c>
       <c r="Q136" s="3" t="n">
-        <v>282.5</v>
+        <v>276.5</v>
       </c>
       <c r="R136" s="3" t="n">
         <v>11.78</v>
@@ -9900,7 +9900,7 @@
         <v>69.53</v>
       </c>
       <c r="Q137" s="3" t="n">
-        <v>4720</v>
+        <v>4585</v>
       </c>
       <c r="R137" s="3" t="n">
         <v>53.5</v>
@@ -9969,7 +9969,7 @@
         <v>99.51000000000001</v>
       </c>
       <c r="Q138" s="3" t="n">
-        <v>532</v>
+        <v>515</v>
       </c>
       <c r="R138" s="3" t="n">
         <v>2.62</v>
@@ -10038,7 +10038,7 @@
         <v>13.06</v>
       </c>
       <c r="Q139" s="3" t="n">
-        <v>128</v>
+        <v>126.5</v>
       </c>
       <c r="R139" s="3" t="n">
         <v>8.851000000000001</v>
@@ -10101,7 +10101,7 @@
         <v>505.26</v>
       </c>
       <c r="Q140" s="3" t="n">
-        <v>193.5</v>
+        <v>188.5</v>
       </c>
       <c r="R140" s="3" t="n">
         <v>0.5</v>
@@ -10170,7 +10170,7 @@
         <v>66.23999999999999</v>
       </c>
       <c r="Q141" s="3" t="n">
-        <v>101.5</v>
+        <v>106</v>
       </c>
       <c r="R141" s="3" t="n"/>
       <c r="S141" s="3">
@@ -10237,7 +10237,7 @@
         <v>53.39</v>
       </c>
       <c r="Q142" s="3" t="n">
-        <v>575</v>
+        <v>552</v>
       </c>
       <c r="R142" s="3" t="n">
         <v>5.5</v>
@@ -10306,7 +10306,7 @@
         <v>22.2</v>
       </c>
       <c r="Q143" s="3" t="n">
-        <v>217</v>
+        <v>213.5</v>
       </c>
       <c r="R143" s="3" t="n">
         <v>3.5</v>
@@ -10444,7 +10444,7 @@
         <v>18.78</v>
       </c>
       <c r="Q145" s="3" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R145" s="3" t="n">
         <v>2.97</v>
@@ -10507,7 +10507,7 @@
         <v>24.79</v>
       </c>
       <c r="Q146" s="3" t="n">
-        <v>124</v>
+        <v>118.5</v>
       </c>
       <c r="R146" s="3" t="n">
         <v>2</v>
@@ -10576,7 +10576,7 @@
         <v>18.09</v>
       </c>
       <c r="Q147" s="3" t="n">
-        <v>156.5</v>
+        <v>157.5</v>
       </c>
       <c r="R147" s="3" t="n">
         <v>7.8</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="Q148" s="3" t="n">
-        <v>154.5</v>
+        <v>150</v>
       </c>
       <c r="R148" s="3" t="n">
         <v>1.8</v>
@@ -10702,7 +10702,7 @@
         <v>214.66</v>
       </c>
       <c r="Q149" s="3" t="n">
-        <v>242</v>
+        <v>237.5</v>
       </c>
       <c r="R149" s="3" t="n">
         <v>0.25</v>
@@ -10771,7 +10771,7 @@
         <v>25.65</v>
       </c>
       <c r="Q150" s="3" t="n">
-        <v>38.6</v>
+        <v>36.9</v>
       </c>
       <c r="R150" s="3" t="n">
         <v>1.2</v>
@@ -10840,7 +10840,7 @@
         <v>33.99</v>
       </c>
       <c r="Q151" s="3" t="n">
-        <v>334</v>
+        <v>311.5</v>
       </c>
       <c r="R151" s="3" t="n">
         <v>2.5</v>
@@ -10903,7 +10903,7 @@
         <v>33.27</v>
       </c>
       <c r="Q152" s="3" t="n">
-        <v>174.5</v>
+        <v>173.5</v>
       </c>
       <c r="R152" s="3" t="n">
         <v>4</v>
@@ -10966,7 +10966,7 @@
         <v>15.64</v>
       </c>
       <c r="Q153" s="3" t="n">
-        <v>40.15</v>
+        <v>39.95</v>
       </c>
       <c r="R153" s="3" t="n">
         <v>0.5</v>
@@ -11035,7 +11035,7 @@
         <v>8.07</v>
       </c>
       <c r="Q154" s="3" t="n">
-        <v>22.25</v>
+        <v>22.15</v>
       </c>
       <c r="R154" s="3" t="n">
         <v>1.2</v>
@@ -11104,7 +11104,7 @@
         <v>9.81</v>
       </c>
       <c r="Q155" s="3" t="n">
-        <v>31.45</v>
+        <v>31.3</v>
       </c>
       <c r="R155" s="3" t="n">
         <v>2.6</v>
@@ -11228,7 +11228,7 @@
         <v>10.85</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>36.75</v>
+        <v>36.45</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>1.62</v>
@@ -11287,7 +11287,7 @@
         <v>29.47</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>19.55</v>
+        <v>20.1</v>
       </c>
       <c r="R158" s="3" t="n"/>
       <c r="S158" s="3">
@@ -11348,7 +11348,7 @@
         <v>8.91</v>
       </c>
       <c r="Q159" s="3" t="n">
-        <v>90.09999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="R159" s="3" t="n">
         <v>4.6</v>
@@ -11417,7 +11417,7 @@
         <v>9.81</v>
       </c>
       <c r="Q160" s="3" t="n">
-        <v>35.35</v>
+        <v>35.15</v>
       </c>
       <c r="R160" s="3" t="n">
         <v>0.6</v>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="P161" s="3" t="n"/>
       <c r="Q161" s="3" t="n">
-        <v>49.45</v>
+        <v>49.1</v>
       </c>
       <c r="R161" s="3" t="n">
         <v>0.62</v>
@@ -11616,7 +11616,7 @@
         <v>13.37</v>
       </c>
       <c r="Q163" s="3" t="n">
-        <v>39.1</v>
+        <v>37.9</v>
       </c>
       <c r="R163" s="3" t="n">
         <v>1.03</v>
@@ -11679,7 +11679,7 @@
         <v>36.53</v>
       </c>
       <c r="Q164" s="3" t="n">
-        <v>34.4</v>
+        <v>33.75</v>
       </c>
       <c r="R164" s="3" t="n">
         <v>2.8</v>
@@ -11738,7 +11738,7 @@
         <v>7.81</v>
       </c>
       <c r="Q165" s="3" t="n">
-        <v>94.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="R165" s="3" t="n">
         <v>8</v>
@@ -11801,7 +11801,7 @@
         <v>14.45</v>
       </c>
       <c r="Q166" s="3" t="n">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="R166" s="3" t="n">
         <v>9.67</v>
@@ -11870,7 +11870,7 @@
         <v>8.68</v>
       </c>
       <c r="Q167" s="3" t="n">
-        <v>231</v>
+        <v>234.5</v>
       </c>
       <c r="R167" s="3" t="n">
         <v>16</v>
@@ -11933,7 +11933,7 @@
         <v>7.47</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>36.25</v>
+        <v>36.5</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>1</v>
@@ -12002,7 +12002,7 @@
         <v>10.71</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>78.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>2.8</v>
@@ -12071,7 +12071,7 @@
         <v>10.46</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>53</v>
+        <v>53.3</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>2.7</v>
@@ -12140,7 +12140,7 @@
         <v>11.62</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>58</v>
+        <v>59.4</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>2</v>
@@ -12209,7 +12209,7 @@
         <v>9.210000000000001</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>20.2</v>
+        <v>20.4</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>0.8100000000000001</v>
@@ -12278,7 +12278,7 @@
         <v>6.22</v>
       </c>
       <c r="Q173" s="3" t="n">
-        <v>110.5</v>
+        <v>112</v>
       </c>
       <c r="R173" s="3" t="n">
         <v>3</v>
@@ -12347,7 +12347,7 @@
         <v>8.4</v>
       </c>
       <c r="Q174" s="3" t="n">
-        <v>41.8</v>
+        <v>42.35</v>
       </c>
       <c r="R174" s="3" t="n">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>21.23</v>
       </c>
       <c r="Q175" s="3" t="n">
-        <v>26</v>
+        <v>26.05</v>
       </c>
       <c r="R175" s="3" t="n">
         <v>1.15</v>
@@ -12554,7 +12554,7 @@
         <v>11.35</v>
       </c>
       <c r="Q177" s="3" t="n">
-        <v>100.5</v>
+        <v>101</v>
       </c>
       <c r="R177" s="3" t="n">
         <v>3.5</v>
@@ -12623,7 +12623,7 @@
         <v>25.51</v>
       </c>
       <c r="Q178" s="3" t="n">
-        <v>172.5</v>
+        <v>173</v>
       </c>
       <c r="R178" s="3" t="n">
         <v>5</v>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P179" s="3" t="n"/>
       <c r="Q179" s="3" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R179" s="3" t="n"/>
       <c r="S179" s="3">
@@ -12757,7 +12757,7 @@
         <v>17.48</v>
       </c>
       <c r="Q180" s="3" t="n">
-        <v>46</v>
+        <v>45.75</v>
       </c>
       <c r="R180" s="3" t="n">
         <v>0.5</v>
@@ -12895,7 +12895,7 @@
         <v>13.19</v>
       </c>
       <c r="Q182" s="3" t="n">
-        <v>229.5</v>
+        <v>229</v>
       </c>
       <c r="R182" s="3" t="n">
         <v>16.12</v>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="P183" s="3" t="n"/>
       <c r="Q183" s="3" t="n">
-        <v>22.5</v>
+        <v>22.3</v>
       </c>
       <c r="R183" s="3" t="n">
         <v>1.25</v>
@@ -13031,7 +13031,7 @@
         <v>6.51</v>
       </c>
       <c r="Q184" s="3" t="n">
-        <v>18.35</v>
+        <v>18.5</v>
       </c>
       <c r="R184" s="3" t="n">
         <v>0</v>
@@ -13100,7 +13100,7 @@
         <v>19.32</v>
       </c>
       <c r="Q185" s="3" t="n">
-        <v>218.5</v>
+        <v>216.5</v>
       </c>
       <c r="R185" s="3" t="n">
         <v>9</v>
@@ -13169,7 +13169,7 @@
         <v>4.28</v>
       </c>
       <c r="Q186" s="3" t="n">
-        <v>56.9</v>
+        <v>56.6</v>
       </c>
       <c r="R186" s="3" t="n">
         <v>1.9</v>
@@ -13236,7 +13236,7 @@
       </c>
       <c r="P187" s="3" t="n"/>
       <c r="Q187" s="3" t="n">
-        <v>27.3</v>
+        <v>25.4</v>
       </c>
       <c r="R187" s="3" t="n">
         <v>0.12</v>
@@ -13305,7 +13305,7 @@
         <v>13.84</v>
       </c>
       <c r="Q188" s="3" t="n">
-        <v>115</v>
+        <v>115.5</v>
       </c>
       <c r="R188" s="3" t="n">
         <v>6.79</v>
@@ -13374,7 +13374,7 @@
         <v>8.09</v>
       </c>
       <c r="Q189" s="3" t="n">
-        <v>312</v>
+        <v>290.5</v>
       </c>
       <c r="R189" s="3" t="n">
         <v>1</v>
@@ -13443,7 +13443,7 @@
         <v>24.52</v>
       </c>
       <c r="Q190" s="3" t="n">
-        <v>6720</v>
+        <v>6660</v>
       </c>
       <c r="R190" s="3" t="n">
         <v>93.5</v>
@@ -13579,7 +13579,7 @@
         <v>15.88</v>
       </c>
       <c r="Q192" s="3" t="n">
-        <v>87.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="R192" s="3" t="n">
         <v>0.4</v>
@@ -13648,7 +13648,7 @@
         <v>13.13</v>
       </c>
       <c r="Q193" s="3" t="n">
-        <v>131.5</v>
+        <v>130.5</v>
       </c>
       <c r="R193" s="3" t="n">
         <v>7.5</v>
@@ -13717,7 +13717,7 @@
         <v>82</v>
       </c>
       <c r="Q194" s="3" t="n">
-        <v>110</v>
+        <v>109.5</v>
       </c>
       <c r="R194" s="3" t="n">
         <v>0.5</v>
@@ -13786,7 +13786,7 @@
         <v>43.12</v>
       </c>
       <c r="Q195" s="3" t="n">
-        <v>3460</v>
+        <v>3370</v>
       </c>
       <c r="R195" s="3" t="n">
         <v>17.9</v>
@@ -13855,7 +13855,7 @@
         <v>22.85</v>
       </c>
       <c r="Q196" s="3" t="n">
-        <v>139</v>
+        <v>137.5</v>
       </c>
       <c r="R196" s="3" t="n">
         <v>4.6</v>
@@ -13924,7 +13924,7 @@
         <v>11.98</v>
       </c>
       <c r="Q197" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>83.2</v>
       </c>
       <c r="R197" s="3" t="n">
         <v>3.5</v>
@@ -13993,7 +13993,7 @@
         <v>23.34</v>
       </c>
       <c r="Q198" s="3" t="n">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="R198" s="3" t="n">
         <v>9.1</v>
@@ -14062,7 +14062,7 @@
         <v>63.12</v>
       </c>
       <c r="Q199" s="3" t="n">
-        <v>803</v>
+        <v>744</v>
       </c>
       <c r="R199" s="3" t="n">
         <v>5.8</v>
@@ -14131,7 +14131,7 @@
         <v>9.35</v>
       </c>
       <c r="Q200" s="3" t="n">
-        <v>62.3</v>
+        <v>61.7</v>
       </c>
       <c r="R200" s="3" t="n">
         <v>3</v>
@@ -14200,7 +14200,7 @@
         <v>15.83</v>
       </c>
       <c r="Q201" s="3" t="n">
-        <v>113</v>
+        <v>116.5</v>
       </c>
       <c r="R201" s="3" t="n">
         <v>5.5</v>
@@ -14269,7 +14269,7 @@
         <v>22.35</v>
       </c>
       <c r="Q202" s="3" t="n">
-        <v>266.5</v>
+        <v>263</v>
       </c>
       <c r="R202" s="3" t="n">
         <v>7</v>
@@ -14338,7 +14338,7 @@
         <v>9.99</v>
       </c>
       <c r="Q203" s="3" t="n">
-        <v>42.05</v>
+        <v>41.55</v>
       </c>
       <c r="R203" s="3" t="n">
         <v>1.92</v>
@@ -14407,7 +14407,7 @@
         <v>17.86</v>
       </c>
       <c r="Q204" s="3" t="n">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="R204" s="3" t="n">
         <v>23</v>
@@ -14476,7 +14476,7 @@
         <v>68.31</v>
       </c>
       <c r="Q205" s="3" t="n">
-        <v>179</v>
+        <v>169.5</v>
       </c>
       <c r="R205" s="3" t="n">
         <v>1.8</v>
@@ -14545,7 +14545,7 @@
         <v>10.57</v>
       </c>
       <c r="Q206" s="3" t="n">
-        <v>192.5</v>
+        <v>191</v>
       </c>
       <c r="R206" s="3" t="n">
         <v>7.8</v>
@@ -14614,7 +14614,7 @@
         <v>67.91</v>
       </c>
       <c r="Q207" s="3" t="n">
-        <v>994</v>
+        <v>977</v>
       </c>
       <c r="R207" s="3" t="n">
         <v>1.98</v>
@@ -14673,7 +14673,7 @@
         <v>32.82</v>
       </c>
       <c r="Q208" s="3" t="n">
-        <v>180.5</v>
+        <v>176</v>
       </c>
       <c r="R208" s="3" t="n">
         <v>4.8</v>
@@ -14742,7 +14742,7 @@
         <v>20.91</v>
       </c>
       <c r="Q209" s="3" t="n">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="R209" s="3" t="n">
         <v>12.7</v>
@@ -14811,7 +14811,7 @@
         <v>21.74</v>
       </c>
       <c r="Q210" s="3" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="R210" s="3" t="n">
         <v>3.94</v>
@@ -14880,7 +14880,7 @@
         <v>218.59</v>
       </c>
       <c r="Q211" s="3" t="n">
-        <v>2830</v>
+        <v>2810</v>
       </c>
       <c r="R211" s="3" t="n">
         <v>3</v>
@@ -14949,7 +14949,7 @@
         <v>15.63</v>
       </c>
       <c r="Q212" s="3" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="R212" s="3" t="n">
         <v>2.9304</v>
@@ -15018,7 +15018,7 @@
         <v>19.92</v>
       </c>
       <c r="Q213" s="3" t="n">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="R213" s="3" t="n">
         <v>4.8</v>
@@ -15087,7 +15087,7 @@
         <v>44.42</v>
       </c>
       <c r="Q214" s="3" t="n">
-        <v>461.5</v>
+        <v>437.5</v>
       </c>
       <c r="R214" s="3" t="n">
         <v>2</v>
@@ -15156,7 +15156,7 @@
         <v>41.08</v>
       </c>
       <c r="Q215" s="3" t="n">
-        <v>2460</v>
+        <v>2325</v>
       </c>
       <c r="R215" s="3" t="n">
         <v>46.08</v>
@@ -15225,7 +15225,7 @@
         <v>6.7</v>
       </c>
       <c r="Q216" s="3" t="n">
-        <v>167</v>
+        <v>162.5</v>
       </c>
       <c r="R216" s="3" t="n">
         <v>3.2586</v>
@@ -15292,7 +15292,7 @@
       </c>
       <c r="P217" s="3" t="n"/>
       <c r="Q217" s="3" t="n">
-        <v>61.4</v>
+        <v>62.3</v>
       </c>
       <c r="R217" s="3" t="n"/>
       <c r="S217" s="3">
@@ -15359,7 +15359,7 @@
         <v>75.09999999999999</v>
       </c>
       <c r="Q218" s="3" t="n">
-        <v>707</v>
+        <v>670</v>
       </c>
       <c r="R218" s="3" t="n">
         <v>1.75</v>
@@ -15428,7 +15428,7 @@
         <v>47.34</v>
       </c>
       <c r="Q219" s="3" t="n">
-        <v>848</v>
+        <v>828</v>
       </c>
       <c r="R219" s="3" t="n">
         <v>3.91</v>
@@ -15497,7 +15497,7 @@
         <v>159.93</v>
       </c>
       <c r="Q220" s="3" t="n">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="R220" s="3" t="n">
         <v>1.52</v>
@@ -15566,7 +15566,7 @@
         <v>52.7</v>
       </c>
       <c r="Q221" s="3" t="n">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="R221" s="3" t="n">
         <v>11.47</v>
@@ -15635,7 +15635,7 @@
         <v>10.97</v>
       </c>
       <c r="Q222" s="3" t="n">
-        <v>127.5</v>
+        <v>127</v>
       </c>
       <c r="R222" s="3" t="n">
         <v>10</v>
@@ -15704,7 +15704,7 @@
         <v>15.77</v>
       </c>
       <c r="Q223" s="3" t="n">
-        <v>183.5</v>
+        <v>181.5</v>
       </c>
       <c r="R223" s="3" t="n">
         <v>10.007</v>
@@ -15773,7 +15773,7 @@
         <v>15.37</v>
       </c>
       <c r="Q224" s="3" t="n">
-        <v>185</v>
+        <v>185.5</v>
       </c>
       <c r="R224" s="3" t="n">
         <v>5.5</v>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="P225" s="3" t="n"/>
       <c r="Q225" s="3" t="n">
-        <v>195</v>
+        <v>187.5</v>
       </c>
       <c r="R225" s="3" t="n">
         <v>0</v>
@@ -15909,7 +15909,7 @@
         <v>5.2</v>
       </c>
       <c r="Q226" s="3" t="n">
-        <v>407</v>
+        <v>402.5</v>
       </c>
       <c r="R226" s="3" t="n">
         <v>17</v>
@@ -15978,7 +15978,7 @@
         <v>29.44</v>
       </c>
       <c r="Q227" s="3" t="n">
-        <v>240</v>
+        <v>230.5</v>
       </c>
       <c r="R227" s="3" t="n">
         <v>4.2</v>
@@ -16047,7 +16047,7 @@
         <v>24.26</v>
       </c>
       <c r="Q228" s="3" t="n">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="R228" s="3" t="n">
         <v>4.1</v>
@@ -16116,7 +16116,7 @@
         <v>30.04</v>
       </c>
       <c r="Q229" s="3" t="n">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="R229" s="3" t="n">
         <v>3.43</v>
@@ -16185,7 +16185,7 @@
         <v>17.33</v>
       </c>
       <c r="Q230" s="3" t="n">
-        <v>704</v>
+        <v>693</v>
       </c>
       <c r="R230" s="3" t="n">
         <v>36</v>
@@ -16254,7 +16254,7 @@
         <v>19.18</v>
       </c>
       <c r="Q231" s="3" t="n">
-        <v>101.5</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="R231" s="3" t="n">
         <v>2.2833</v>
@@ -16323,7 +16323,7 @@
         <v>23.29</v>
       </c>
       <c r="Q232" s="3" t="n">
-        <v>1440</v>
+        <v>1360</v>
       </c>
       <c r="R232" s="3" t="n">
         <v>11.9</v>
@@ -16392,7 +16392,7 @@
         <v>21.44</v>
       </c>
       <c r="Q233" s="3" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="R233" s="3" t="n">
         <v>5.08</v>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="P234" s="3" t="n"/>
       <c r="Q234" s="3" t="n">
-        <v>182.5</v>
+        <v>179.5</v>
       </c>
       <c r="R234" s="3" t="n">
         <v>0</v>
@@ -16526,7 +16526,7 @@
       </c>
       <c r="P235" s="3" t="n"/>
       <c r="Q235" s="3" t="n">
-        <v>714</v>
+        <v>681</v>
       </c>
       <c r="R235" s="3" t="n">
         <v>0</v>
@@ -16595,7 +16595,7 @@
         <v>51.02</v>
       </c>
       <c r="Q236" s="3" t="n">
-        <v>488</v>
+        <v>463.5</v>
       </c>
       <c r="R236" s="3" t="n">
         <v>2.5</v>
@@ -16664,7 +16664,7 @@
         <v>126.21</v>
       </c>
       <c r="Q237" s="3" t="n">
-        <v>189.5</v>
+        <v>183</v>
       </c>
       <c r="R237" s="3" t="n">
         <v>2</v>
@@ -16733,7 +16733,7 @@
         <v>188.94</v>
       </c>
       <c r="Q238" s="3" t="n">
-        <v>30.65</v>
+        <v>30.75</v>
       </c>
       <c r="R238" s="3" t="n"/>
       <c r="S238" s="3">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="P239" s="3" t="n"/>
       <c r="Q239" s="3" t="n">
-        <v>1070</v>
+        <v>1060</v>
       </c>
       <c r="R239" s="3" t="n">
         <v>17</v>
@@ -16867,7 +16867,7 @@
         <v>14.17</v>
       </c>
       <c r="Q240" s="3" t="n">
-        <v>283.5</v>
+        <v>279.5</v>
       </c>
       <c r="R240" s="3" t="n">
         <v>10.98</v>
@@ -16936,7 +16936,7 @@
         <v>20.39</v>
       </c>
       <c r="Q241" s="3" t="n">
-        <v>161</v>
+        <v>160.5</v>
       </c>
       <c r="R241" s="3" t="n">
         <v>5.0959</v>
@@ -17005,7 +17005,7 @@
         <v>137.52</v>
       </c>
       <c r="Q242" s="3" t="n">
-        <v>6225</v>
+        <v>6120</v>
       </c>
       <c r="R242" s="3" t="n">
         <v>20</v>
@@ -17074,7 +17074,7 @@
         <v>111.76</v>
       </c>
       <c r="Q243" s="3" t="n">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="R243" s="3" t="n">
         <v>1</v>
@@ -17143,7 +17143,7 @@
         <v>64.23</v>
       </c>
       <c r="Q244" s="3" t="n">
-        <v>49.35</v>
+        <v>47.7</v>
       </c>
       <c r="R244" s="3" t="n">
         <v>0.5</v>
@@ -17212,7 +17212,7 @@
         <v>109.3</v>
       </c>
       <c r="Q245" s="3" t="n">
-        <v>1355</v>
+        <v>1415</v>
       </c>
       <c r="R245" s="3" t="n">
         <v>6</v>
@@ -17281,7 +17281,7 @@
         <v>14.28</v>
       </c>
       <c r="Q246" s="3" t="n">
-        <v>221.5</v>
+        <v>207</v>
       </c>
       <c r="R246" s="3" t="n">
         <v>11</v>
@@ -17348,7 +17348,7 @@
       </c>
       <c r="P247" s="3" t="n"/>
       <c r="Q247" s="3" t="n">
-        <v>273</v>
+        <v>268.5</v>
       </c>
       <c r="R247" s="3" t="n">
         <v>13.53</v>
@@ -17417,7 +17417,7 @@
         <v>74.14</v>
       </c>
       <c r="Q248" s="3" t="n">
-        <v>2730</v>
+        <v>2580</v>
       </c>
       <c r="R248" s="3" t="n">
         <v>20.5</v>
@@ -17484,7 +17484,7 @@
       </c>
       <c r="P249" s="3" t="n"/>
       <c r="Q249" s="3" t="n">
-        <v>410</v>
+        <v>423</v>
       </c>
       <c r="R249" s="3" t="n">
         <v>1</v>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="P250" s="3" t="n"/>
       <c r="Q250" s="3" t="n">
-        <v>1575</v>
+        <v>1580</v>
       </c>
       <c r="R250" s="3" t="n">
         <v>34.93</v>
@@ -17620,7 +17620,7 @@
         <v>39.02</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>668</v>
+        <v>659</v>
       </c>
       <c r="R251" s="3" t="n">
         <v>12</v>
@@ -17689,7 +17689,7 @@
         <v>32.04</v>
       </c>
       <c r="Q252" s="3" t="n">
-        <v>16.65</v>
+        <v>16.4</v>
       </c>
       <c r="R252" s="3" t="n"/>
       <c r="S252" s="3">
@@ -17756,7 +17756,7 @@
         <v>40.66</v>
       </c>
       <c r="Q253" s="3" t="n">
-        <v>713</v>
+        <v>704</v>
       </c>
       <c r="R253" s="3" t="n">
         <v>11.7476</v>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="P254" s="3" t="n"/>
       <c r="Q254" s="3" t="n">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="R254" s="3" t="n">
         <v>4.21</v>
@@ -17892,7 +17892,7 @@
         <v>13.12</v>
       </c>
       <c r="Q255" s="3" t="n">
-        <v>221.5</v>
+        <v>219.5</v>
       </c>
       <c r="R255" s="3" t="n">
         <v>14.6</v>
@@ -17961,7 +17961,7 @@
         <v>12.38</v>
       </c>
       <c r="Q256" s="3" t="n">
-        <v>154.5</v>
+        <v>152.5</v>
       </c>
       <c r="R256" s="3" t="n">
         <v>8</v>
@@ -18030,7 +18030,7 @@
         <v>12.24</v>
       </c>
       <c r="Q257" s="3" t="n">
-        <v>239</v>
+        <v>242.5</v>
       </c>
       <c r="R257" s="3" t="n">
         <v>9.937099999999999</v>
@@ -18099,7 +18099,7 @@
         <v>126.38</v>
       </c>
       <c r="Q258" s="3" t="n">
-        <v>5790</v>
+        <v>5765</v>
       </c>
       <c r="R258" s="3" t="n">
         <v>21.72</v>
@@ -18158,7 +18158,7 @@
         <v>61.7</v>
       </c>
       <c r="Q259" s="3" t="n">
-        <v>4055</v>
+        <v>3650</v>
       </c>
       <c r="R259" s="3" t="n">
         <v>32.55</v>
@@ -18227,7 +18227,7 @@
         <v>44.4</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>1930</v>
+        <v>1875</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>15.18</v>
@@ -18296,7 +18296,7 @@
         <v>16.35</v>
       </c>
       <c r="Q261" s="3" t="n">
-        <v>62.6</v>
+        <v>61.7</v>
       </c>
       <c r="R261" s="3" t="n">
         <v>1.8</v>
@@ -18365,7 +18365,7 @@
         <v>46.77</v>
       </c>
       <c r="Q262" s="3" t="n">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="R262" s="3" t="n">
         <v>4</v>
@@ -18434,7 +18434,7 @@
         <v>31.17</v>
       </c>
       <c r="Q263" s="3" t="n">
-        <v>535</v>
+        <v>510</v>
       </c>
       <c r="R263" s="3" t="n">
         <v>5</v>
@@ -18503,7 +18503,7 @@
         <v>34.76</v>
       </c>
       <c r="Q264" s="3" t="n">
-        <v>691</v>
+        <v>663</v>
       </c>
       <c r="R264" s="3" t="n">
         <v>8</v>
@@ -18572,7 +18572,7 @@
         <v>9.85</v>
       </c>
       <c r="Q265" s="3" t="n">
-        <v>108</v>
+        <v>106.5</v>
       </c>
       <c r="R265" s="3" t="n">
         <v>3.64</v>
@@ -18641,7 +18641,7 @@
         <v>10.08</v>
       </c>
       <c r="Q266" s="3" t="n">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="R266" s="3" t="n">
         <v>1.05</v>
@@ -18710,7 +18710,7 @@
         <v>13.74</v>
       </c>
       <c r="Q267" s="3" t="n">
-        <v>39.4</v>
+        <v>40.5</v>
       </c>
       <c r="R267" s="3" t="n">
         <v>0.4</v>
@@ -18779,7 +18779,7 @@
         <v>15.93</v>
       </c>
       <c r="Q268" s="3" t="n">
-        <v>56</v>
+        <v>55.8</v>
       </c>
       <c r="R268" s="3" t="n">
         <v>3</v>
@@ -18848,7 +18848,7 @@
         <v>16.55</v>
       </c>
       <c r="Q269" s="3" t="n">
-        <v>82</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="R269" s="3" t="n"/>
       <c r="S269" s="3">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="P270" s="3" t="n"/>
       <c r="Q270" s="3" t="n">
-        <v>61.8</v>
+        <v>59.2</v>
       </c>
       <c r="R270" s="3" t="n"/>
       <c r="S270" s="3">
@@ -18980,7 +18980,7 @@
         <v>44.57</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>650</v>
+        <v>618</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>6.58</v>
@@ -19047,7 +19047,7 @@
       </c>
       <c r="P272" s="3" t="n"/>
       <c r="Q272" s="3" t="n">
-        <v>62</v>
+        <v>61.7</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>0.9</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="P273" s="3" t="n"/>
       <c r="Q273" s="3" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>1.08</v>
@@ -19183,7 +19183,7 @@
         <v>10.92</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>77.40000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>4.5</v>
@@ -19248,7 +19248,7 @@
         <v>18.4</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>29.75</v>
+        <v>29.5</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>0.85</v>
@@ -19317,7 +19317,7 @@
         <v>25.79</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>30.35</v>
+        <v>30.25</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>1.747</v>
@@ -19384,7 +19384,7 @@
       </c>
       <c r="P277" s="3" t="n"/>
       <c r="Q277" s="3" t="n">
-        <v>61.6</v>
+        <v>59.8</v>
       </c>
       <c r="R277" s="3" t="n"/>
       <c r="S277" s="3">
@@ -19451,7 +19451,7 @@
         <v>15.89</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>5.3</v>
@@ -19520,7 +19520,7 @@
         <v>12.98</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>164.5</v>
+        <v>162</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>8</v>
@@ -19589,7 +19589,7 @@
         <v>18.1</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>4.2</v>
@@ -19658,7 +19658,7 @@
         <v>60.42</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>0.8</v>
@@ -19723,7 +19723,7 @@
         <v>35.71</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>8</v>
@@ -19792,7 +19792,7 @@
         <v>105.22</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>290.5</v>
+        <v>298</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>1</v>
@@ -19861,7 +19861,7 @@
         <v>25.23</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>26.75</v>
+        <v>26.15</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>0.5</v>
@@ -19930,7 +19930,7 @@
         <v>110.95</v>
       </c>
       <c r="Q285" s="3" t="n">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="R285" s="3" t="n">
         <v>1.18</v>
@@ -19999,7 +19999,7 @@
         <v>25.87</v>
       </c>
       <c r="Q286" s="3" t="n">
-        <v>391</v>
+        <v>0</v>
       </c>
       <c r="R286" s="3" t="n">
         <v>12.1</v>
@@ -20068,7 +20068,7 @@
         <v>357.69</v>
       </c>
       <c r="Q287" s="3" t="n">
-        <v>45.55</v>
+        <v>43.9</v>
       </c>
       <c r="R287" s="3" t="n"/>
       <c r="S287" s="3">
@@ -20135,7 +20135,7 @@
         <v>61.06</v>
       </c>
       <c r="Q288" s="3" t="n">
-        <v>757</v>
+        <v>721</v>
       </c>
       <c r="R288" s="3" t="n">
         <v>8</v>
@@ -20194,7 +20194,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="Q289" s="3" t="n">
-        <v>48.35</v>
+        <v>48.85</v>
       </c>
       <c r="R289" s="3" t="n"/>
       <c r="S289" s="3">
@@ -20261,7 +20261,7 @@
         <v>66.61</v>
       </c>
       <c r="Q290" s="3" t="n">
-        <v>220.5</v>
+        <v>215</v>
       </c>
       <c r="R290" s="3" t="n">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>15.04</v>
       </c>
       <c r="Q291" s="3" t="n">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="R291" s="3" t="n">
         <v>18</v>
@@ -20397,7 +20397,7 @@
       </c>
       <c r="P292" s="3" t="n"/>
       <c r="Q292" s="3" t="n">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="R292" s="3" t="n">
         <v>0.22</v>
@@ -20466,7 +20466,7 @@
         <v>20.23</v>
       </c>
       <c r="Q293" s="3" t="n">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="R293" s="3" t="n">
         <v>6</v>
@@ -20535,7 +20535,7 @@
         <v>45.85</v>
       </c>
       <c r="Q294" s="3" t="n">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="R294" s="3" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         <v>24.09</v>
       </c>
       <c r="Q295" s="3" t="n">
-        <v>104.5</v>
+        <v>105.5</v>
       </c>
       <c r="R295" s="3" t="n">
         <v>3.45</v>
@@ -20673,7 +20673,7 @@
         <v>283.33</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>36.35</v>
+        <v>35.9</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>0.47</v>
@@ -20742,7 +20742,7 @@
         <v>12.22</v>
       </c>
       <c r="Q297" s="3" t="n">
-        <v>62.1</v>
+        <v>62.8</v>
       </c>
       <c r="R297" s="3" t="n">
         <v>4.57</v>
@@ -20809,7 +20809,7 @@
       </c>
       <c r="P298" s="3" t="n"/>
       <c r="Q298" s="3" t="n">
-        <v>116.5</v>
+        <v>112.5</v>
       </c>
       <c r="R298" s="3" t="n"/>
       <c r="S298" s="3">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="P299" s="3" t="n"/>
       <c r="Q299" s="3" t="n">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>2.5</v>
@@ -21008,7 +21008,7 @@
         <v>57.93</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>494.5</v>
+        <v>495</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>3.42</v>
@@ -21077,7 +21077,7 @@
         <v>18.65</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>172.5</v>
+        <v>170</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>7.72</v>
@@ -21146,7 +21146,7 @@
         <v>18.13</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>540</v>
+        <v>528</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>17.79</v>
@@ -21215,7 +21215,7 @@
         <v>4.13</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>276.5</v>
+        <v>280.5</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>3.45</v>
@@ -21274,7 +21274,7 @@
         <v>94.3</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>0.85</v>
@@ -21343,7 +21343,7 @@
         <v>85.43000000000001</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>571</v>
+        <v>531</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>2.15</v>
@@ -21402,7 +21402,7 @@
         <v>190.08</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>488</v>
+        <v>448.5</v>
       </c>
       <c r="R307" s="3" t="n"/>
       <c r="S307" s="3">
@@ -21469,7 +21469,7 @@
         <v>15.93</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>56.2</v>
+        <v>55.8</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>2.73</v>
@@ -21538,7 +21538,7 @@
         <v>15.55</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>32.55</v>
+        <v>32.35</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>1.2</v>
@@ -21607,7 +21607,7 @@
         <v>13.01</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>20.85</v>
+        <v>20.7</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>2.8</v>
@@ -21676,7 +21676,7 @@
         <v>36.1</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>6.5</v>
@@ -21735,7 +21735,7 @@
         <v>17.93</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>90.2</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>2.2</v>
@@ -21804,7 +21804,7 @@
         <v>14.72</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>1360</v>
+        <v>1315</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>45.38</v>
@@ -21873,7 +21873,7 @@
         <v>118</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>18700</v>
+        <v>17885</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>80</v>
@@ -21932,7 +21932,7 @@
         <v>23.77</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>308</v>
+        <v>297.5</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>5</v>
@@ -22001,7 +22001,7 @@
         <v>8.19</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>1290</v>
+        <v>1295</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>16.83</v>
@@ -22070,7 +22070,7 @@
         <v>3.5</v>
       </c>
       <c r="Q317" s="3" t="n">
-        <v>46.8</v>
+        <v>42.15</v>
       </c>
       <c r="R317" s="3" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>42.25</v>
       </c>
       <c r="Q318" s="3" t="n">
-        <v>85.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="R318" s="3" t="n">
         <v>0.6</v>
@@ -22208,7 +22208,7 @@
         <v>34.74</v>
       </c>
       <c r="Q319" s="3" t="n">
-        <v>161.5</v>
+        <v>157.5</v>
       </c>
       <c r="R319" s="3" t="n">
         <v>4.47</v>
@@ -22277,7 +22277,7 @@
         <v>20.59</v>
       </c>
       <c r="Q320" s="3" t="n">
-        <v>115.5</v>
+        <v>108.5</v>
       </c>
       <c r="R320" s="3" t="n"/>
       <c r="S320" s="3">
@@ -22413,7 +22413,7 @@
         <v>17.36</v>
       </c>
       <c r="Q322" s="3" t="n">
-        <v>71.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="R322" s="3" t="n">
         <v>2.5</v>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="P323" s="3" t="n"/>
       <c r="Q323" s="3" t="n">
-        <v>89.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="R323" s="3" t="n">
         <v>2.02</v>
@@ -22618,7 +22618,7 @@
         <v>13.65</v>
       </c>
       <c r="Q325" s="3" t="n">
-        <v>258</v>
+        <v>249.5</v>
       </c>
       <c r="R325" s="3" t="n">
         <v>7.2</v>
@@ -22687,7 +22687,7 @@
         <v>46.7</v>
       </c>
       <c r="Q326" s="3" t="n">
-        <v>108</v>
+        <v>105.5</v>
       </c>
       <c r="R326" s="3" t="n">
         <v>2.2</v>
@@ -22756,7 +22756,7 @@
         <v>13.07</v>
       </c>
       <c r="Q327" s="3" t="n">
-        <v>71.7</v>
+        <v>72.3</v>
       </c>
       <c r="R327" s="3" t="n">
         <v>2.52</v>
@@ -22825,7 +22825,7 @@
         <v>132.17</v>
       </c>
       <c r="Q328" s="3" t="n">
-        <v>184.5</v>
+        <v>175</v>
       </c>
       <c r="R328" s="3" t="n"/>
       <c r="S328" s="3">
@@ -22892,7 +22892,7 @@
         <v>12.16</v>
       </c>
       <c r="Q329" s="3" t="n">
-        <v>97</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="R329" s="3" t="n">
         <v>7.5</v>
@@ -22961,7 +22961,7 @@
         <v>20.96</v>
       </c>
       <c r="Q330" s="3" t="n">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="R330" s="3" t="n">
         <v>2.5</v>
@@ -23030,7 +23030,7 @@
         <v>6.19</v>
       </c>
       <c r="Q331" s="3" t="n">
-        <v>62.7</v>
+        <v>62.6</v>
       </c>
       <c r="R331" s="3" t="n">
         <v>5.5</v>
@@ -23099,7 +23099,7 @@
         <v>15.16</v>
       </c>
       <c r="Q332" s="3" t="n">
-        <v>49.4</v>
+        <v>49.45</v>
       </c>
       <c r="R332" s="3" t="n"/>
       <c r="S332" s="3">
@@ -23166,7 +23166,7 @@
         <v>13.42</v>
       </c>
       <c r="Q333" s="3" t="n">
-        <v>74.5</v>
+        <v>74</v>
       </c>
       <c r="R333" s="3" t="n">
         <v>5.06</v>
@@ -23235,7 +23235,7 @@
         <v>21.94</v>
       </c>
       <c r="Q334" s="3" t="n">
-        <v>864</v>
+        <v>836</v>
       </c>
       <c r="R334" s="3" t="n">
         <v>20</v>
@@ -23304,7 +23304,7 @@
         <v>15.21</v>
       </c>
       <c r="Q335" s="3" t="n">
-        <v>52.3</v>
+        <v>53</v>
       </c>
       <c r="R335" s="3" t="n">
         <v>1.8</v>
@@ -23367,7 +23367,7 @@
         <v>10.44</v>
       </c>
       <c r="Q336" s="3" t="n">
-        <v>112.5</v>
+        <v>111.5</v>
       </c>
       <c r="R336" s="3" t="n">
         <v>5.8</v>
@@ -23436,7 +23436,7 @@
         <v>23.69</v>
       </c>
       <c r="Q337" s="3" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="R337" s="3" t="n">
         <v>6.5</v>
@@ -23505,7 +23505,7 @@
         <v>23.24</v>
       </c>
       <c r="Q338" s="3" t="n">
-        <v>71.5</v>
+        <v>72.3</v>
       </c>
       <c r="R338" s="3" t="n">
         <v>25.5</v>
@@ -23572,7 +23572,7 @@
       </c>
       <c r="P339" s="3" t="n"/>
       <c r="Q339" s="3" t="n">
-        <v>14.7</v>
+        <v>14.1</v>
       </c>
       <c r="R339" s="3" t="n"/>
       <c r="S339" s="3">
@@ -23639,7 +23639,7 @@
         <v>12.44</v>
       </c>
       <c r="Q340" s="3" t="n">
-        <v>378.5</v>
+        <v>380.5</v>
       </c>
       <c r="R340" s="3" t="n">
         <v>12.3</v>
@@ -23708,7 +23708,7 @@
         <v>177.93</v>
       </c>
       <c r="Q341" s="3" t="n">
-        <v>49.8</v>
+        <v>48.5</v>
       </c>
       <c r="R341" s="3" t="n">
         <v>0.1</v>
@@ -23777,7 +23777,7 @@
         <v>19.84</v>
       </c>
       <c r="Q342" s="3" t="n">
-        <v>271.5</v>
+        <v>265</v>
       </c>
       <c r="R342" s="3" t="n">
         <v>10.15</v>
@@ -23846,7 +23846,7 @@
         <v>16.08</v>
       </c>
       <c r="Q343" s="3" t="n">
-        <v>753</v>
+        <v>709</v>
       </c>
       <c r="R343" s="3" t="n">
         <v>23</v>
@@ -23915,7 +23915,7 @@
         <v>17</v>
       </c>
       <c r="Q344" s="3" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="R344" s="3" t="n">
         <v>12</v>
@@ -23984,7 +23984,7 @@
         <v>38.04</v>
       </c>
       <c r="Q345" s="3" t="n">
-        <v>190.5</v>
+        <v>181</v>
       </c>
       <c r="R345" s="3" t="n">
         <v>2.8</v>
@@ -24122,7 +24122,7 @@
         <v>38.27</v>
       </c>
       <c r="Q347" s="3" t="n">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="R347" s="3" t="n">
         <v>1.8</v>
@@ -24191,7 +24191,7 @@
         <v>10.05</v>
       </c>
       <c r="Q348" s="3" t="n">
-        <v>89.09999999999999</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="R348" s="3" t="n">
         <v>3.5</v>
@@ -24329,7 +24329,7 @@
         <v>2787.5</v>
       </c>
       <c r="Q350" s="3" t="n">
-        <v>108.5</v>
+        <v>104.5</v>
       </c>
       <c r="R350" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Q351" s="3" t="n">
-        <v>1280</v>
+        <v>1250</v>
       </c>
       <c r="R351" s="3" t="n">
         <v>11.66</v>
@@ -24467,7 +24467,7 @@
         <v>24.45</v>
       </c>
       <c r="Q352" s="3" t="n">
-        <v>63.5</v>
+        <v>62.6</v>
       </c>
       <c r="R352" s="3" t="n">
         <v>2.5</v>
@@ -24536,7 +24536,7 @@
         <v>26.68</v>
       </c>
       <c r="Q353" s="3" t="n">
-        <v>68.09999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="R353" s="3" t="n">
         <v>1.93</v>
@@ -24605,7 +24605,7 @@
         <v>14.29</v>
       </c>
       <c r="Q354" s="3" t="n">
-        <v>82</v>
+        <v>82.3</v>
       </c>
       <c r="R354" s="3" t="n">
         <v>2.6</v>
@@ -24672,7 +24672,7 @@
       </c>
       <c r="P355" s="3" t="n"/>
       <c r="Q355" s="3" t="n">
-        <v>535</v>
+        <v>511</v>
       </c>
       <c r="R355" s="3" t="n">
         <v>6.45</v>
@@ -24741,7 +24741,7 @@
         <v>25.23</v>
       </c>
       <c r="Q356" s="3" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="R356" s="3" t="n">
         <v>6.92</v>
@@ -24810,7 +24810,7 @@
         <v>46.75</v>
       </c>
       <c r="Q357" s="3" t="n">
-        <v>56.6</v>
+        <v>55.2</v>
       </c>
       <c r="R357" s="3" t="n">
         <v>0.68</v>
@@ -24879,7 +24879,7 @@
         <v>16.24</v>
       </c>
       <c r="Q358" s="3" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="R358" s="3" t="n">
         <v>5.5</v>
@@ -24948,7 +24948,7 @@
         <v>74.42</v>
       </c>
       <c r="Q359" s="3" t="n">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="R359" s="3" t="n">
         <v>3</v>
@@ -25011,7 +25011,7 @@
         <v>16.75</v>
       </c>
       <c r="Q360" s="3" t="n">
-        <v>187.5</v>
+        <v>188.5</v>
       </c>
       <c r="R360" s="3" t="n">
         <v>6</v>
@@ -25078,7 +25078,7 @@
       </c>
       <c r="P361" s="3" t="n"/>
       <c r="Q361" s="3" t="n">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="R361" s="3" t="n"/>
       <c r="S361" s="3">
@@ -25214,7 +25214,7 @@
         <v>26.53</v>
       </c>
       <c r="Q363" s="3" t="n">
-        <v>283.5</v>
+        <v>273</v>
       </c>
       <c r="R363" s="3" t="n"/>
       <c r="S363" s="3">
@@ -25281,7 +25281,7 @@
         <v>24.33</v>
       </c>
       <c r="Q364" s="3" t="n">
-        <v>217</v>
+        <v>211.5</v>
       </c>
       <c r="R364" s="3" t="n">
         <v>2.73</v>
@@ -25338,7 +25338,7 @@
       <c r="O365" s="3" t="n"/>
       <c r="P365" s="3" t="n"/>
       <c r="Q365" s="3" t="n">
-        <v>66.59999999999999</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R365" s="3" t="n"/>
       <c r="S365" s="3">
@@ -25405,7 +25405,7 @@
         <v>21.7</v>
       </c>
       <c r="Q366" s="3" t="n">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="R366" s="3" t="n">
         <v>3</v>
@@ -25470,7 +25470,7 @@
         <v>85.06999999999999</v>
       </c>
       <c r="Q367" s="3" t="n">
-        <v>1395</v>
+        <v>1365</v>
       </c>
       <c r="R367" s="3" t="n">
         <v>7.5066</v>
@@ -25539,7 +25539,7 @@
         <v>19.07</v>
       </c>
       <c r="Q368" s="3" t="n">
-        <v>191.5</v>
+        <v>186.5</v>
       </c>
       <c r="R368" s="3" t="n">
         <v>5.565</v>
@@ -25598,7 +25598,7 @@
         <v>36.58</v>
       </c>
       <c r="Q369" s="3" t="n">
-        <v>43.2</v>
+        <v>42.75</v>
       </c>
       <c r="R369" s="3" t="n">
         <v>0.8</v>
@@ -25667,7 +25667,7 @@
         <v>20.21</v>
       </c>
       <c r="Q370" s="3" t="n">
-        <v>78.8</v>
+        <v>75.5</v>
       </c>
       <c r="R370" s="3" t="n">
         <v>1.8896</v>
@@ -25736,7 +25736,7 @@
         <v>26.83</v>
       </c>
       <c r="Q371" s="3" t="n">
-        <v>227</v>
+        <v>222.5</v>
       </c>
       <c r="R371" s="3" t="n">
         <v>4.3</v>
@@ -25805,7 +25805,7 @@
         <v>23.27</v>
       </c>
       <c r="Q372" s="3" t="n">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="R372" s="3" t="n">
         <v>6.19</v>
@@ -25874,7 +25874,7 @@
         <v>33.25</v>
       </c>
       <c r="Q373" s="3" t="n">
-        <v>495</v>
+        <v>478</v>
       </c>
       <c r="R373" s="3" t="n">
         <v>6</v>
@@ -25943,7 +25943,7 @@
         <v>39.33</v>
       </c>
       <c r="Q374" s="3" t="n">
-        <v>876</v>
+        <v>861</v>
       </c>
       <c r="R374" s="3" t="n">
         <v>36.7702</v>
@@ -26081,7 +26081,7 @@
         <v>16.4</v>
       </c>
       <c r="Q376" s="3" t="n">
-        <v>372.5</v>
+        <v>370</v>
       </c>
       <c r="R376" s="3" t="n">
         <v>13.78</v>
@@ -26140,7 +26140,7 @@
         <v>64.52</v>
       </c>
       <c r="Q377" s="3" t="n">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="R377" s="3" t="n">
         <v>2.55</v>
@@ -26209,7 +26209,7 @@
         <v>46.15</v>
       </c>
       <c r="Q378" s="3" t="n">
-        <v>1800</v>
+        <v>1670</v>
       </c>
       <c r="R378" s="3" t="n">
         <v>11.2587</v>
@@ -26276,7 +26276,7 @@
       </c>
       <c r="P379" s="3" t="n"/>
       <c r="Q379" s="3" t="n">
-        <v>23.65</v>
+        <v>23.2</v>
       </c>
       <c r="R379" s="3" t="n"/>
       <c r="S379" s="3">
@@ -26343,7 +26343,7 @@
         <v>73.45999999999999</v>
       </c>
       <c r="Q380" s="3" t="n">
-        <v>1320</v>
+        <v>1280</v>
       </c>
       <c r="R380" s="3" t="n">
         <v>1.49</v>
@@ -26412,7 +26412,7 @@
         <v>23.83</v>
       </c>
       <c r="Q381" s="3" t="n">
-        <v>226.5</v>
+        <v>217</v>
       </c>
       <c r="R381" s="3" t="n">
         <v>4.2</v>
@@ -26469,7 +26469,7 @@
       <c r="O382" s="3" t="n"/>
       <c r="P382" s="3" t="n"/>
       <c r="Q382" s="3" t="n">
-        <v>425</v>
+        <v>409.5</v>
       </c>
       <c r="R382" s="3" t="n">
         <v>0.2177</v>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="P383" s="3" t="n"/>
       <c r="Q383" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>63.4</v>
       </c>
       <c r="R383" s="3" t="n"/>
       <c r="S383" s="3">
@@ -26603,7 +26603,7 @@
         <v>37.51</v>
       </c>
       <c r="Q384" s="3" t="n">
-        <v>405.5</v>
+        <v>399</v>
       </c>
       <c r="R384" s="3" t="n">
         <v>10</v>
@@ -26672,7 +26672,7 @@
         <v>49.03</v>
       </c>
       <c r="Q385" s="3" t="n">
-        <v>917</v>
+        <v>902</v>
       </c>
       <c r="R385" s="3" t="n">
         <v>5.7</v>
@@ -26737,7 +26737,7 @@
         <v>15.51</v>
       </c>
       <c r="Q386" s="3" t="n">
-        <v>366.5</v>
+        <v>367.5</v>
       </c>
       <c r="R386" s="3" t="n">
         <v>10</v>
@@ -26806,7 +26806,7 @@
         <v>12.31</v>
       </c>
       <c r="Q387" s="3" t="n">
-        <v>86.2</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="R387" s="3" t="n">
         <v>1.2</v>
@@ -26875,7 +26875,7 @@
         <v>70.52</v>
       </c>
       <c r="Q388" s="3" t="n">
-        <v>3670</v>
+        <v>3480</v>
       </c>
       <c r="R388" s="3" t="n">
         <v>15.23</v>
@@ -26944,7 +26944,7 @@
         <v>110.51</v>
       </c>
       <c r="Q389" s="3" t="n">
-        <v>7195</v>
+        <v>6890</v>
       </c>
       <c r="R389" s="3" t="n">
         <v>24.72</v>
@@ -27003,7 +27003,7 @@
         <v>19.19</v>
       </c>
       <c r="Q390" s="3" t="n">
-        <v>129.5</v>
+        <v>124.5</v>
       </c>
       <c r="R390" s="3" t="n">
         <v>5</v>
@@ -27072,7 +27072,7 @@
         <v>33.83</v>
       </c>
       <c r="Q391" s="3" t="n">
-        <v>642</v>
+        <v>624</v>
       </c>
       <c r="R391" s="3" t="n">
         <v>7.5</v>
@@ -27141,7 +27141,7 @@
         <v>53.75</v>
       </c>
       <c r="Q392" s="3" t="n">
-        <v>1030</v>
+        <v>988</v>
       </c>
       <c r="R392" s="3" t="n">
         <v>6.99</v>
@@ -27208,7 +27208,7 @@
       </c>
       <c r="P393" s="3" t="n"/>
       <c r="Q393" s="3" t="n">
-        <v>78.2</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="R393" s="3" t="n"/>
       <c r="S393" s="3">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="P394" s="3" t="n"/>
       <c r="Q394" s="3" t="n">
-        <v>61.4</v>
+        <v>58.8</v>
       </c>
       <c r="R394" s="3" t="n"/>
       <c r="S394" s="3">
@@ -27340,7 +27340,7 @@
         <v>32.7</v>
       </c>
       <c r="Q395" s="3" t="n">
-        <v>70.8</v>
+        <v>70</v>
       </c>
       <c r="R395" s="3" t="n">
         <v>0.9</v>
@@ -27405,7 +27405,7 @@
         <v>21.5</v>
       </c>
       <c r="Q396" s="3" t="n">
-        <v>317.5</v>
+        <v>315</v>
       </c>
       <c r="R396" s="3" t="n">
         <v>7.6988</v>
@@ -27468,7 +27468,7 @@
         <v>20.22</v>
       </c>
       <c r="Q397" s="3" t="n">
-        <v>148.5</v>
+        <v>148</v>
       </c>
       <c r="R397" s="3" t="n">
         <v>3.75</v>
@@ -27537,7 +27537,7 @@
         <v>53.79</v>
       </c>
       <c r="Q398" s="3" t="n">
-        <v>554</v>
+        <v>567</v>
       </c>
       <c r="R398" s="3" t="n"/>
       <c r="S398" s="3">
@@ -27604,7 +27604,7 @@
         <v>12.33</v>
       </c>
       <c r="Q399" s="3" t="n">
-        <v>60</v>
+        <v>59.8</v>
       </c>
       <c r="R399" s="3" t="n">
         <v>3</v>
@@ -27663,7 +27663,7 @@
         <v>8.73</v>
       </c>
       <c r="Q400" s="3" t="n">
-        <v>135.5</v>
+        <v>137.5</v>
       </c>
       <c r="R400" s="3" t="n"/>
       <c r="S400" s="3">
@@ -27730,7 +27730,7 @@
         <v>16.06</v>
       </c>
       <c r="Q401" s="3" t="n">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="R401" s="3" t="n">
         <v>10</v>
@@ -27799,7 +27799,7 @@
         <v>64.78</v>
       </c>
       <c r="Q402" s="3" t="n">
-        <v>1210</v>
+        <v>1170</v>
       </c>
       <c r="R402" s="3" t="n">
         <v>12</v>
@@ -27868,7 +27868,7 @@
         <v>463.16</v>
       </c>
       <c r="Q403" s="3" t="n">
-        <v>423.5</v>
+        <v>406</v>
       </c>
       <c r="R403" s="3" t="n">
         <v>1.19</v>
@@ -27937,7 +27937,7 @@
         <v>20.96</v>
       </c>
       <c r="Q404" s="3" t="n">
-        <v>346.5</v>
+        <v>336</v>
       </c>
       <c r="R404" s="3" t="n">
         <v>10.14</v>
@@ -28002,7 +28002,7 @@
         <v>20.63</v>
       </c>
       <c r="Q405" s="3" t="n">
-        <v>2345</v>
+        <v>2310</v>
       </c>
       <c r="R405" s="3" t="n">
         <v>144.39</v>
@@ -28061,7 +28061,7 @@
         <v>10.85</v>
       </c>
       <c r="Q406" s="3" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="R406" s="3" t="n">
         <v>16</v>
@@ -28130,7 +28130,7 @@
         <v>40.41</v>
       </c>
       <c r="Q407" s="3" t="n">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="R407" s="3" t="n">
         <v>3.35</v>
@@ -28268,7 +28268,7 @@
         <v>21.78</v>
       </c>
       <c r="Q409" s="3" t="n">
-        <v>622</v>
+        <v>609</v>
       </c>
       <c r="R409" s="3" t="n">
         <v>21</v>
@@ -28337,7 +28337,7 @@
         <v>31.61</v>
       </c>
       <c r="Q410" s="3" t="n">
-        <v>156.5</v>
+        <v>154</v>
       </c>
       <c r="R410" s="3" t="n">
         <v>3.5</v>
@@ -28406,7 +28406,7 @@
         <v>294.74</v>
       </c>
       <c r="Q411" s="3" t="n">
-        <v>336.5</v>
+        <v>321.5</v>
       </c>
       <c r="R411" s="3" t="n">
         <v>1.9431</v>
@@ -28475,7 +28475,7 @@
         <v>21.79</v>
       </c>
       <c r="Q412" s="3" t="n">
-        <v>184.5</v>
+        <v>180</v>
       </c>
       <c r="R412" s="3" t="n">
         <v>4.6</v>
@@ -28544,7 +28544,7 @@
         <v>42.78</v>
       </c>
       <c r="Q413" s="3" t="n">
-        <v>1320</v>
+        <v>1270</v>
       </c>
       <c r="R413" s="3" t="n">
         <v>13</v>
@@ -28613,7 +28613,7 @@
         <v>13.5</v>
       </c>
       <c r="Q414" s="3" t="n">
-        <v>135.5</v>
+        <v>134</v>
       </c>
       <c r="R414" s="3" t="n">
         <v>1.25</v>
@@ -28743,7 +28743,7 @@
         <v>13.07</v>
       </c>
       <c r="Q416" s="3" t="n">
-        <v>62.4</v>
+        <v>61.5</v>
       </c>
       <c r="R416" s="3" t="n">
         <v>5.16</v>
@@ -28812,7 +28812,7 @@
         <v>26.13</v>
       </c>
       <c r="Q417" s="3" t="n">
-        <v>73.5</v>
+        <v>70.7</v>
       </c>
       <c r="R417" s="3" t="n">
         <v>0.23</v>
@@ -28871,7 +28871,7 @@
         <v>28.62</v>
       </c>
       <c r="Q418" s="3" t="n">
-        <v>1030</v>
+        <v>1005</v>
       </c>
       <c r="R418" s="3" t="n">
         <v>19.1</v>
@@ -28940,7 +28940,7 @@
         <v>84.45</v>
       </c>
       <c r="Q419" s="3" t="n">
-        <v>469.5</v>
+        <v>446</v>
       </c>
       <c r="R419" s="3" t="n">
         <v>3</v>
@@ -29009,7 +29009,7 @@
         <v>14.56</v>
       </c>
       <c r="Q420" s="3" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="R420" s="3" t="n">
         <v>15.78</v>
@@ -29078,7 +29078,7 @@
         <v>38.61</v>
       </c>
       <c r="Q421" s="3" t="n">
-        <v>2190</v>
+        <v>2150</v>
       </c>
       <c r="R421" s="3" t="n">
         <v>10.5</v>
@@ -29137,7 +29137,7 @@
         <v>1</v>
       </c>
       <c r="Q422" s="3" t="n">
-        <v>591</v>
+        <v>551</v>
       </c>
       <c r="R422" s="3" t="n">
         <v>1</v>
@@ -29206,7 +29206,7 @@
         <v>115.9</v>
       </c>
       <c r="Q423" s="3" t="n">
-        <v>552</v>
+        <v>567</v>
       </c>
       <c r="R423" s="3" t="n">
         <v>3</v>
@@ -29265,7 +29265,7 @@
         <v>16.67</v>
       </c>
       <c r="Q424" s="3" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="R424" s="3" t="n">
         <v>6.97</v>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="P425" s="3" t="n"/>
       <c r="Q425" s="3" t="n">
-        <v>15</v>
+        <v>14.75</v>
       </c>
       <c r="R425" s="3" t="n"/>
       <c r="S425" s="3">
@@ -29387,7 +29387,7 @@
         <v>14.41</v>
       </c>
       <c r="Q426" s="3" t="n">
-        <v>300.5</v>
+        <v>296.5</v>
       </c>
       <c r="R426" s="3" t="n">
         <v>8.5</v>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="P427" s="3" t="n"/>
       <c r="Q427" s="3" t="n">
-        <v>85.59999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="R427" s="3" t="n"/>
       <c r="S427" s="3">
@@ -29511,7 +29511,7 @@
         <v>57.36</v>
       </c>
       <c r="Q428" s="3" t="n">
-        <v>296</v>
+        <v>288.5</v>
       </c>
       <c r="R428" s="3" t="n">
         <v>1.4</v>
@@ -29580,7 +29580,7 @@
         <v>17.59</v>
       </c>
       <c r="Q429" s="3" t="n">
-        <v>709</v>
+        <v>690</v>
       </c>
       <c r="R429" s="3" t="n">
         <v>17</v>
@@ -29635,7 +29635,7 @@
       </c>
       <c r="P430" s="3" t="n"/>
       <c r="Q430" s="3" t="n">
-        <v>58.8</v>
+        <v>53</v>
       </c>
       <c r="R430" s="3" t="n"/>
       <c r="S430" s="3">
@@ -29702,7 +29702,7 @@
         <v>20.63</v>
       </c>
       <c r="Q431" s="3" t="n">
-        <v>30.8</v>
+        <v>30.4</v>
       </c>
       <c r="R431" s="3" t="n">
         <v>1</v>
@@ -29771,7 +29771,7 @@
         <v>48.36</v>
       </c>
       <c r="Q432" s="3" t="n">
-        <v>2035</v>
+        <v>1975</v>
       </c>
       <c r="R432" s="3" t="n">
         <v>0.5</v>
@@ -29840,7 +29840,7 @@
         <v>19.38</v>
       </c>
       <c r="Q433" s="3" t="n">
-        <v>590</v>
+        <v>531</v>
       </c>
       <c r="R433" s="3" t="n">
         <v>8.9871</v>
@@ -29909,7 +29909,7 @@
         <v>34.98</v>
       </c>
       <c r="Q434" s="3" t="n">
-        <v>267.5</v>
+        <v>261.5</v>
       </c>
       <c r="R434" s="3" t="n">
         <v>1.5</v>
@@ -29978,7 +29978,7 @@
         <v>65.13</v>
       </c>
       <c r="Q435" s="3" t="n">
-        <v>2810</v>
+        <v>2580</v>
       </c>
       <c r="R435" s="3" t="n">
         <v>19.85</v>
@@ -30047,7 +30047,7 @@
         <v>21.64</v>
       </c>
       <c r="Q436" s="3" t="n">
-        <v>514</v>
+        <v>497</v>
       </c>
       <c r="R436" s="3" t="n">
         <v>7</v>
@@ -30106,7 +30106,7 @@
         <v>30.21</v>
       </c>
       <c r="Q437" s="3" t="n">
-        <v>355.5</v>
+        <v>349.5</v>
       </c>
       <c r="R437" s="3" t="n">
         <v>9</v>
@@ -30175,7 +30175,7 @@
         <v>40.48</v>
       </c>
       <c r="Q438" s="3" t="n">
-        <v>2215</v>
+        <v>1995</v>
       </c>
       <c r="R438" s="3" t="n">
         <v>16</v>
@@ -30244,7 +30244,7 @@
         <v>56.01</v>
       </c>
       <c r="Q439" s="3" t="n">
-        <v>1500</v>
+        <v>1425</v>
       </c>
       <c r="R439" s="3" t="n">
         <v>10</v>
@@ -30313,7 +30313,7 @@
         <v>66.52</v>
       </c>
       <c r="Q440" s="3" t="n">
-        <v>271.5</v>
+        <v>263</v>
       </c>
       <c r="R440" s="3" t="n">
         <v>2.46</v>
@@ -30382,7 +30382,7 @@
         <v>68.04000000000001</v>
       </c>
       <c r="Q441" s="3" t="n">
-        <v>6475</v>
+        <v>6310</v>
       </c>
       <c r="R441" s="3" t="n">
         <v>54.99</v>
@@ -30445,7 +30445,7 @@
         <v>31.03</v>
       </c>
       <c r="Q442" s="3" t="n">
-        <v>16.55</v>
+        <v>16.4</v>
       </c>
       <c r="R442" s="3" t="n">
         <v>0.8934</v>
@@ -30514,7 +30514,7 @@
         <v>11.44</v>
       </c>
       <c r="Q443" s="3" t="n">
-        <v>114.5</v>
+        <v>115</v>
       </c>
       <c r="R443" s="3" t="n">
         <v>5.6</v>
@@ -30577,7 +30577,7 @@
         <v>29.91</v>
       </c>
       <c r="Q444" s="3" t="n">
-        <v>308</v>
+        <v>286.5</v>
       </c>
       <c r="R444" s="3" t="n">
         <v>2</v>
@@ -30646,7 +30646,7 @@
         <v>251.33</v>
       </c>
       <c r="Q445" s="3" t="n">
-        <v>534</v>
+        <v>507</v>
       </c>
       <c r="R445" s="3" t="n">
         <v>2.15</v>
@@ -30713,7 +30713,7 @@
       </c>
       <c r="P446" s="3" t="n"/>
       <c r="Q446" s="3" t="n">
-        <v>425</v>
+        <v>414.5</v>
       </c>
       <c r="R446" s="3" t="n"/>
       <c r="S446" s="3">
@@ -30780,7 +30780,7 @@
         <v>14.24</v>
       </c>
       <c r="Q447" s="3" t="n">
-        <v>506</v>
+        <v>495</v>
       </c>
       <c r="R447" s="3" t="n">
         <v>38</v>
@@ -30849,7 +30849,7 @@
         <v>51.64</v>
       </c>
       <c r="Q448" s="3" t="n">
-        <v>866</v>
+        <v>834</v>
       </c>
       <c r="R448" s="3" t="n">
         <v>6.39</v>
@@ -30898,7 +30898,7 @@
       <c r="O449" s="3" t="n"/>
       <c r="P449" s="3" t="n"/>
       <c r="Q449" s="3" t="n">
-        <v>153</v>
+        <v>152.5</v>
       </c>
       <c r="R449" s="3" t="n"/>
       <c r="S449" s="3">
@@ -30965,7 +30965,7 @@
         <v>174.44</v>
       </c>
       <c r="Q450" s="3" t="n">
-        <v>2055</v>
+        <v>1975</v>
       </c>
       <c r="R450" s="3" t="n">
         <v>4.53</v>
@@ -31034,7 +31034,7 @@
         <v>14.77</v>
       </c>
       <c r="Q451" s="3" t="n">
-        <v>279</v>
+        <v>277.5</v>
       </c>
       <c r="R451" s="3" t="n">
         <v>11.5</v>
@@ -31103,7 +31103,7 @@
         <v>78.33</v>
       </c>
       <c r="Q452" s="3" t="n">
-        <v>438</v>
+        <v>418.5</v>
       </c>
       <c r="R452" s="3" t="n">
         <v>1.97</v>
@@ -31172,7 +31172,7 @@
         <v>558.33</v>
       </c>
       <c r="Q453" s="3" t="n">
-        <v>174</v>
+        <v>167.5</v>
       </c>
       <c r="R453" s="3" t="n"/>
       <c r="S453" s="3">
@@ -31239,7 +31239,7 @@
         <v>43.46</v>
       </c>
       <c r="Q454" s="3" t="n">
-        <v>229.5</v>
+        <v>225.5</v>
       </c>
       <c r="R454" s="3" t="n">
         <v>2.7</v>
@@ -31308,7 +31308,7 @@
         <v>385.42</v>
       </c>
       <c r="Q455" s="3" t="n">
-        <v>171.5</v>
+        <v>172.5</v>
       </c>
       <c r="R455" s="3" t="n"/>
       <c r="S455" s="3">
@@ -31375,7 +31375,7 @@
         <v>89.52</v>
       </c>
       <c r="Q456" s="3" t="n">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="R456" s="3" t="n">
         <v>1.99</v>
@@ -31444,7 +31444,7 @@
         <v>153.35</v>
       </c>
       <c r="Q457" s="3" t="n">
-        <v>1070</v>
+        <v>1080</v>
       </c>
       <c r="R457" s="3" t="n">
         <v>2</v>
@@ -31513,7 +31513,7 @@
         <v>42.18</v>
       </c>
       <c r="Q458" s="3" t="n">
-        <v>126.5</v>
+        <v>115</v>
       </c>
       <c r="R458" s="3" t="n">
         <v>0.98</v>
@@ -31582,7 +31582,7 @@
         <v>16.1</v>
       </c>
       <c r="Q459" s="3" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="R459" s="3" t="n">
         <v>5.89</v>
@@ -31651,7 +31651,7 @@
         <v>28.99</v>
       </c>
       <c r="Q460" s="3" t="n">
-        <v>49.45</v>
+        <v>49</v>
       </c>
       <c r="R460" s="3" t="n">
         <v>0.68</v>
@@ -31720,7 +31720,7 @@
         <v>13.97</v>
       </c>
       <c r="Q461" s="3" t="n">
-        <v>247.5</v>
+        <v>247</v>
       </c>
       <c r="R461" s="3" t="n">
         <v>16</v>
@@ -31789,7 +31789,7 @@
         <v>21.27</v>
       </c>
       <c r="Q462" s="3" t="n">
-        <v>109.5</v>
+        <v>106</v>
       </c>
       <c r="R462" s="3" t="n">
         <v>1.68</v>
@@ -31858,7 +31858,7 @@
         <v>24.06</v>
       </c>
       <c r="Q463" s="3" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R463" s="3" t="n">
         <v>4.22</v>
@@ -31927,7 +31927,7 @@
         <v>32.18</v>
       </c>
       <c r="Q464" s="3" t="n">
-        <v>91.8</v>
+        <v>90.7</v>
       </c>
       <c r="R464" s="3" t="n"/>
       <c r="S464" s="3">
@@ -31994,7 +31994,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="Q465" s="3" t="n">
-        <v>42.75</v>
+        <v>42.15</v>
       </c>
       <c r="R465" s="3" t="n">
         <v>1.49</v>
@@ -32063,7 +32063,7 @@
         <v>7.22</v>
       </c>
       <c r="Q466" s="3" t="n">
-        <v>85.90000000000001</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="R466" s="3" t="n">
         <v>3.8</v>
@@ -32132,7 +32132,7 @@
         <v>13.93</v>
       </c>
       <c r="Q467" s="3" t="n">
-        <v>178.5</v>
+        <v>177.5</v>
       </c>
       <c r="R467" s="3" t="n">
         <v>11.47</v>
@@ -32201,7 +32201,7 @@
         <v>18.09</v>
       </c>
       <c r="Q468" s="3" t="n">
-        <v>62</v>
+        <v>60.3</v>
       </c>
       <c r="R468" s="3" t="n">
         <v>1</v>
@@ -32270,7 +32270,7 @@
         <v>27.01</v>
       </c>
       <c r="Q469" s="3" t="n">
-        <v>90.90000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="R469" s="3" t="n">
         <v>0</v>
@@ -32339,7 +32339,7 @@
         <v>27.63</v>
       </c>
       <c r="Q470" s="3" t="n">
-        <v>339</v>
+        <v>325.5</v>
       </c>
       <c r="R470" s="3" t="n">
         <v>3.89</v>
@@ -32408,7 +32408,7 @@
         <v>25.27</v>
       </c>
       <c r="Q471" s="3" t="n">
-        <v>910</v>
+        <v>900</v>
       </c>
       <c r="R471" s="3" t="n">
         <v>14</v>
@@ -32477,7 +32477,7 @@
         <v>22.07</v>
       </c>
       <c r="Q472" s="3" t="n">
-        <v>137</v>
+        <v>133.5</v>
       </c>
       <c r="R472" s="3" t="n">
         <v>3.5</v>
@@ -32546,7 +32546,7 @@
         <v>26.61</v>
       </c>
       <c r="Q473" s="3" t="n">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="R473" s="3" t="n"/>
       <c r="S473" s="3">
@@ -32613,7 +32613,7 @@
         <v>5.78</v>
       </c>
       <c r="Q474" s="3" t="n">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="R474" s="3" t="n">
         <v>4.448</v>
@@ -32680,7 +32680,7 @@
       </c>
       <c r="P475" s="3" t="n"/>
       <c r="Q475" s="3" t="n">
-        <v>2065</v>
+        <v>1990</v>
       </c>
       <c r="R475" s="3" t="n">
         <v>16.96</v>
@@ -32749,7 +32749,7 @@
         <v>63.86</v>
       </c>
       <c r="Q476" s="3" t="n">
-        <v>521</v>
+        <v>485</v>
       </c>
       <c r="R476" s="3" t="n">
         <v>2</v>
@@ -32818,7 +32818,7 @@
         <v>9.449999999999999</v>
       </c>
       <c r="Q477" s="3" t="n">
-        <v>36.35</v>
+        <v>35.55</v>
       </c>
       <c r="R477" s="3" t="n">
         <v>1.5</v>
@@ -32887,7 +32887,7 @@
         <v>27.97</v>
       </c>
       <c r="Q478" s="3" t="n">
-        <v>26.3</v>
+        <v>26.05</v>
       </c>
       <c r="R478" s="3" t="n">
         <v>1.198</v>
@@ -32956,7 +32956,7 @@
         <v>25.26</v>
       </c>
       <c r="Q479" s="3" t="n">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="R479" s="3" t="n">
         <v>10</v>
@@ -33025,7 +33025,7 @@
         <v>16.47</v>
       </c>
       <c r="Q480" s="3" t="n">
-        <v>368.5</v>
+        <v>371</v>
       </c>
       <c r="R480" s="3" t="n">
         <v>16</v>
@@ -33094,7 +33094,7 @@
         <v>9.94</v>
       </c>
       <c r="Q481" s="3" t="n">
-        <v>141</v>
+        <v>141.5</v>
       </c>
       <c r="R481" s="3" t="n">
         <v>6.5</v>
@@ -33163,7 +33163,7 @@
         <v>15.74</v>
       </c>
       <c r="Q482" s="3" t="n">
-        <v>58.7</v>
+        <v>58</v>
       </c>
       <c r="R482" s="3" t="n">
         <v>2.12</v>
@@ -33232,7 +33232,7 @@
         <v>51.18</v>
       </c>
       <c r="Q483" s="3" t="n">
-        <v>92.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="R483" s="3" t="n">
         <v>0.72</v>
@@ -33301,7 +33301,7 @@
         <v>86.2</v>
       </c>
       <c r="Q484" s="3" t="n">
-        <v>1300</v>
+        <v>1330</v>
       </c>
       <c r="R484" s="3" t="n">
         <v>4.56</v>
@@ -33370,7 +33370,7 @@
         <v>14.1</v>
       </c>
       <c r="Q485" s="3" t="n">
-        <v>66</v>
+        <v>64.7</v>
       </c>
       <c r="R485" s="3" t="n">
         <v>2</v>
@@ -33439,7 +33439,7 @@
         <v>5.35</v>
       </c>
       <c r="Q486" s="3" t="n">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="R486" s="3" t="n">
         <v>1.3</v>
@@ -33508,7 +33508,7 @@
         <v>16.11</v>
       </c>
       <c r="Q487" s="3" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="R487" s="3" t="n">
         <v>1.18</v>
@@ -33577,7 +33577,7 @@
         <v>13.9</v>
       </c>
       <c r="Q488" s="3" t="n">
-        <v>29.05</v>
+        <v>28.95</v>
       </c>
       <c r="R488" s="3" t="n">
         <v>1.2</v>
@@ -33646,7 +33646,7 @@
         <v>14.11</v>
       </c>
       <c r="Q489" s="3" t="n">
-        <v>68.5</v>
+        <v>67.8</v>
       </c>
       <c r="R489" s="3" t="n">
         <v>4.1</v>
@@ -33784,7 +33784,7 @@
         <v>24.49</v>
       </c>
       <c r="Q491" s="3" t="n">
-        <v>77.40000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="R491" s="3" t="n">
         <v>2.8</v>
@@ -33922,7 +33922,7 @@
         <v>68.39</v>
       </c>
       <c r="Q493" s="3" t="n">
-        <v>97.3</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="R493" s="3" t="n">
         <v>1.819</v>
@@ -33991,7 +33991,7 @@
         <v>13.15</v>
       </c>
       <c r="Q494" s="3" t="n">
-        <v>39.7</v>
+        <v>39.55</v>
       </c>
       <c r="R494" s="3" t="n">
         <v>2</v>
@@ -34060,7 +34060,7 @@
         <v>14.5</v>
       </c>
       <c r="Q495" s="3" t="n">
-        <v>62.2</v>
+        <v>62</v>
       </c>
       <c r="R495" s="3" t="n">
         <v>4</v>
@@ -34129,7 +34129,7 @@
         <v>7.78</v>
       </c>
       <c r="Q496" s="3" t="n">
-        <v>40.35</v>
+        <v>41.7</v>
       </c>
       <c r="R496" s="3" t="n"/>
       <c r="S496" s="3">
@@ -34196,7 +34196,7 @@
         <v>21.44</v>
       </c>
       <c r="Q497" s="3" t="n">
-        <v>55.6</v>
+        <v>55</v>
       </c>
       <c r="R497" s="3" t="n">
         <v>2.2</v>
@@ -34265,7 +34265,7 @@
         <v>12.18</v>
       </c>
       <c r="Q498" s="3" t="n">
-        <v>128</v>
+        <v>129.5</v>
       </c>
       <c r="R498" s="3" t="n">
         <v>6.2</v>
@@ -34403,7 +34403,7 @@
         <v>5.21</v>
       </c>
       <c r="Q500" s="3" t="n">
-        <v>27.75</v>
+        <v>28.1</v>
       </c>
       <c r="R500" s="3" t="n">
         <v>1.1</v>
@@ -34472,7 +34472,7 @@
         <v>14.49</v>
       </c>
       <c r="Q501" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="R501" s="3" t="n">
         <v>4.5</v>

</xml_diff>